<commit_message>
Load X analytics export into simple tracker
Replaces the public-profile X numbers with the account's X analytics
export (Sep 1-28): impressions, bookmarks, reposts, new follows and
clicks (detail expands + profile visits + link clicks) per post, plus
video watch data in the notes. Removes the thread self-replies that the
public page showed as replies, and renames Link Clicks to Clicks since
both platforms count all post clicks in their engagement rate.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019Z3cCo91h4eCLVp6tiH6Ms
</commit_message>
<xml_diff>
--- a/social-media-tracker/AlphaNodus_Simple_Post_Tracker.xlsx
+++ b/social-media-tracker/AlphaNodus_Simple_Post_Tracker.xlsx
@@ -84,7 +84,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">Clicks on the post (LinkedIn counts these in its engagement rate).</t>
+          <t xml:space="preserve">All clicks on the post. LinkedIn: 'Clicks'. X: detail expands + profile visits + link clicks. Both platforms count these in their own engagement rate.</t>
         </r>
       </text>
     </comment>
@@ -221,7 +221,7 @@
     <t xml:space="preserve">Below Standard = under 0.8× our average</t>
   </si>
   <si>
-    <t xml:space="preserve">Instagram &amp; X: public profiles, 9/28/2026</t>
+    <t xml:space="preserve">X: X analytics export (Sep 1–28). Instagram: public profile, 9/28/2026</t>
   </si>
   <si>
     <t xml:space="preserve">Followers Today: update every Monday.</t>
@@ -269,7 +269,7 @@
     <t xml:space="preserve">Saves</t>
   </si>
   <si>
-    <t xml:space="preserve">Link Clicks</t>
+    <t xml:space="preserve">Clicks</t>
   </si>
   <si>
     <t xml:space="preserve">New Followers (3 days after post)</t>
@@ -440,16 +440,16 @@
     <t xml:space="preserve">Tell process stories as a carousel or short Reel. Avoid two Revenue Cycle posts in a row.</t>
   </si>
   <si>
-    <t xml:space="preserve">Video: Gravity AI explainer + demo link</t>
+    <t xml:space="preserve">Video: 3-min Gravity AI explainer + demo link</t>
   </si>
   <si>
     <t xml:space="preserve">https://x.com/AlphaNodus/status/2098433794022006872</t>
   </si>
   <si>
-    <t xml:space="preserve">27 views and no engagement. The account only has 46 followers.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Post a short clip instead of the full video. Reply in radiology / imaging threads to get seen.</t>
+    <t xml:space="preserve">Only 6 video views all month and nobody watched to the end (average watch 2–14 sec). No likes, replies or link clicks — the 5 engagements were 4 'show more' taps + 1 profile visit.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Post a 20–30 sec clip with captions instead of the 3-min video, with the demo link in the text.</t>
   </si>
   <si>
     <t xml:space="preserve">Image: 'Scanners idle a third of the day' + comment GravityAI ask</t>
@@ -458,34 +458,34 @@
     <t xml:space="preserve">https://x.com/AlphaNodus/status/2099545479755583973</t>
   </si>
   <si>
-    <t xml:space="preserve">Fewest views of the month and no engagement.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tag 1–2 relevant industry accounts or people. Turn the stat into a short thread.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Image: an order with one field missing — when is it flagged?</t>
+    <t xml:space="preserve">16 impressions and only 1 'show more' tap. Nobody replied to the 'comment GravityAI' ask.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Drop the comment-keyword ask. Tag 1–2 relevant industry accounts so more people see it.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3-tweet thread: an order with one field missing — when is it flagged?</t>
   </si>
   <si>
     <t xml:space="preserve">https://x.com/AlphaNodus/status/2101017252221128863</t>
   </si>
   <si>
-    <t xml:space="preserve">Only got a reply, no likes or reposts.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ending with a question worked here — keep doing it. Add a clear visual.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Image: 4 manual handoffs before an order is billable (pinned)</t>
+    <t xml:space="preserve">Only 1 'show more' tap. The '1 reply' X shows is our own next tweet in the thread, not a customer. The question sat in tweet 3, which only 3 people saw.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Put the question in the first tweet. Keep threads to 1–2 tweets.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2-tweet thread: 4 manual handoffs before an order is billable (pinned)</t>
   </si>
   <si>
     <t xml:space="preserve">https://x.com/AlphaNodus/status/2102915695722045558</t>
   </si>
   <si>
-    <t xml:space="preserve">Rated Good only because 1 reply came from very few views — 13, the lowest of the month, even though it was pinned.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Keep the question ending. Get it seen: tag 1–2 industry accounts and pin whichever post is doing best.</t>
+    <t xml:space="preserve">Rated Good only because 2 of 13 viewers tapped 'show more' — too few views to mean much. The '1 reply' is our own thread tweet. No likes or replies from others.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Keep the short list format, but get it seen: ask the team to repost and tag 1–2 industry accounts.</t>
   </si>
 </sst>
 </file>
@@ -1367,7 +1367,7 @@
       </c>
       <c r="D7" s="9" t="n">
         <f aca="false">IFERROR(AVERAGEIF($B$12:$B$211,A7,$Q$12:$Q$211),"")</f>
-        <v>0.0288461538461538</v>
+        <v>0.109998219373219</v>
       </c>
       <c r="E7" s="8" t="n">
         <f aca="false">COUNTIFS($B$12:$B$211,A7,$R$12:$R$211,"Good")</f>
@@ -2074,23 +2074,29 @@
       <c r="K21" s="18" t="n">
         <v>0</v>
       </c>
-      <c r="L21" s="19"/>
-      <c r="M21" s="19"/>
-      <c r="N21" s="19"/>
+      <c r="L21" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="M21" s="18" t="n">
+        <v>5</v>
+      </c>
+      <c r="N21" s="18" t="n">
+        <v>0</v>
+      </c>
       <c r="O21" s="20" t="s">
         <v>48</v>
       </c>
       <c r="P21" s="21" t="n">
         <f aca="false">IF(OR(A21="",B21=""),"",IF(COUNT(I21:M21)=0,"",SUM(I21:M21)))</f>
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="Q21" s="22" t="n">
         <f aca="false">IF(OR(OR(A21="",B21=""),P21=""),"",IFERROR(P21/(IF(N(H21)&gt;0,H21,IF(N(G21)&gt;0,G21,IF(COUNTIFS($B$12:$B$211,B21,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B21,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B21,$A$5:$A$7,0)))))),""))</f>
-        <v>0</v>
+        <v>0.185185185185185</v>
       </c>
       <c r="R21" s="23" t="str">
         <f aca="false">IF(OR(A21="",B21=""),"",IF(OR(Q21="",COUNTIFS($B$12:$B$211,B21,$Q$12:$Q$211,"&gt;=0")&lt;2),"No Data Yet",IFERROR(IF(Q21/AVERAGEIFS($Q$12:$Q$211,$B$12:$B$211,B21)&gt;=1.2,"Good",IF(Q21/AVERAGEIFS($Q$12:$Q$211,$B$12:$B$211,B21)&gt;=0.8,"Average","Below Standard")),"Average")))</f>
-        <v>Below Standard</v>
+        <v>Good</v>
       </c>
       <c r="S21" s="24" t="s">
         <v>93</v>
@@ -2138,19 +2144,25 @@
       <c r="K22" s="18" t="n">
         <v>0</v>
       </c>
-      <c r="L22" s="19"/>
-      <c r="M22" s="19"/>
-      <c r="N22" s="19"/>
+      <c r="L22" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="M22" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="N22" s="18" t="n">
+        <v>0</v>
+      </c>
       <c r="O22" s="20" t="s">
         <v>48</v>
       </c>
       <c r="P22" s="21" t="n">
         <f aca="false">IF(OR(A22="",B22=""),"",IF(COUNT(I22:M22)=0,"",SUM(I22:M22)))</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q22" s="22" t="n">
         <f aca="false">IF(OR(OR(A22="",B22=""),P22=""),"",IFERROR(P22/(IF(N(H22)&gt;0,H22,IF(N(G22)&gt;0,G22,IF(COUNTIFS($B$12:$B$211,B22,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B22,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B22,$A$5:$A$7,0)))))),""))</f>
-        <v>0</v>
+        <v>0.0625</v>
       </c>
       <c r="R22" s="23" t="str">
         <f aca="false">IF(OR(A22="",B22=""),"",IF(OR(Q22="",COUNTIFS($B$12:$B$211,B22,$Q$12:$Q$211,"&gt;=0")&lt;2),"No Data Yet",IFERROR(IF(Q22/AVERAGEIFS($Q$12:$Q$211,$B$12:$B$211,B22)&gt;=1.2,"Good",IF(Q22/AVERAGEIFS($Q$12:$Q$211,$B$12:$B$211,B22)&gt;=0.8,"Average","Below Standard")),"Average")))</f>
@@ -2197,14 +2209,20 @@
         <v>0</v>
       </c>
       <c r="J23" s="18" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K23" s="18" t="n">
         <v>0</v>
       </c>
-      <c r="L23" s="19"/>
-      <c r="M23" s="19"/>
-      <c r="N23" s="19"/>
+      <c r="L23" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="M23" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="N23" s="18" t="n">
+        <v>0</v>
+      </c>
       <c r="O23" s="20" t="s">
         <v>48</v>
       </c>
@@ -2218,7 +2236,7 @@
       </c>
       <c r="R23" s="23" t="str">
         <f aca="false">IF(OR(A23="",B23=""),"",IF(OR(Q23="",COUNTIFS($B$12:$B$211,B23,$Q$12:$Q$211,"&gt;=0")&lt;2),"No Data Yet",IFERROR(IF(Q23/AVERAGEIFS($Q$12:$Q$211,$B$12:$B$211,B23)&gt;=1.2,"Good",IF(Q23/AVERAGEIFS($Q$12:$Q$211,$B$12:$B$211,B23)&gt;=0.8,"Average","Below Standard")),"Average")))</f>
-        <v>Good</v>
+        <v>Below Standard</v>
       </c>
       <c r="S23" s="24" t="s">
         <v>101</v>
@@ -2227,7 +2245,7 @@
         <v>102</v>
       </c>
       <c r="U23" s="20" t="s">
-        <v>58</v>
+        <v>51</v>
       </c>
       <c r="V23" s="23" t="str">
         <f aca="false">IF(OR(A23="",B23=""),"","https://www.alphanodus.com/contact?utm_source="&amp;IF(B23="X","twitter",LOWER(B23))&amp;"&amp;utm_medium=social&amp;utm_campaign="&amp;IF(D23="","general",LOWER(SUBSTITUTE(SUBSTITUTE(D23," / ","-")," ","-")))&amp;"&amp;utm_content="&amp;LOWER(LEFT(B23,2))&amp;"-"&amp;TEXT(A23,"yymmdd"))</f>
@@ -2261,24 +2279,30 @@
         <v>0</v>
       </c>
       <c r="J24" s="18" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K24" s="18" t="n">
         <v>0</v>
       </c>
-      <c r="L24" s="19"/>
-      <c r="M24" s="19"/>
-      <c r="N24" s="19"/>
+      <c r="L24" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="M24" s="18" t="n">
+        <v>2</v>
+      </c>
+      <c r="N24" s="18" t="n">
+        <v>0</v>
+      </c>
       <c r="O24" s="20" t="s">
         <v>48</v>
       </c>
       <c r="P24" s="21" t="n">
         <f aca="false">IF(OR(A24="",B24=""),"",IF(COUNT(I24:M24)=0,"",SUM(I24:M24)))</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Q24" s="22" t="n">
         <f aca="false">IF(OR(OR(A24="",B24=""),P24=""),"",IFERROR(P24/(IF(N(H24)&gt;0,H24,IF(N(G24)&gt;0,G24,IF(COUNTIFS($B$12:$B$211,B24,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B24,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B24,$A$5:$A$7,0)))))),""))</f>
-        <v>0.0769230769230769</v>
+        <v>0.153846153846154</v>
       </c>
       <c r="R24" s="23" t="str">
         <f aca="false">IF(OR(A24="",B24=""),"",IF(OR(Q24="",COUNTIFS($B$12:$B$211,B24,$Q$12:$Q$211,"&gt;=0")&lt;2),"No Data Yet",IFERROR(IF(Q24/AVERAGEIFS($Q$12:$Q$211,$B$12:$B$211,B24)&gt;=1.2,"Good",IF(Q24/AVERAGEIFS($Q$12:$Q$211,$B$12:$B$211,B24)&gt;=0.8,"Average","Below Standard")),"Average")))</f>

</xml_diff>

<commit_message>
Load Instagram Insights into simple tracker
Adds views, reach, saves, shares, profile visits, link taps and follows
for the four September Instagram posts from Instagram Insights, plus two
story rows (Sep 18 question-box story, Sep 23 four-frame story series).
Engagement rate now divides by impressions/views first on every
platform, matching how LinkedIn and X report it, so rows that do and
don't have reach stay comparable.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019Z3cCo91h4eCLVp6tiH6Ms
</commit_message>
<xml_diff>
--- a/social-media-tracker/AlphaNodus_Simple_Post_Tracker.xlsx
+++ b/social-media-tracker/AlphaNodus_Simple_Post_Tracker.xlsx
@@ -84,7 +84,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">All clicks on the post. LinkedIn: 'Clicks'. X: detail expands + profile visits + link clicks. Both platforms count these in their own engagement rate.</t>
+          <t xml:space="preserve">All clicks on the post. LinkedIn: 'Clicks'. X: detail expands + profile visits + link clicks. Instagram: profile visits + link taps.</t>
         </r>
       </text>
     </comment>
@@ -96,7 +96,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">Followers gained on the post day + the next 2 days. LinkedIn doesn't credit follows to organic posts, so this is the closest fair signal.</t>
+          <t xml:space="preserve">Instagram &amp; X: follows credited to the post. LinkedIn doesn't credit follows to posts, so use followers gained on the post day + the next 2 days.</t>
         </r>
       </text>
     </comment>
@@ -132,7 +132,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">Total Engagement ÷ Reach (or Impressions). Only if no post on that platform has impressions yet: ÷ followers in the box above.</t>
+          <t xml:space="preserve">Total Engagement ÷ Impressions/Views (or Reach if views are missing). Only if no post on that platform has either yet: ÷ followers in the box above.</t>
         </r>
       </text>
     </comment>
@@ -165,7 +165,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="162" uniqueCount="107">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="180" uniqueCount="114">
   <si>
     <t xml:space="preserve">Alpha Nodus — Social Post Tracker</t>
   </si>
@@ -221,7 +221,7 @@
     <t xml:space="preserve">Below Standard = under 0.8× our average</t>
   </si>
   <si>
-    <t xml:space="preserve">X: X analytics export (Sep 1–28). Instagram: public profile, 9/28/2026</t>
+    <t xml:space="preserve">X: X analytics export (Sep 1–28). Instagram: Instagram Insights (9/29/2026)</t>
   </si>
   <si>
     <t xml:space="preserve">Followers Today: update every Monday.</t>
@@ -230,7 +230,7 @@
     <t xml:space="preserve">No Data Yet = numbers not entered, or fewer than 2 posts on that platform</t>
   </si>
   <si>
-    <t xml:space="preserve">Engagement Rate = (likes + comments + shares + saves + clicks) ÷ reach, or ÷ impressions if reach is blank</t>
+    <t xml:space="preserve">Engagement Rate = (likes + comments + shares + saves + clicks) ÷ impressions / views — the way LinkedIn and X calculate it</t>
   </si>
   <si>
     <t xml:space="preserve">Why our own average: each platform behaves differently, and it improves as we post more.</t>
@@ -272,7 +272,7 @@
     <t xml:space="preserve">Clicks</t>
   </si>
   <si>
-    <t xml:space="preserve">New Followers (3 days after post)</t>
+    <t xml:space="preserve">New Followers</t>
   </si>
   <si>
     <t xml:space="preserve">Target List Engaged?</t>
@@ -398,10 +398,10 @@
     <t xml:space="preserve">https://www.instagram.com/alphanodus/reel/DdJxFt3t07x/</t>
   </si>
   <si>
-    <t xml:space="preserve">No comments. 3 minutes is far too long for a Reel.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cut a 20–30 sec Reel with on-screen text. End with 'link in bio to book a demo'.</t>
+    <t xml:space="preserve">Low engagement rate (8 interactions on 224 views), no comments, no profile visits. But it's the only Instagram post reaching new people: 86% of views were non-followers.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Keep making Reels — they reach new people. Cut to 20–30 sec with on-screen text and end with 'link in bio to book a demo'.</t>
   </si>
   <si>
     <t xml:space="preserve">Image: 'Scanners idle a third of the day, next slot 3 weeks out'</t>
@@ -410,7 +410,7 @@
     <t xml:space="preserve">https://www.instagram.com/alphanodus/p/DdRoAPjkqqy/</t>
   </si>
   <si>
-    <t xml:space="preserve">Best Instagram post, but the caption is very long and the 'comment GravityAI' ask got 0 comments.</t>
+    <t xml:space="preserve">Most likes of any post (8) but 0 comments, saves or shares. 3 in 4 views came from existing followers. The 'comment GravityAI' ask got nothing.</t>
   </si>
   <si>
     <t xml:space="preserve">Keep the stat-led visual. Shorten the caption to 3–4 lines with one question at the end.</t>
@@ -422,22 +422,43 @@
     <t xml:space="preserve">https://www.instagram.com/alphanodus/p/DdcD_2JkjH0/</t>
   </si>
   <si>
-    <t xml:space="preserve">Ended with a question but got 0 comments — the question was only in the caption.</t>
+    <t xml:space="preserve">Most profile visits of any post (5) but 0 comments, even though it ended with a question — the question was only in the caption.</t>
   </si>
   <si>
     <t xml:space="preserve">Put the question on the last slide too, with 2–3 answer options people can reply with.</t>
   </si>
   <si>
+    <t xml:space="preserve">Story: 'Wanna see Gravity in action?' question box + website link (shares the carousel)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.instagram.com/alphanodus/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nobody typed an answer in the question box, and 11 of 54 views exited here. 2 likes, 1 link click, 1 profile visit.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Use a one-tap poll instead of a type-in question box. Keep the website link sticker.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Image: 4 manual handoffs before an order is billable</t>
   </si>
   <si>
     <t xml:space="preserve">https://www.instagram.com/alphanodus/p/DdpdTFWN9JR/</t>
   </si>
   <si>
-    <t xml:space="preserve">Weakest Instagram post: text-heavy single image, same theme as Sep 18.</t>
+    <t xml:space="preserve">Fewest views (88) and only 2 likes. Text-heavy single image; second billing post in 5 days.</t>
   </si>
   <si>
     <t xml:space="preserve">Tell process stories as a carousel or short Reel. Avoid two Revenue Cycle posts in a row.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Story series (4 frames): fax poll → handoffs poll → 'Gravity watches' → Book a demo + link</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Best Instagram result for the website: the 'Book a demo' frame got 2 link clicks and the series got 5 profile visits. But 0 votes on both polls, viewers fell from 38 to 29 across the frames, and 96% were existing followers.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Keep the Book-a-demo frame with the link sticker. Cut to 2 frames (hook + demo link) and use one poll at most.</t>
   </si>
   <si>
     <t xml:space="preserve">Video: 3-min Gravity AI explainer + demo link</t>
@@ -1250,8 +1271,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="7"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="10" style="0" width="9"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="12" style="0" width="7"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="0" width="11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="17" min="15" style="0" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="17" min="14" style="0" width="10"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="18" min="18" style="0" width="14"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="20" min="19" style="0" width="40"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="21" min="21" style="0" width="14"/>
@@ -1333,11 +1353,11 @@
       </c>
       <c r="C6" s="8" t="n">
         <f aca="false">COUNTIF($B$12:$B$211,A6)</f>
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="D6" s="9" t="n">
         <f aca="false">IFERROR(AVERAGEIF($B$12:$B$211,A6,$Q$12:$Q$211),"")</f>
-        <v>0.0983606557377049</v>
+        <v>0.0651741237175819</v>
       </c>
       <c r="E6" s="8" t="n">
         <f aca="false">COUNTIFS($B$12:$B$211,A6,$R$12:$R$211,"Good")</f>
@@ -1345,7 +1365,7 @@
       </c>
       <c r="F6" s="8" t="n">
         <f aca="false">COUNTIFS($B$12:$B$211,A6,$R$12:$R$211,"Below Standard")</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H6" s="10" t="s">
         <v>14</v>
@@ -1517,7 +1537,7 @@
         <v>39</v>
       </c>
       <c r="Q12" s="22" t="n">
-        <f aca="false">IF(OR(OR(A12="",B12=""),P12=""),"",IFERROR(P12/(IF(N(H12)&gt;0,H12,IF(N(G12)&gt;0,G12,IF(COUNTIFS($B$12:$B$211,B12,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B12,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B12,$A$5:$A$7,0)))))),""))</f>
+        <f aca="false">IF(OR(OR(A12="",B12=""),P12=""),"",IFERROR(P12/(IF(N(G12)&gt;0,G12,IF(N(H12)&gt;0,H12,IF(COUNTIFS($B$12:$B$211,B12,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B12,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B12,$A$5:$A$7,0)))))),""))</f>
         <v>0.0944309927360775</v>
       </c>
       <c r="R12" s="23" t="str">
@@ -1585,7 +1605,7 @@
         <v>34</v>
       </c>
       <c r="Q13" s="22" t="n">
-        <f aca="false">IF(OR(OR(A13="",B13=""),P13=""),"",IFERROR(P13/(IF(N(H13)&gt;0,H13,IF(N(G13)&gt;0,G13,IF(COUNTIFS($B$12:$B$211,B13,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B13,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B13,$A$5:$A$7,0)))))),""))</f>
+        <f aca="false">IF(OR(OR(A13="",B13=""),P13=""),"",IFERROR(P13/(IF(N(G13)&gt;0,G13,IF(N(H13)&gt;0,H13,IF(COUNTIFS($B$12:$B$211,B13,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B13,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B13,$A$5:$A$7,0)))))),""))</f>
         <v>0.105590062111801</v>
       </c>
       <c r="R13" s="23" t="str">
@@ -1653,7 +1673,7 @@
         <v>25</v>
       </c>
       <c r="Q14" s="22" t="n">
-        <f aca="false">IF(OR(OR(A14="",B14=""),P14=""),"",IFERROR(P14/(IF(N(H14)&gt;0,H14,IF(N(G14)&gt;0,G14,IF(COUNTIFS($B$12:$B$211,B14,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B14,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B14,$A$5:$A$7,0)))))),""))</f>
+        <f aca="false">IF(OR(OR(A14="",B14=""),P14=""),"",IFERROR(P14/(IF(N(G14)&gt;0,G14,IF(N(H14)&gt;0,H14,IF(COUNTIFS($B$12:$B$211,B14,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B14,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B14,$A$5:$A$7,0)))))),""))</f>
         <v>0.115207373271889</v>
       </c>
       <c r="R14" s="23" t="str">
@@ -1721,7 +1741,7 @@
         <v>21</v>
       </c>
       <c r="Q15" s="22" t="n">
-        <f aca="false">IF(OR(OR(A15="",B15=""),P15=""),"",IFERROR(P15/(IF(N(H15)&gt;0,H15,IF(N(G15)&gt;0,G15,IF(COUNTIFS($B$12:$B$211,B15,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B15,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B15,$A$5:$A$7,0)))))),""))</f>
+        <f aca="false">IF(OR(OR(A15="",B15=""),P15=""),"",IFERROR(P15/(IF(N(G15)&gt;0,G15,IF(N(H15)&gt;0,H15,IF(COUNTIFS($B$12:$B$211,B15,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B15,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B15,$A$5:$A$7,0)))))),""))</f>
         <v>0.0897435897435897</v>
       </c>
       <c r="R15" s="23" t="str">
@@ -1781,7 +1801,7 @@
         <v>2</v>
       </c>
       <c r="Q16" s="22" t="str">
-        <f aca="false">IF(OR(OR(A16="",B16=""),P16=""),"",IFERROR(P16/(IF(N(H16)&gt;0,H16,IF(N(G16)&gt;0,G16,IF(COUNTIFS($B$12:$B$211,B16,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B16,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B16,$A$5:$A$7,0)))))),""))</f>
+        <f aca="false">IF(OR(OR(A16="",B16=""),P16=""),"",IFERROR(P16/(IF(N(G16)&gt;0,G16,IF(N(H16)&gt;0,H16,IF(COUNTIFS($B$12:$B$211,B16,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B16,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B16,$A$5:$A$7,0)))))),""))</f>
         <v/>
       </c>
       <c r="R16" s="23" t="str">
@@ -1821,32 +1841,44 @@
       <c r="F17" s="16" t="s">
         <v>76</v>
       </c>
-      <c r="G17" s="19"/>
-      <c r="H17" s="19"/>
+      <c r="G17" s="18" t="n">
+        <v>224</v>
+      </c>
+      <c r="H17" s="18" t="n">
+        <v>158</v>
+      </c>
       <c r="I17" s="18" t="n">
         <v>7</v>
       </c>
       <c r="J17" s="18" t="n">
         <v>0</v>
       </c>
-      <c r="K17" s="19"/>
-      <c r="L17" s="19"/>
-      <c r="M17" s="19"/>
-      <c r="N17" s="19"/>
+      <c r="K17" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="L17" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="M17" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="N17" s="18" t="n">
+        <v>0</v>
+      </c>
       <c r="O17" s="20" t="s">
         <v>48</v>
       </c>
       <c r="P17" s="21" t="n">
         <f aca="false">IF(OR(A17="",B17=""),"",IF(COUNT(I17:M17)=0,"",SUM(I17:M17)))</f>
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="Q17" s="22" t="n">
-        <f aca="false">IF(OR(OR(A17="",B17=""),P17=""),"",IFERROR(P17/(IF(N(H17)&gt;0,H17,IF(N(G17)&gt;0,G17,IF(COUNTIFS($B$12:$B$211,B17,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B17,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B17,$A$5:$A$7,0)))))),""))</f>
-        <v>0.114754098360656</v>
+        <f aca="false">IF(OR(OR(A17="",B17=""),P17=""),"",IFERROR(P17/(IF(N(G17)&gt;0,G17,IF(N(H17)&gt;0,H17,IF(COUNTIFS($B$12:$B$211,B17,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B17,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B17,$A$5:$A$7,0)))))),""))</f>
+        <v>0.0357142857142857</v>
       </c>
       <c r="R17" s="23" t="str">
         <f aca="false">IF(OR(A17="",B17=""),"",IF(OR(Q17="",COUNTIFS($B$12:$B$211,B17,$Q$12:$Q$211,"&gt;=0")&lt;2),"No Data Yet",IFERROR(IF(Q17/AVERAGEIFS($Q$12:$Q$211,$B$12:$B$211,B17)&gt;=1.2,"Good",IF(Q17/AVERAGEIFS($Q$12:$Q$211,$B$12:$B$211,B17)&gt;=0.8,"Average","Below Standard")),"Average")))</f>
-        <v>Average</v>
+        <v>Below Standard</v>
       </c>
       <c r="S17" s="24" t="s">
         <v>77</v>
@@ -1881,32 +1913,44 @@
       <c r="F18" s="16" t="s">
         <v>80</v>
       </c>
-      <c r="G18" s="19"/>
-      <c r="H18" s="19"/>
+      <c r="G18" s="18" t="n">
+        <v>157</v>
+      </c>
+      <c r="H18" s="18" t="n">
+        <v>53</v>
+      </c>
       <c r="I18" s="18" t="n">
         <v>8</v>
       </c>
       <c r="J18" s="18" t="n">
         <v>0</v>
       </c>
-      <c r="K18" s="19"/>
-      <c r="L18" s="19"/>
-      <c r="M18" s="19"/>
-      <c r="N18" s="19"/>
+      <c r="K18" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="L18" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="M18" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="N18" s="18" t="n">
+        <v>0</v>
+      </c>
       <c r="O18" s="20" t="s">
         <v>48</v>
       </c>
       <c r="P18" s="21" t="n">
         <f aca="false">IF(OR(A18="",B18=""),"",IF(COUNT(I18:M18)=0,"",SUM(I18:M18)))</f>
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="Q18" s="22" t="n">
-        <f aca="false">IF(OR(OR(A18="",B18=""),P18=""),"",IFERROR(P18/(IF(N(H18)&gt;0,H18,IF(N(G18)&gt;0,G18,IF(COUNTIFS($B$12:$B$211,B18,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B18,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B18,$A$5:$A$7,0)))))),""))</f>
-        <v>0.131147540983607</v>
+        <f aca="false">IF(OR(OR(A18="",B18=""),P18=""),"",IFERROR(P18/(IF(N(G18)&gt;0,G18,IF(N(H18)&gt;0,H18,IF(COUNTIFS($B$12:$B$211,B18,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B18,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B18,$A$5:$A$7,0)))))),""))</f>
+        <v>0.0573248407643312</v>
       </c>
       <c r="R18" s="23" t="str">
         <f aca="false">IF(OR(A18="",B18=""),"",IF(OR(Q18="",COUNTIFS($B$12:$B$211,B18,$Q$12:$Q$211,"&gt;=0")&lt;2),"No Data Yet",IFERROR(IF(Q18/AVERAGEIFS($Q$12:$Q$211,$B$12:$B$211,B18)&gt;=1.2,"Good",IF(Q18/AVERAGEIFS($Q$12:$Q$211,$B$12:$B$211,B18)&gt;=0.8,"Average","Below Standard")),"Average")))</f>
-        <v>Good</v>
+        <v>Average</v>
       </c>
       <c r="S18" s="24" t="s">
         <v>81</v>
@@ -1941,28 +1985,40 @@
       <c r="F19" s="16" t="s">
         <v>84</v>
       </c>
-      <c r="G19" s="19"/>
-      <c r="H19" s="19"/>
+      <c r="G19" s="18" t="n">
+        <v>183</v>
+      </c>
+      <c r="H19" s="18" t="n">
+        <v>57</v>
+      </c>
       <c r="I19" s="18" t="n">
         <v>7</v>
       </c>
       <c r="J19" s="18" t="n">
         <v>0</v>
       </c>
-      <c r="K19" s="19"/>
-      <c r="L19" s="19"/>
-      <c r="M19" s="19"/>
-      <c r="N19" s="19"/>
+      <c r="K19" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="L19" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="M19" s="18" t="n">
+        <v>5</v>
+      </c>
+      <c r="N19" s="18" t="n">
+        <v>0</v>
+      </c>
       <c r="O19" s="20" t="s">
         <v>48</v>
       </c>
       <c r="P19" s="21" t="n">
         <f aca="false">IF(OR(A19="",B19=""),"",IF(COUNT(I19:M19)=0,"",SUM(I19:M19)))</f>
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="Q19" s="22" t="n">
-        <f aca="false">IF(OR(OR(A19="",B19=""),P19=""),"",IFERROR(P19/(IF(N(H19)&gt;0,H19,IF(N(G19)&gt;0,G19,IF(COUNTIFS($B$12:$B$211,B19,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B19,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B19,$A$5:$A$7,0)))))),""))</f>
-        <v>0.114754098360656</v>
+        <f aca="false">IF(OR(OR(A19="",B19=""),P19=""),"",IFERROR(P19/(IF(N(G19)&gt;0,G19,IF(N(H19)&gt;0,H19,IF(COUNTIFS($B$12:$B$211,B19,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B19,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B19,$A$5:$A$7,0)))))),""))</f>
+        <v>0.0655737704918033</v>
       </c>
       <c r="R19" s="23" t="str">
         <f aca="false">IF(OR(A19="",B19=""),"",IF(OR(Q19="",COUNTIFS($B$12:$B$211,B19,$Q$12:$Q$211,"&gt;=0")&lt;2),"No Data Yet",IFERROR(IF(Q19/AVERAGEIFS($Q$12:$Q$211,$B$12:$B$211,B19)&gt;=1.2,"Good",IF(Q19/AVERAGEIFS($Q$12:$Q$211,$B$12:$B$211,B19)&gt;=0.8,"Average","Below Standard")),"Average")))</f>
@@ -1984,7 +2040,7 @@
     </row>
     <row r="20" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="15" t="n">
-        <v>46288</v>
+        <v>46283</v>
       </c>
       <c r="B20" s="16" t="s">
         <v>13</v>
@@ -1996,37 +2052,47 @@
         <v>60</v>
       </c>
       <c r="E20" s="16" t="s">
-        <v>61</v>
+        <v>46</v>
       </c>
       <c r="F20" s="16" t="s">
         <v>88</v>
       </c>
-      <c r="G20" s="19"/>
-      <c r="H20" s="19"/>
+      <c r="G20" s="18" t="n">
+        <v>54</v>
+      </c>
+      <c r="H20" s="18" t="n">
+        <v>40</v>
+      </c>
       <c r="I20" s="18" t="n">
         <v>2</v>
       </c>
       <c r="J20" s="18" t="n">
         <v>0</v>
       </c>
-      <c r="K20" s="19"/>
+      <c r="K20" s="18" t="n">
+        <v>0</v>
+      </c>
       <c r="L20" s="19"/>
-      <c r="M20" s="19"/>
-      <c r="N20" s="19"/>
+      <c r="M20" s="18" t="n">
+        <v>2</v>
+      </c>
+      <c r="N20" s="18" t="n">
+        <v>0</v>
+      </c>
       <c r="O20" s="20" t="s">
         <v>48</v>
       </c>
       <c r="P20" s="21" t="n">
         <f aca="false">IF(OR(A20="",B20=""),"",IF(COUNT(I20:M20)=0,"",SUM(I20:M20)))</f>
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="Q20" s="22" t="n">
-        <f aca="false">IF(OR(OR(A20="",B20=""),P20=""),"",IFERROR(P20/(IF(N(H20)&gt;0,H20,IF(N(G20)&gt;0,G20,IF(COUNTIFS($B$12:$B$211,B20,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B20,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B20,$A$5:$A$7,0)))))),""))</f>
-        <v>0.0327868852459016</v>
+        <f aca="false">IF(OR(OR(A20="",B20=""),P20=""),"",IFERROR(P20/(IF(N(G20)&gt;0,G20,IF(N(H20)&gt;0,H20,IF(COUNTIFS($B$12:$B$211,B20,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B20,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B20,$A$5:$A$7,0)))))),""))</f>
+        <v>0.0740740740740741</v>
       </c>
       <c r="R20" s="23" t="str">
         <f aca="false">IF(OR(A20="",B20=""),"",IF(OR(Q20="",COUNTIFS($B$12:$B$211,B20,$Q$12:$Q$211,"&gt;=0")&lt;2),"No Data Yet",IFERROR(IF(Q20/AVERAGEIFS($Q$12:$Q$211,$B$12:$B$211,B20)&gt;=1.2,"Good",IF(Q20/AVERAGEIFS($Q$12:$Q$211,$B$12:$B$211,B20)&gt;=0.8,"Average","Below Standard")),"Average")))</f>
-        <v>Below Standard</v>
+        <v>Average</v>
       </c>
       <c r="S20" s="24" t="s">
         <v>89</v>
@@ -2039,34 +2105,36 @@
       </c>
       <c r="V20" s="23" t="str">
         <f aca="false">IF(OR(A20="",B20=""),"","https://www.alphanodus.com/contact?utm_source="&amp;IF(B20="X","twitter",LOWER(B20))&amp;"&amp;utm_medium=social&amp;utm_campaign="&amp;IF(D20="","general",LOWER(SUBSTITUTE(SUBSTITUTE(D20," / ","-")," ","-")))&amp;"&amp;utm_content="&amp;LOWER(LEFT(B20,2))&amp;"-"&amp;TEXT(A20,"yymmdd"))</f>
-        <v>https://www.alphanodus.com/contact?utm_source=instagram&amp;utm_medium=social&amp;utm_campaign=revenue-cycle&amp;utm_content=in-260923</v>
+        <v>https://www.alphanodus.com/contact?utm_source=instagram&amp;utm_medium=social&amp;utm_campaign=revenue-cycle&amp;utm_content=in-260918</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="15" t="n">
-        <v>46276</v>
+        <v>46288</v>
       </c>
       <c r="B21" s="16" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="C21" s="17" t="s">
         <v>91</v>
       </c>
       <c r="D21" s="16" t="s">
-        <v>45</v>
+        <v>60</v>
       </c>
       <c r="E21" s="16" t="s">
-        <v>46</v>
+        <v>61</v>
       </c>
       <c r="F21" s="16" t="s">
         <v>92</v>
       </c>
       <c r="G21" s="18" t="n">
-        <v>27</v>
-      </c>
-      <c r="H21" s="19"/>
+        <v>88</v>
+      </c>
+      <c r="H21" s="18" t="n">
+        <v>37</v>
+      </c>
       <c r="I21" s="18" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J21" s="18" t="n">
         <v>0</v>
@@ -2078,7 +2146,7 @@
         <v>0</v>
       </c>
       <c r="M21" s="18" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="N21" s="18" t="n">
         <v>0</v>
@@ -2088,15 +2156,15 @@
       </c>
       <c r="P21" s="21" t="n">
         <f aca="false">IF(OR(A21="",B21=""),"",IF(COUNT(I21:M21)=0,"",SUM(I21:M21)))</f>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="Q21" s="22" t="n">
-        <f aca="false">IF(OR(OR(A21="",B21=""),P21=""),"",IFERROR(P21/(IF(N(H21)&gt;0,H21,IF(N(G21)&gt;0,G21,IF(COUNTIFS($B$12:$B$211,B21,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B21,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B21,$A$5:$A$7,0)))))),""))</f>
-        <v>0.185185185185185</v>
+        <f aca="false">IF(OR(OR(A21="",B21=""),P21=""),"",IFERROR(P21/(IF(N(G21)&gt;0,G21,IF(N(H21)&gt;0,H21,IF(COUNTIFS($B$12:$B$211,B21,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B21,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B21,$A$5:$A$7,0)))))),""))</f>
+        <v>0.0454545454545455</v>
       </c>
       <c r="R21" s="23" t="str">
         <f aca="false">IF(OR(A21="",B21=""),"",IF(OR(Q21="",COUNTIFS($B$12:$B$211,B21,$Q$12:$Q$211,"&gt;=0")&lt;2),"No Data Yet",IFERROR(IF(Q21/AVERAGEIFS($Q$12:$Q$211,$B$12:$B$211,B21)&gt;=1.2,"Good",IF(Q21/AVERAGEIFS($Q$12:$Q$211,$B$12:$B$211,B21)&gt;=0.8,"Average","Below Standard")),"Average")))</f>
-        <v>Good</v>
+        <v>Below Standard</v>
       </c>
       <c r="S21" s="24" t="s">
         <v>93</v>
@@ -2109,32 +2177,34 @@
       </c>
       <c r="V21" s="23" t="str">
         <f aca="false">IF(OR(A21="",B21=""),"","https://www.alphanodus.com/contact?utm_source="&amp;IF(B21="X","twitter",LOWER(B21))&amp;"&amp;utm_medium=social&amp;utm_campaign="&amp;IF(D21="","general",LOWER(SUBSTITUTE(SUBSTITUTE(D21," / ","-")," ","-")))&amp;"&amp;utm_content="&amp;LOWER(LEFT(B21,2))&amp;"-"&amp;TEXT(A21,"yymmdd"))</f>
-        <v>https://www.alphanodus.com/contact?utm_source=twitter&amp;utm_medium=social&amp;utm_campaign=product-demo&amp;utm_content=x-260911</v>
+        <v>https://www.alphanodus.com/contact?utm_source=instagram&amp;utm_medium=social&amp;utm_campaign=revenue-cycle&amp;utm_content=in-260923</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="15" t="n">
-        <v>46279</v>
+        <v>46288</v>
       </c>
       <c r="B22" s="16" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="C22" s="17" t="s">
         <v>95</v>
       </c>
       <c r="D22" s="16" t="s">
-        <v>53</v>
+        <v>60</v>
       </c>
       <c r="E22" s="16" t="s">
-        <v>54</v>
+        <v>46</v>
       </c>
       <c r="F22" s="16" t="s">
-        <v>96</v>
+        <v>88</v>
       </c>
       <c r="G22" s="18" t="n">
-        <v>16</v>
-      </c>
-      <c r="H22" s="19"/>
+        <v>62</v>
+      </c>
+      <c r="H22" s="18" t="n">
+        <v>38</v>
+      </c>
       <c r="I22" s="18" t="n">
         <v>0</v>
       </c>
@@ -2144,11 +2214,9 @@
       <c r="K22" s="18" t="n">
         <v>0</v>
       </c>
-      <c r="L22" s="18" t="n">
-        <v>0</v>
-      </c>
+      <c r="L22" s="19"/>
       <c r="M22" s="18" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="N22" s="18" t="n">
         <v>0</v>
@@ -2158,51 +2226,51 @@
       </c>
       <c r="P22" s="21" t="n">
         <f aca="false">IF(OR(A22="",B22=""),"",IF(COUNT(I22:M22)=0,"",SUM(I22:M22)))</f>
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="Q22" s="22" t="n">
-        <f aca="false">IF(OR(OR(A22="",B22=""),P22=""),"",IFERROR(P22/(IF(N(H22)&gt;0,H22,IF(N(G22)&gt;0,G22,IF(COUNTIFS($B$12:$B$211,B22,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B22,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B22,$A$5:$A$7,0)))))),""))</f>
-        <v>0.0625</v>
+        <f aca="false">IF(OR(OR(A22="",B22=""),P22=""),"",IFERROR(P22/(IF(N(G22)&gt;0,G22,IF(N(H22)&gt;0,H22,IF(COUNTIFS($B$12:$B$211,B22,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B22,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B22,$A$5:$A$7,0)))))),""))</f>
+        <v>0.112903225806452</v>
       </c>
       <c r="R22" s="23" t="str">
         <f aca="false">IF(OR(A22="",B22=""),"",IF(OR(Q22="",COUNTIFS($B$12:$B$211,B22,$Q$12:$Q$211,"&gt;=0")&lt;2),"No Data Yet",IFERROR(IF(Q22/AVERAGEIFS($Q$12:$Q$211,$B$12:$B$211,B22)&gt;=1.2,"Good",IF(Q22/AVERAGEIFS($Q$12:$Q$211,$B$12:$B$211,B22)&gt;=0.8,"Average","Below Standard")),"Average")))</f>
-        <v>Below Standard</v>
+        <v>Good</v>
       </c>
       <c r="S22" s="24" t="s">
+        <v>96</v>
+      </c>
+      <c r="T22" s="24" t="s">
         <v>97</v>
       </c>
-      <c r="T22" s="24" t="s">
-        <v>98</v>
-      </c>
       <c r="U22" s="20" t="s">
-        <v>51</v>
+        <v>58</v>
       </c>
       <c r="V22" s="23" t="str">
         <f aca="false">IF(OR(A22="",B22=""),"","https://www.alphanodus.com/contact?utm_source="&amp;IF(B22="X","twitter",LOWER(B22))&amp;"&amp;utm_medium=social&amp;utm_campaign="&amp;IF(D22="","general",LOWER(SUBSTITUTE(SUBSTITUTE(D22," / ","-")," ","-")))&amp;"&amp;utm_content="&amp;LOWER(LEFT(B22,2))&amp;"-"&amp;TEXT(A22,"yymmdd"))</f>
-        <v>https://www.alphanodus.com/contact?utm_source=twitter&amp;utm_medium=social&amp;utm_campaign=operations-tips&amp;utm_content=x-260914</v>
+        <v>https://www.alphanodus.com/contact?utm_source=instagram&amp;utm_medium=social&amp;utm_campaign=revenue-cycle&amp;utm_content=in-260923</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="15" t="n">
-        <v>46283</v>
+        <v>46276</v>
       </c>
       <c r="B23" s="16" t="s">
         <v>16</v>
       </c>
       <c r="C23" s="17" t="s">
+        <v>98</v>
+      </c>
+      <c r="D23" s="16" t="s">
+        <v>45</v>
+      </c>
+      <c r="E23" s="16" t="s">
+        <v>46</v>
+      </c>
+      <c r="F23" s="16" t="s">
         <v>99</v>
       </c>
-      <c r="D23" s="16" t="s">
-        <v>60</v>
-      </c>
-      <c r="E23" s="16" t="s">
-        <v>61</v>
-      </c>
-      <c r="F23" s="16" t="s">
-        <v>100</v>
-      </c>
       <c r="G23" s="18" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="H23" s="19"/>
       <c r="I23" s="18" t="n">
@@ -2218,7 +2286,7 @@
         <v>0</v>
       </c>
       <c r="M23" s="18" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="N23" s="18" t="n">
         <v>0</v>
@@ -2228,51 +2296,51 @@
       </c>
       <c r="P23" s="21" t="n">
         <f aca="false">IF(OR(A23="",B23=""),"",IF(COUNT(I23:M23)=0,"",SUM(I23:M23)))</f>
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="Q23" s="22" t="n">
-        <f aca="false">IF(OR(OR(A23="",B23=""),P23=""),"",IFERROR(P23/(IF(N(H23)&gt;0,H23,IF(N(G23)&gt;0,G23,IF(COUNTIFS($B$12:$B$211,B23,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B23,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B23,$A$5:$A$7,0)))))),""))</f>
-        <v>0.0384615384615385</v>
+        <f aca="false">IF(OR(OR(A23="",B23=""),P23=""),"",IFERROR(P23/(IF(N(G23)&gt;0,G23,IF(N(H23)&gt;0,H23,IF(COUNTIFS($B$12:$B$211,B23,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B23,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B23,$A$5:$A$7,0)))))),""))</f>
+        <v>0.185185185185185</v>
       </c>
       <c r="R23" s="23" t="str">
         <f aca="false">IF(OR(A23="",B23=""),"",IF(OR(Q23="",COUNTIFS($B$12:$B$211,B23,$Q$12:$Q$211,"&gt;=0")&lt;2),"No Data Yet",IFERROR(IF(Q23/AVERAGEIFS($Q$12:$Q$211,$B$12:$B$211,B23)&gt;=1.2,"Good",IF(Q23/AVERAGEIFS($Q$12:$Q$211,$B$12:$B$211,B23)&gt;=0.8,"Average","Below Standard")),"Average")))</f>
-        <v>Below Standard</v>
+        <v>Good</v>
       </c>
       <c r="S23" s="24" t="s">
+        <v>100</v>
+      </c>
+      <c r="T23" s="24" t="s">
         <v>101</v>
-      </c>
-      <c r="T23" s="24" t="s">
-        <v>102</v>
       </c>
       <c r="U23" s="20" t="s">
         <v>51</v>
       </c>
       <c r="V23" s="23" t="str">
         <f aca="false">IF(OR(A23="",B23=""),"","https://www.alphanodus.com/contact?utm_source="&amp;IF(B23="X","twitter",LOWER(B23))&amp;"&amp;utm_medium=social&amp;utm_campaign="&amp;IF(D23="","general",LOWER(SUBSTITUTE(SUBSTITUTE(D23," / ","-")," ","-")))&amp;"&amp;utm_content="&amp;LOWER(LEFT(B23,2))&amp;"-"&amp;TEXT(A23,"yymmdd"))</f>
-        <v>https://www.alphanodus.com/contact?utm_source=twitter&amp;utm_medium=social&amp;utm_campaign=revenue-cycle&amp;utm_content=x-260918</v>
+        <v>https://www.alphanodus.com/contact?utm_source=twitter&amp;utm_medium=social&amp;utm_campaign=product-demo&amp;utm_content=x-260911</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="15" t="n">
-        <v>46288</v>
+        <v>46279</v>
       </c>
       <c r="B24" s="16" t="s">
         <v>16</v>
       </c>
       <c r="C24" s="17" t="s">
+        <v>102</v>
+      </c>
+      <c r="D24" s="16" t="s">
+        <v>53</v>
+      </c>
+      <c r="E24" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="F24" s="16" t="s">
         <v>103</v>
       </c>
-      <c r="D24" s="16" t="s">
-        <v>60</v>
-      </c>
-      <c r="E24" s="16" t="s">
-        <v>61</v>
-      </c>
-      <c r="F24" s="16" t="s">
-        <v>104</v>
-      </c>
       <c r="G24" s="18" t="n">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="H24" s="19"/>
       <c r="I24" s="18" t="n">
@@ -2288,7 +2356,7 @@
         <v>0</v>
       </c>
       <c r="M24" s="18" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N24" s="18" t="n">
         <v>0</v>
@@ -2298,100 +2366,168 @@
       </c>
       <c r="P24" s="21" t="n">
         <f aca="false">IF(OR(A24="",B24=""),"",IF(COUNT(I24:M24)=0,"",SUM(I24:M24)))</f>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="Q24" s="22" t="n">
-        <f aca="false">IF(OR(OR(A24="",B24=""),P24=""),"",IFERROR(P24/(IF(N(H24)&gt;0,H24,IF(N(G24)&gt;0,G24,IF(COUNTIFS($B$12:$B$211,B24,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B24,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B24,$A$5:$A$7,0)))))),""))</f>
-        <v>0.153846153846154</v>
+        <f aca="false">IF(OR(OR(A24="",B24=""),P24=""),"",IFERROR(P24/(IF(N(G24)&gt;0,G24,IF(N(H24)&gt;0,H24,IF(COUNTIFS($B$12:$B$211,B24,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B24,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B24,$A$5:$A$7,0)))))),""))</f>
+        <v>0.0625</v>
       </c>
       <c r="R24" s="23" t="str">
         <f aca="false">IF(OR(A24="",B24=""),"",IF(OR(Q24="",COUNTIFS($B$12:$B$211,B24,$Q$12:$Q$211,"&gt;=0")&lt;2),"No Data Yet",IFERROR(IF(Q24/AVERAGEIFS($Q$12:$Q$211,$B$12:$B$211,B24)&gt;=1.2,"Good",IF(Q24/AVERAGEIFS($Q$12:$Q$211,$B$12:$B$211,B24)&gt;=0.8,"Average","Below Standard")),"Average")))</f>
-        <v>Good</v>
+        <v>Below Standard</v>
       </c>
       <c r="S24" s="24" t="s">
+        <v>104</v>
+      </c>
+      <c r="T24" s="24" t="s">
         <v>105</v>
-      </c>
-      <c r="T24" s="24" t="s">
-        <v>106</v>
       </c>
       <c r="U24" s="20" t="s">
         <v>51</v>
       </c>
       <c r="V24" s="23" t="str">
         <f aca="false">IF(OR(A24="",B24=""),"","https://www.alphanodus.com/contact?utm_source="&amp;IF(B24="X","twitter",LOWER(B24))&amp;"&amp;utm_medium=social&amp;utm_campaign="&amp;IF(D24="","general",LOWER(SUBSTITUTE(SUBSTITUTE(D24," / ","-")," ","-")))&amp;"&amp;utm_content="&amp;LOWER(LEFT(B24,2))&amp;"-"&amp;TEXT(A24,"yymmdd"))</f>
-        <v>https://www.alphanodus.com/contact?utm_source=twitter&amp;utm_medium=social&amp;utm_campaign=revenue-cycle&amp;utm_content=x-260923</v>
-      </c>
-    </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="25"/>
-      <c r="B25" s="20"/>
-      <c r="C25" s="24"/>
-      <c r="D25" s="20"/>
-      <c r="E25" s="20"/>
-      <c r="F25" s="20"/>
-      <c r="G25" s="19"/>
+        <v>https://www.alphanodus.com/contact?utm_source=twitter&amp;utm_medium=social&amp;utm_campaign=operations-tips&amp;utm_content=x-260914</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A25" s="15" t="n">
+        <v>46283</v>
+      </c>
+      <c r="B25" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="C25" s="17" t="s">
+        <v>106</v>
+      </c>
+      <c r="D25" s="16" t="s">
+        <v>60</v>
+      </c>
+      <c r="E25" s="16" t="s">
+        <v>61</v>
+      </c>
+      <c r="F25" s="16" t="s">
+        <v>107</v>
+      </c>
+      <c r="G25" s="18" t="n">
+        <v>26</v>
+      </c>
       <c r="H25" s="19"/>
-      <c r="I25" s="19"/>
-      <c r="J25" s="19"/>
-      <c r="K25" s="19"/>
-      <c r="L25" s="19"/>
-      <c r="M25" s="19"/>
-      <c r="N25" s="19"/>
-      <c r="O25" s="20"/>
-      <c r="P25" s="21" t="str">
+      <c r="I25" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="J25" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="K25" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="L25" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="M25" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="N25" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="O25" s="20" t="s">
+        <v>48</v>
+      </c>
+      <c r="P25" s="21" t="n">
         <f aca="false">IF(OR(A25="",B25=""),"",IF(COUNT(I25:M25)=0,"",SUM(I25:M25)))</f>
-        <v/>
-      </c>
-      <c r="Q25" s="22" t="str">
-        <f aca="false">IF(OR(OR(A25="",B25=""),P25=""),"",IFERROR(P25/(IF(N(H25)&gt;0,H25,IF(N(G25)&gt;0,G25,IF(COUNTIFS($B$12:$B$211,B25,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B25,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B25,$A$5:$A$7,0)))))),""))</f>
-        <v/>
+        <v>1</v>
+      </c>
+      <c r="Q25" s="22" t="n">
+        <f aca="false">IF(OR(OR(A25="",B25=""),P25=""),"",IFERROR(P25/(IF(N(G25)&gt;0,G25,IF(N(H25)&gt;0,H25,IF(COUNTIFS($B$12:$B$211,B25,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B25,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B25,$A$5:$A$7,0)))))),""))</f>
+        <v>0.0384615384615385</v>
       </c>
       <c r="R25" s="23" t="str">
         <f aca="false">IF(OR(A25="",B25=""),"",IF(OR(Q25="",COUNTIFS($B$12:$B$211,B25,$Q$12:$Q$211,"&gt;=0")&lt;2),"No Data Yet",IFERROR(IF(Q25/AVERAGEIFS($Q$12:$Q$211,$B$12:$B$211,B25)&gt;=1.2,"Good",IF(Q25/AVERAGEIFS($Q$12:$Q$211,$B$12:$B$211,B25)&gt;=0.8,"Average","Below Standard")),"Average")))</f>
-        <v/>
-      </c>
-      <c r="S25" s="24"/>
-      <c r="T25" s="24"/>
-      <c r="U25" s="20"/>
+        <v>Below Standard</v>
+      </c>
+      <c r="S25" s="24" t="s">
+        <v>108</v>
+      </c>
+      <c r="T25" s="24" t="s">
+        <v>109</v>
+      </c>
+      <c r="U25" s="20" t="s">
+        <v>51</v>
+      </c>
       <c r="V25" s="23" t="str">
         <f aca="false">IF(OR(A25="",B25=""),"","https://www.alphanodus.com/contact?utm_source="&amp;IF(B25="X","twitter",LOWER(B25))&amp;"&amp;utm_medium=social&amp;utm_campaign="&amp;IF(D25="","general",LOWER(SUBSTITUTE(SUBSTITUTE(D25," / ","-")," ","-")))&amp;"&amp;utm_content="&amp;LOWER(LEFT(B25,2))&amp;"-"&amp;TEXT(A25,"yymmdd"))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="25"/>
-      <c r="B26" s="20"/>
-      <c r="C26" s="24"/>
-      <c r="D26" s="20"/>
-      <c r="E26" s="20"/>
-      <c r="F26" s="20"/>
-      <c r="G26" s="19"/>
+        <v>https://www.alphanodus.com/contact?utm_source=twitter&amp;utm_medium=social&amp;utm_campaign=revenue-cycle&amp;utm_content=x-260918</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="54" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A26" s="15" t="n">
+        <v>46288</v>
+      </c>
+      <c r="B26" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="C26" s="17" t="s">
+        <v>110</v>
+      </c>
+      <c r="D26" s="16" t="s">
+        <v>60</v>
+      </c>
+      <c r="E26" s="16" t="s">
+        <v>61</v>
+      </c>
+      <c r="F26" s="16" t="s">
+        <v>111</v>
+      </c>
+      <c r="G26" s="18" t="n">
+        <v>13</v>
+      </c>
       <c r="H26" s="19"/>
-      <c r="I26" s="19"/>
-      <c r="J26" s="19"/>
-      <c r="K26" s="19"/>
-      <c r="L26" s="19"/>
-      <c r="M26" s="19"/>
-      <c r="N26" s="19"/>
-      <c r="O26" s="20"/>
-      <c r="P26" s="21" t="str">
+      <c r="I26" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="J26" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="K26" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="L26" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="M26" s="18" t="n">
+        <v>2</v>
+      </c>
+      <c r="N26" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="O26" s="20" t="s">
+        <v>48</v>
+      </c>
+      <c r="P26" s="21" t="n">
         <f aca="false">IF(OR(A26="",B26=""),"",IF(COUNT(I26:M26)=0,"",SUM(I26:M26)))</f>
-        <v/>
-      </c>
-      <c r="Q26" s="22" t="str">
-        <f aca="false">IF(OR(OR(A26="",B26=""),P26=""),"",IFERROR(P26/(IF(N(H26)&gt;0,H26,IF(N(G26)&gt;0,G26,IF(COUNTIFS($B$12:$B$211,B26,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B26,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B26,$A$5:$A$7,0)))))),""))</f>
-        <v/>
+        <v>2</v>
+      </c>
+      <c r="Q26" s="22" t="n">
+        <f aca="false">IF(OR(OR(A26="",B26=""),P26=""),"",IFERROR(P26/(IF(N(G26)&gt;0,G26,IF(N(H26)&gt;0,H26,IF(COUNTIFS($B$12:$B$211,B26,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B26,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B26,$A$5:$A$7,0)))))),""))</f>
+        <v>0.153846153846154</v>
       </c>
       <c r="R26" s="23" t="str">
         <f aca="false">IF(OR(A26="",B26=""),"",IF(OR(Q26="",COUNTIFS($B$12:$B$211,B26,$Q$12:$Q$211,"&gt;=0")&lt;2),"No Data Yet",IFERROR(IF(Q26/AVERAGEIFS($Q$12:$Q$211,$B$12:$B$211,B26)&gt;=1.2,"Good",IF(Q26/AVERAGEIFS($Q$12:$Q$211,$B$12:$B$211,B26)&gt;=0.8,"Average","Below Standard")),"Average")))</f>
-        <v/>
-      </c>
-      <c r="S26" s="24"/>
-      <c r="T26" s="24"/>
-      <c r="U26" s="20"/>
+        <v>Good</v>
+      </c>
+      <c r="S26" s="24" t="s">
+        <v>112</v>
+      </c>
+      <c r="T26" s="24" t="s">
+        <v>113</v>
+      </c>
+      <c r="U26" s="20" t="s">
+        <v>51</v>
+      </c>
       <c r="V26" s="23" t="str">
         <f aca="false">IF(OR(A26="",B26=""),"","https://www.alphanodus.com/contact?utm_source="&amp;IF(B26="X","twitter",LOWER(B26))&amp;"&amp;utm_medium=social&amp;utm_campaign="&amp;IF(D26="","general",LOWER(SUBSTITUTE(SUBSTITUTE(D26," / ","-")," ","-")))&amp;"&amp;utm_content="&amp;LOWER(LEFT(B26,2))&amp;"-"&amp;TEXT(A26,"yymmdd"))</f>
-        <v/>
+        <v>https://www.alphanodus.com/contact?utm_source=twitter&amp;utm_medium=social&amp;utm_campaign=revenue-cycle&amp;utm_content=x-260923</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2415,7 +2551,7 @@
         <v/>
       </c>
       <c r="Q27" s="22" t="str">
-        <f aca="false">IF(OR(OR(A27="",B27=""),P27=""),"",IFERROR(P27/(IF(N(H27)&gt;0,H27,IF(N(G27)&gt;0,G27,IF(COUNTIFS($B$12:$B$211,B27,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B27,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B27,$A$5:$A$7,0)))))),""))</f>
+        <f aca="false">IF(OR(OR(A27="",B27=""),P27=""),"",IFERROR(P27/(IF(N(G27)&gt;0,G27,IF(N(H27)&gt;0,H27,IF(COUNTIFS($B$12:$B$211,B27,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B27,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B27,$A$5:$A$7,0)))))),""))</f>
         <v/>
       </c>
       <c r="R27" s="23" t="str">
@@ -2451,7 +2587,7 @@
         <v/>
       </c>
       <c r="Q28" s="22" t="str">
-        <f aca="false">IF(OR(OR(A28="",B28=""),P28=""),"",IFERROR(P28/(IF(N(H28)&gt;0,H28,IF(N(G28)&gt;0,G28,IF(COUNTIFS($B$12:$B$211,B28,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B28,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B28,$A$5:$A$7,0)))))),""))</f>
+        <f aca="false">IF(OR(OR(A28="",B28=""),P28=""),"",IFERROR(P28/(IF(N(G28)&gt;0,G28,IF(N(H28)&gt;0,H28,IF(COUNTIFS($B$12:$B$211,B28,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B28,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B28,$A$5:$A$7,0)))))),""))</f>
         <v/>
       </c>
       <c r="R28" s="23" t="str">
@@ -2487,7 +2623,7 @@
         <v/>
       </c>
       <c r="Q29" s="22" t="str">
-        <f aca="false">IF(OR(OR(A29="",B29=""),P29=""),"",IFERROR(P29/(IF(N(H29)&gt;0,H29,IF(N(G29)&gt;0,G29,IF(COUNTIFS($B$12:$B$211,B29,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B29,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B29,$A$5:$A$7,0)))))),""))</f>
+        <f aca="false">IF(OR(OR(A29="",B29=""),P29=""),"",IFERROR(P29/(IF(N(G29)&gt;0,G29,IF(N(H29)&gt;0,H29,IF(COUNTIFS($B$12:$B$211,B29,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B29,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B29,$A$5:$A$7,0)))))),""))</f>
         <v/>
       </c>
       <c r="R29" s="23" t="str">
@@ -2523,7 +2659,7 @@
         <v/>
       </c>
       <c r="Q30" s="22" t="str">
-        <f aca="false">IF(OR(OR(A30="",B30=""),P30=""),"",IFERROR(P30/(IF(N(H30)&gt;0,H30,IF(N(G30)&gt;0,G30,IF(COUNTIFS($B$12:$B$211,B30,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B30,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B30,$A$5:$A$7,0)))))),""))</f>
+        <f aca="false">IF(OR(OR(A30="",B30=""),P30=""),"",IFERROR(P30/(IF(N(G30)&gt;0,G30,IF(N(H30)&gt;0,H30,IF(COUNTIFS($B$12:$B$211,B30,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B30,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B30,$A$5:$A$7,0)))))),""))</f>
         <v/>
       </c>
       <c r="R30" s="23" t="str">
@@ -2559,7 +2695,7 @@
         <v/>
       </c>
       <c r="Q31" s="22" t="str">
-        <f aca="false">IF(OR(OR(A31="",B31=""),P31=""),"",IFERROR(P31/(IF(N(H31)&gt;0,H31,IF(N(G31)&gt;0,G31,IF(COUNTIFS($B$12:$B$211,B31,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B31,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B31,$A$5:$A$7,0)))))),""))</f>
+        <f aca="false">IF(OR(OR(A31="",B31=""),P31=""),"",IFERROR(P31/(IF(N(G31)&gt;0,G31,IF(N(H31)&gt;0,H31,IF(COUNTIFS($B$12:$B$211,B31,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B31,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B31,$A$5:$A$7,0)))))),""))</f>
         <v/>
       </c>
       <c r="R31" s="23" t="str">
@@ -2595,7 +2731,7 @@
         <v/>
       </c>
       <c r="Q32" s="22" t="str">
-        <f aca="false">IF(OR(OR(A32="",B32=""),P32=""),"",IFERROR(P32/(IF(N(H32)&gt;0,H32,IF(N(G32)&gt;0,G32,IF(COUNTIFS($B$12:$B$211,B32,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B32,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B32,$A$5:$A$7,0)))))),""))</f>
+        <f aca="false">IF(OR(OR(A32="",B32=""),P32=""),"",IFERROR(P32/(IF(N(G32)&gt;0,G32,IF(N(H32)&gt;0,H32,IF(COUNTIFS($B$12:$B$211,B32,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B32,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B32,$A$5:$A$7,0)))))),""))</f>
         <v/>
       </c>
       <c r="R32" s="23" t="str">
@@ -2631,7 +2767,7 @@
         <v/>
       </c>
       <c r="Q33" s="22" t="str">
-        <f aca="false">IF(OR(OR(A33="",B33=""),P33=""),"",IFERROR(P33/(IF(N(H33)&gt;0,H33,IF(N(G33)&gt;0,G33,IF(COUNTIFS($B$12:$B$211,B33,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B33,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B33,$A$5:$A$7,0)))))),""))</f>
+        <f aca="false">IF(OR(OR(A33="",B33=""),P33=""),"",IFERROR(P33/(IF(N(G33)&gt;0,G33,IF(N(H33)&gt;0,H33,IF(COUNTIFS($B$12:$B$211,B33,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B33,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B33,$A$5:$A$7,0)))))),""))</f>
         <v/>
       </c>
       <c r="R33" s="23" t="str">
@@ -2667,7 +2803,7 @@
         <v/>
       </c>
       <c r="Q34" s="22" t="str">
-        <f aca="false">IF(OR(OR(A34="",B34=""),P34=""),"",IFERROR(P34/(IF(N(H34)&gt;0,H34,IF(N(G34)&gt;0,G34,IF(COUNTIFS($B$12:$B$211,B34,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B34,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B34,$A$5:$A$7,0)))))),""))</f>
+        <f aca="false">IF(OR(OR(A34="",B34=""),P34=""),"",IFERROR(P34/(IF(N(G34)&gt;0,G34,IF(N(H34)&gt;0,H34,IF(COUNTIFS($B$12:$B$211,B34,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B34,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B34,$A$5:$A$7,0)))))),""))</f>
         <v/>
       </c>
       <c r="R34" s="23" t="str">
@@ -2703,7 +2839,7 @@
         <v/>
       </c>
       <c r="Q35" s="22" t="str">
-        <f aca="false">IF(OR(OR(A35="",B35=""),P35=""),"",IFERROR(P35/(IF(N(H35)&gt;0,H35,IF(N(G35)&gt;0,G35,IF(COUNTIFS($B$12:$B$211,B35,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B35,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B35,$A$5:$A$7,0)))))),""))</f>
+        <f aca="false">IF(OR(OR(A35="",B35=""),P35=""),"",IFERROR(P35/(IF(N(G35)&gt;0,G35,IF(N(H35)&gt;0,H35,IF(COUNTIFS($B$12:$B$211,B35,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B35,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B35,$A$5:$A$7,0)))))),""))</f>
         <v/>
       </c>
       <c r="R35" s="23" t="str">
@@ -2739,7 +2875,7 @@
         <v/>
       </c>
       <c r="Q36" s="22" t="str">
-        <f aca="false">IF(OR(OR(A36="",B36=""),P36=""),"",IFERROR(P36/(IF(N(H36)&gt;0,H36,IF(N(G36)&gt;0,G36,IF(COUNTIFS($B$12:$B$211,B36,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B36,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B36,$A$5:$A$7,0)))))),""))</f>
+        <f aca="false">IF(OR(OR(A36="",B36=""),P36=""),"",IFERROR(P36/(IF(N(G36)&gt;0,G36,IF(N(H36)&gt;0,H36,IF(COUNTIFS($B$12:$B$211,B36,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B36,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B36,$A$5:$A$7,0)))))),""))</f>
         <v/>
       </c>
       <c r="R36" s="23" t="str">
@@ -2775,7 +2911,7 @@
         <v/>
       </c>
       <c r="Q37" s="22" t="str">
-        <f aca="false">IF(OR(OR(A37="",B37=""),P37=""),"",IFERROR(P37/(IF(N(H37)&gt;0,H37,IF(N(G37)&gt;0,G37,IF(COUNTIFS($B$12:$B$211,B37,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B37,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B37,$A$5:$A$7,0)))))),""))</f>
+        <f aca="false">IF(OR(OR(A37="",B37=""),P37=""),"",IFERROR(P37/(IF(N(G37)&gt;0,G37,IF(N(H37)&gt;0,H37,IF(COUNTIFS($B$12:$B$211,B37,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B37,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B37,$A$5:$A$7,0)))))),""))</f>
         <v/>
       </c>
       <c r="R37" s="23" t="str">
@@ -2811,7 +2947,7 @@
         <v/>
       </c>
       <c r="Q38" s="22" t="str">
-        <f aca="false">IF(OR(OR(A38="",B38=""),P38=""),"",IFERROR(P38/(IF(N(H38)&gt;0,H38,IF(N(G38)&gt;0,G38,IF(COUNTIFS($B$12:$B$211,B38,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B38,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B38,$A$5:$A$7,0)))))),""))</f>
+        <f aca="false">IF(OR(OR(A38="",B38=""),P38=""),"",IFERROR(P38/(IF(N(G38)&gt;0,G38,IF(N(H38)&gt;0,H38,IF(COUNTIFS($B$12:$B$211,B38,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B38,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B38,$A$5:$A$7,0)))))),""))</f>
         <v/>
       </c>
       <c r="R38" s="23" t="str">
@@ -2847,7 +2983,7 @@
         <v/>
       </c>
       <c r="Q39" s="22" t="str">
-        <f aca="false">IF(OR(OR(A39="",B39=""),P39=""),"",IFERROR(P39/(IF(N(H39)&gt;0,H39,IF(N(G39)&gt;0,G39,IF(COUNTIFS($B$12:$B$211,B39,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B39,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B39,$A$5:$A$7,0)))))),""))</f>
+        <f aca="false">IF(OR(OR(A39="",B39=""),P39=""),"",IFERROR(P39/(IF(N(G39)&gt;0,G39,IF(N(H39)&gt;0,H39,IF(COUNTIFS($B$12:$B$211,B39,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B39,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B39,$A$5:$A$7,0)))))),""))</f>
         <v/>
       </c>
       <c r="R39" s="23" t="str">
@@ -2883,7 +3019,7 @@
         <v/>
       </c>
       <c r="Q40" s="22" t="str">
-        <f aca="false">IF(OR(OR(A40="",B40=""),P40=""),"",IFERROR(P40/(IF(N(H40)&gt;0,H40,IF(N(G40)&gt;0,G40,IF(COUNTIFS($B$12:$B$211,B40,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B40,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B40,$A$5:$A$7,0)))))),""))</f>
+        <f aca="false">IF(OR(OR(A40="",B40=""),P40=""),"",IFERROR(P40/(IF(N(G40)&gt;0,G40,IF(N(H40)&gt;0,H40,IF(COUNTIFS($B$12:$B$211,B40,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B40,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B40,$A$5:$A$7,0)))))),""))</f>
         <v/>
       </c>
       <c r="R40" s="23" t="str">
@@ -2919,7 +3055,7 @@
         <v/>
       </c>
       <c r="Q41" s="22" t="str">
-        <f aca="false">IF(OR(OR(A41="",B41=""),P41=""),"",IFERROR(P41/(IF(N(H41)&gt;0,H41,IF(N(G41)&gt;0,G41,IF(COUNTIFS($B$12:$B$211,B41,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B41,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B41,$A$5:$A$7,0)))))),""))</f>
+        <f aca="false">IF(OR(OR(A41="",B41=""),P41=""),"",IFERROR(P41/(IF(N(G41)&gt;0,G41,IF(N(H41)&gt;0,H41,IF(COUNTIFS($B$12:$B$211,B41,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B41,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B41,$A$5:$A$7,0)))))),""))</f>
         <v/>
       </c>
       <c r="R41" s="23" t="str">
@@ -2955,7 +3091,7 @@
         <v/>
       </c>
       <c r="Q42" s="22" t="str">
-        <f aca="false">IF(OR(OR(A42="",B42=""),P42=""),"",IFERROR(P42/(IF(N(H42)&gt;0,H42,IF(N(G42)&gt;0,G42,IF(COUNTIFS($B$12:$B$211,B42,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B42,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B42,$A$5:$A$7,0)))))),""))</f>
+        <f aca="false">IF(OR(OR(A42="",B42=""),P42=""),"",IFERROR(P42/(IF(N(G42)&gt;0,G42,IF(N(H42)&gt;0,H42,IF(COUNTIFS($B$12:$B$211,B42,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B42,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B42,$A$5:$A$7,0)))))),""))</f>
         <v/>
       </c>
       <c r="R42" s="23" t="str">
@@ -2991,7 +3127,7 @@
         <v/>
       </c>
       <c r="Q43" s="22" t="str">
-        <f aca="false">IF(OR(OR(A43="",B43=""),P43=""),"",IFERROR(P43/(IF(N(H43)&gt;0,H43,IF(N(G43)&gt;0,G43,IF(COUNTIFS($B$12:$B$211,B43,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B43,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B43,$A$5:$A$7,0)))))),""))</f>
+        <f aca="false">IF(OR(OR(A43="",B43=""),P43=""),"",IFERROR(P43/(IF(N(G43)&gt;0,G43,IF(N(H43)&gt;0,H43,IF(COUNTIFS($B$12:$B$211,B43,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B43,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B43,$A$5:$A$7,0)))))),""))</f>
         <v/>
       </c>
       <c r="R43" s="23" t="str">
@@ -3027,7 +3163,7 @@
         <v/>
       </c>
       <c r="Q44" s="22" t="str">
-        <f aca="false">IF(OR(OR(A44="",B44=""),P44=""),"",IFERROR(P44/(IF(N(H44)&gt;0,H44,IF(N(G44)&gt;0,G44,IF(COUNTIFS($B$12:$B$211,B44,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B44,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B44,$A$5:$A$7,0)))))),""))</f>
+        <f aca="false">IF(OR(OR(A44="",B44=""),P44=""),"",IFERROR(P44/(IF(N(G44)&gt;0,G44,IF(N(H44)&gt;0,H44,IF(COUNTIFS($B$12:$B$211,B44,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B44,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B44,$A$5:$A$7,0)))))),""))</f>
         <v/>
       </c>
       <c r="R44" s="23" t="str">
@@ -3063,7 +3199,7 @@
         <v/>
       </c>
       <c r="Q45" s="22" t="str">
-        <f aca="false">IF(OR(OR(A45="",B45=""),P45=""),"",IFERROR(P45/(IF(N(H45)&gt;0,H45,IF(N(G45)&gt;0,G45,IF(COUNTIFS($B$12:$B$211,B45,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B45,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B45,$A$5:$A$7,0)))))),""))</f>
+        <f aca="false">IF(OR(OR(A45="",B45=""),P45=""),"",IFERROR(P45/(IF(N(G45)&gt;0,G45,IF(N(H45)&gt;0,H45,IF(COUNTIFS($B$12:$B$211,B45,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B45,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B45,$A$5:$A$7,0)))))),""))</f>
         <v/>
       </c>
       <c r="R45" s="23" t="str">
@@ -3099,7 +3235,7 @@
         <v/>
       </c>
       <c r="Q46" s="22" t="str">
-        <f aca="false">IF(OR(OR(A46="",B46=""),P46=""),"",IFERROR(P46/(IF(N(H46)&gt;0,H46,IF(N(G46)&gt;0,G46,IF(COUNTIFS($B$12:$B$211,B46,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B46,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B46,$A$5:$A$7,0)))))),""))</f>
+        <f aca="false">IF(OR(OR(A46="",B46=""),P46=""),"",IFERROR(P46/(IF(N(G46)&gt;0,G46,IF(N(H46)&gt;0,H46,IF(COUNTIFS($B$12:$B$211,B46,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B46,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B46,$A$5:$A$7,0)))))),""))</f>
         <v/>
       </c>
       <c r="R46" s="23" t="str">
@@ -3135,7 +3271,7 @@
         <v/>
       </c>
       <c r="Q47" s="22" t="str">
-        <f aca="false">IF(OR(OR(A47="",B47=""),P47=""),"",IFERROR(P47/(IF(N(H47)&gt;0,H47,IF(N(G47)&gt;0,G47,IF(COUNTIFS($B$12:$B$211,B47,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B47,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B47,$A$5:$A$7,0)))))),""))</f>
+        <f aca="false">IF(OR(OR(A47="",B47=""),P47=""),"",IFERROR(P47/(IF(N(G47)&gt;0,G47,IF(N(H47)&gt;0,H47,IF(COUNTIFS($B$12:$B$211,B47,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B47,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B47,$A$5:$A$7,0)))))),""))</f>
         <v/>
       </c>
       <c r="R47" s="23" t="str">
@@ -3171,7 +3307,7 @@
         <v/>
       </c>
       <c r="Q48" s="22" t="str">
-        <f aca="false">IF(OR(OR(A48="",B48=""),P48=""),"",IFERROR(P48/(IF(N(H48)&gt;0,H48,IF(N(G48)&gt;0,G48,IF(COUNTIFS($B$12:$B$211,B48,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B48,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B48,$A$5:$A$7,0)))))),""))</f>
+        <f aca="false">IF(OR(OR(A48="",B48=""),P48=""),"",IFERROR(P48/(IF(N(G48)&gt;0,G48,IF(N(H48)&gt;0,H48,IF(COUNTIFS($B$12:$B$211,B48,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B48,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B48,$A$5:$A$7,0)))))),""))</f>
         <v/>
       </c>
       <c r="R48" s="23" t="str">
@@ -3207,7 +3343,7 @@
         <v/>
       </c>
       <c r="Q49" s="22" t="str">
-        <f aca="false">IF(OR(OR(A49="",B49=""),P49=""),"",IFERROR(P49/(IF(N(H49)&gt;0,H49,IF(N(G49)&gt;0,G49,IF(COUNTIFS($B$12:$B$211,B49,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B49,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B49,$A$5:$A$7,0)))))),""))</f>
+        <f aca="false">IF(OR(OR(A49="",B49=""),P49=""),"",IFERROR(P49/(IF(N(G49)&gt;0,G49,IF(N(H49)&gt;0,H49,IF(COUNTIFS($B$12:$B$211,B49,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B49,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B49,$A$5:$A$7,0)))))),""))</f>
         <v/>
       </c>
       <c r="R49" s="23" t="str">
@@ -3243,7 +3379,7 @@
         <v/>
       </c>
       <c r="Q50" s="22" t="str">
-        <f aca="false">IF(OR(OR(A50="",B50=""),P50=""),"",IFERROR(P50/(IF(N(H50)&gt;0,H50,IF(N(G50)&gt;0,G50,IF(COUNTIFS($B$12:$B$211,B50,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B50,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B50,$A$5:$A$7,0)))))),""))</f>
+        <f aca="false">IF(OR(OR(A50="",B50=""),P50=""),"",IFERROR(P50/(IF(N(G50)&gt;0,G50,IF(N(H50)&gt;0,H50,IF(COUNTIFS($B$12:$B$211,B50,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B50,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B50,$A$5:$A$7,0)))))),""))</f>
         <v/>
       </c>
       <c r="R50" s="23" t="str">
@@ -3279,7 +3415,7 @@
         <v/>
       </c>
       <c r="Q51" s="22" t="str">
-        <f aca="false">IF(OR(OR(A51="",B51=""),P51=""),"",IFERROR(P51/(IF(N(H51)&gt;0,H51,IF(N(G51)&gt;0,G51,IF(COUNTIFS($B$12:$B$211,B51,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B51,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B51,$A$5:$A$7,0)))))),""))</f>
+        <f aca="false">IF(OR(OR(A51="",B51=""),P51=""),"",IFERROR(P51/(IF(N(G51)&gt;0,G51,IF(N(H51)&gt;0,H51,IF(COUNTIFS($B$12:$B$211,B51,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B51,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B51,$A$5:$A$7,0)))))),""))</f>
         <v/>
       </c>
       <c r="R51" s="23" t="str">
@@ -3315,7 +3451,7 @@
         <v/>
       </c>
       <c r="Q52" s="22" t="str">
-        <f aca="false">IF(OR(OR(A52="",B52=""),P52=""),"",IFERROR(P52/(IF(N(H52)&gt;0,H52,IF(N(G52)&gt;0,G52,IF(COUNTIFS($B$12:$B$211,B52,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B52,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B52,$A$5:$A$7,0)))))),""))</f>
+        <f aca="false">IF(OR(OR(A52="",B52=""),P52=""),"",IFERROR(P52/(IF(N(G52)&gt;0,G52,IF(N(H52)&gt;0,H52,IF(COUNTIFS($B$12:$B$211,B52,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B52,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B52,$A$5:$A$7,0)))))),""))</f>
         <v/>
       </c>
       <c r="R52" s="23" t="str">
@@ -3351,7 +3487,7 @@
         <v/>
       </c>
       <c r="Q53" s="22" t="str">
-        <f aca="false">IF(OR(OR(A53="",B53=""),P53=""),"",IFERROR(P53/(IF(N(H53)&gt;0,H53,IF(N(G53)&gt;0,G53,IF(COUNTIFS($B$12:$B$211,B53,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B53,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B53,$A$5:$A$7,0)))))),""))</f>
+        <f aca="false">IF(OR(OR(A53="",B53=""),P53=""),"",IFERROR(P53/(IF(N(G53)&gt;0,G53,IF(N(H53)&gt;0,H53,IF(COUNTIFS($B$12:$B$211,B53,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B53,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B53,$A$5:$A$7,0)))))),""))</f>
         <v/>
       </c>
       <c r="R53" s="23" t="str">
@@ -3387,7 +3523,7 @@
         <v/>
       </c>
       <c r="Q54" s="22" t="str">
-        <f aca="false">IF(OR(OR(A54="",B54=""),P54=""),"",IFERROR(P54/(IF(N(H54)&gt;0,H54,IF(N(G54)&gt;0,G54,IF(COUNTIFS($B$12:$B$211,B54,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B54,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B54,$A$5:$A$7,0)))))),""))</f>
+        <f aca="false">IF(OR(OR(A54="",B54=""),P54=""),"",IFERROR(P54/(IF(N(G54)&gt;0,G54,IF(N(H54)&gt;0,H54,IF(COUNTIFS($B$12:$B$211,B54,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B54,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B54,$A$5:$A$7,0)))))),""))</f>
         <v/>
       </c>
       <c r="R54" s="23" t="str">
@@ -3423,7 +3559,7 @@
         <v/>
       </c>
       <c r="Q55" s="22" t="str">
-        <f aca="false">IF(OR(OR(A55="",B55=""),P55=""),"",IFERROR(P55/(IF(N(H55)&gt;0,H55,IF(N(G55)&gt;0,G55,IF(COUNTIFS($B$12:$B$211,B55,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B55,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B55,$A$5:$A$7,0)))))),""))</f>
+        <f aca="false">IF(OR(OR(A55="",B55=""),P55=""),"",IFERROR(P55/(IF(N(G55)&gt;0,G55,IF(N(H55)&gt;0,H55,IF(COUNTIFS($B$12:$B$211,B55,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B55,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B55,$A$5:$A$7,0)))))),""))</f>
         <v/>
       </c>
       <c r="R55" s="23" t="str">
@@ -3459,7 +3595,7 @@
         <v/>
       </c>
       <c r="Q56" s="22" t="str">
-        <f aca="false">IF(OR(OR(A56="",B56=""),P56=""),"",IFERROR(P56/(IF(N(H56)&gt;0,H56,IF(N(G56)&gt;0,G56,IF(COUNTIFS($B$12:$B$211,B56,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B56,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B56,$A$5:$A$7,0)))))),""))</f>
+        <f aca="false">IF(OR(OR(A56="",B56=""),P56=""),"",IFERROR(P56/(IF(N(G56)&gt;0,G56,IF(N(H56)&gt;0,H56,IF(COUNTIFS($B$12:$B$211,B56,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B56,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B56,$A$5:$A$7,0)))))),""))</f>
         <v/>
       </c>
       <c r="R56" s="23" t="str">
@@ -3495,7 +3631,7 @@
         <v/>
       </c>
       <c r="Q57" s="22" t="str">
-        <f aca="false">IF(OR(OR(A57="",B57=""),P57=""),"",IFERROR(P57/(IF(N(H57)&gt;0,H57,IF(N(G57)&gt;0,G57,IF(COUNTIFS($B$12:$B$211,B57,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B57,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B57,$A$5:$A$7,0)))))),""))</f>
+        <f aca="false">IF(OR(OR(A57="",B57=""),P57=""),"",IFERROR(P57/(IF(N(G57)&gt;0,G57,IF(N(H57)&gt;0,H57,IF(COUNTIFS($B$12:$B$211,B57,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B57,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B57,$A$5:$A$7,0)))))),""))</f>
         <v/>
       </c>
       <c r="R57" s="23" t="str">
@@ -3531,7 +3667,7 @@
         <v/>
       </c>
       <c r="Q58" s="22" t="str">
-        <f aca="false">IF(OR(OR(A58="",B58=""),P58=""),"",IFERROR(P58/(IF(N(H58)&gt;0,H58,IF(N(G58)&gt;0,G58,IF(COUNTIFS($B$12:$B$211,B58,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B58,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B58,$A$5:$A$7,0)))))),""))</f>
+        <f aca="false">IF(OR(OR(A58="",B58=""),P58=""),"",IFERROR(P58/(IF(N(G58)&gt;0,G58,IF(N(H58)&gt;0,H58,IF(COUNTIFS($B$12:$B$211,B58,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B58,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B58,$A$5:$A$7,0)))))),""))</f>
         <v/>
       </c>
       <c r="R58" s="23" t="str">
@@ -3567,7 +3703,7 @@
         <v/>
       </c>
       <c r="Q59" s="22" t="str">
-        <f aca="false">IF(OR(OR(A59="",B59=""),P59=""),"",IFERROR(P59/(IF(N(H59)&gt;0,H59,IF(N(G59)&gt;0,G59,IF(COUNTIFS($B$12:$B$211,B59,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B59,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B59,$A$5:$A$7,0)))))),""))</f>
+        <f aca="false">IF(OR(OR(A59="",B59=""),P59=""),"",IFERROR(P59/(IF(N(G59)&gt;0,G59,IF(N(H59)&gt;0,H59,IF(COUNTIFS($B$12:$B$211,B59,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B59,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B59,$A$5:$A$7,0)))))),""))</f>
         <v/>
       </c>
       <c r="R59" s="23" t="str">
@@ -3603,7 +3739,7 @@
         <v/>
       </c>
       <c r="Q60" s="22" t="str">
-        <f aca="false">IF(OR(OR(A60="",B60=""),P60=""),"",IFERROR(P60/(IF(N(H60)&gt;0,H60,IF(N(G60)&gt;0,G60,IF(COUNTIFS($B$12:$B$211,B60,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B60,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B60,$A$5:$A$7,0)))))),""))</f>
+        <f aca="false">IF(OR(OR(A60="",B60=""),P60=""),"",IFERROR(P60/(IF(N(G60)&gt;0,G60,IF(N(H60)&gt;0,H60,IF(COUNTIFS($B$12:$B$211,B60,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B60,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B60,$A$5:$A$7,0)))))),""))</f>
         <v/>
       </c>
       <c r="R60" s="23" t="str">
@@ -3639,7 +3775,7 @@
         <v/>
       </c>
       <c r="Q61" s="22" t="str">
-        <f aca="false">IF(OR(OR(A61="",B61=""),P61=""),"",IFERROR(P61/(IF(N(H61)&gt;0,H61,IF(N(G61)&gt;0,G61,IF(COUNTIFS($B$12:$B$211,B61,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B61,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B61,$A$5:$A$7,0)))))),""))</f>
+        <f aca="false">IF(OR(OR(A61="",B61=""),P61=""),"",IFERROR(P61/(IF(N(G61)&gt;0,G61,IF(N(H61)&gt;0,H61,IF(COUNTIFS($B$12:$B$211,B61,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B61,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B61,$A$5:$A$7,0)))))),""))</f>
         <v/>
       </c>
       <c r="R61" s="23" t="str">
@@ -3675,7 +3811,7 @@
         <v/>
       </c>
       <c r="Q62" s="22" t="str">
-        <f aca="false">IF(OR(OR(A62="",B62=""),P62=""),"",IFERROR(P62/(IF(N(H62)&gt;0,H62,IF(N(G62)&gt;0,G62,IF(COUNTIFS($B$12:$B$211,B62,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B62,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B62,$A$5:$A$7,0)))))),""))</f>
+        <f aca="false">IF(OR(OR(A62="",B62=""),P62=""),"",IFERROR(P62/(IF(N(G62)&gt;0,G62,IF(N(H62)&gt;0,H62,IF(COUNTIFS($B$12:$B$211,B62,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B62,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B62,$A$5:$A$7,0)))))),""))</f>
         <v/>
       </c>
       <c r="R62" s="23" t="str">
@@ -3711,7 +3847,7 @@
         <v/>
       </c>
       <c r="Q63" s="22" t="str">
-        <f aca="false">IF(OR(OR(A63="",B63=""),P63=""),"",IFERROR(P63/(IF(N(H63)&gt;0,H63,IF(N(G63)&gt;0,G63,IF(COUNTIFS($B$12:$B$211,B63,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B63,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B63,$A$5:$A$7,0)))))),""))</f>
+        <f aca="false">IF(OR(OR(A63="",B63=""),P63=""),"",IFERROR(P63/(IF(N(G63)&gt;0,G63,IF(N(H63)&gt;0,H63,IF(COUNTIFS($B$12:$B$211,B63,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B63,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B63,$A$5:$A$7,0)))))),""))</f>
         <v/>
       </c>
       <c r="R63" s="23" t="str">
@@ -3747,7 +3883,7 @@
         <v/>
       </c>
       <c r="Q64" s="22" t="str">
-        <f aca="false">IF(OR(OR(A64="",B64=""),P64=""),"",IFERROR(P64/(IF(N(H64)&gt;0,H64,IF(N(G64)&gt;0,G64,IF(COUNTIFS($B$12:$B$211,B64,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B64,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B64,$A$5:$A$7,0)))))),""))</f>
+        <f aca="false">IF(OR(OR(A64="",B64=""),P64=""),"",IFERROR(P64/(IF(N(G64)&gt;0,G64,IF(N(H64)&gt;0,H64,IF(COUNTIFS($B$12:$B$211,B64,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B64,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B64,$A$5:$A$7,0)))))),""))</f>
         <v/>
       </c>
       <c r="R64" s="23" t="str">
@@ -3783,7 +3919,7 @@
         <v/>
       </c>
       <c r="Q65" s="22" t="str">
-        <f aca="false">IF(OR(OR(A65="",B65=""),P65=""),"",IFERROR(P65/(IF(N(H65)&gt;0,H65,IF(N(G65)&gt;0,G65,IF(COUNTIFS($B$12:$B$211,B65,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B65,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B65,$A$5:$A$7,0)))))),""))</f>
+        <f aca="false">IF(OR(OR(A65="",B65=""),P65=""),"",IFERROR(P65/(IF(N(G65)&gt;0,G65,IF(N(H65)&gt;0,H65,IF(COUNTIFS($B$12:$B$211,B65,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B65,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B65,$A$5:$A$7,0)))))),""))</f>
         <v/>
       </c>
       <c r="R65" s="23" t="str">
@@ -3819,7 +3955,7 @@
         <v/>
       </c>
       <c r="Q66" s="22" t="str">
-        <f aca="false">IF(OR(OR(A66="",B66=""),P66=""),"",IFERROR(P66/(IF(N(H66)&gt;0,H66,IF(N(G66)&gt;0,G66,IF(COUNTIFS($B$12:$B$211,B66,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B66,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B66,$A$5:$A$7,0)))))),""))</f>
+        <f aca="false">IF(OR(OR(A66="",B66=""),P66=""),"",IFERROR(P66/(IF(N(G66)&gt;0,G66,IF(N(H66)&gt;0,H66,IF(COUNTIFS($B$12:$B$211,B66,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B66,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B66,$A$5:$A$7,0)))))),""))</f>
         <v/>
       </c>
       <c r="R66" s="23" t="str">
@@ -3855,7 +3991,7 @@
         <v/>
       </c>
       <c r="Q67" s="22" t="str">
-        <f aca="false">IF(OR(OR(A67="",B67=""),P67=""),"",IFERROR(P67/(IF(N(H67)&gt;0,H67,IF(N(G67)&gt;0,G67,IF(COUNTIFS($B$12:$B$211,B67,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B67,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B67,$A$5:$A$7,0)))))),""))</f>
+        <f aca="false">IF(OR(OR(A67="",B67=""),P67=""),"",IFERROR(P67/(IF(N(G67)&gt;0,G67,IF(N(H67)&gt;0,H67,IF(COUNTIFS($B$12:$B$211,B67,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B67,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B67,$A$5:$A$7,0)))))),""))</f>
         <v/>
       </c>
       <c r="R67" s="23" t="str">
@@ -3891,7 +4027,7 @@
         <v/>
       </c>
       <c r="Q68" s="22" t="str">
-        <f aca="false">IF(OR(OR(A68="",B68=""),P68=""),"",IFERROR(P68/(IF(N(H68)&gt;0,H68,IF(N(G68)&gt;0,G68,IF(COUNTIFS($B$12:$B$211,B68,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B68,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B68,$A$5:$A$7,0)))))),""))</f>
+        <f aca="false">IF(OR(OR(A68="",B68=""),P68=""),"",IFERROR(P68/(IF(N(G68)&gt;0,G68,IF(N(H68)&gt;0,H68,IF(COUNTIFS($B$12:$B$211,B68,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B68,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B68,$A$5:$A$7,0)))))),""))</f>
         <v/>
       </c>
       <c r="R68" s="23" t="str">
@@ -3927,7 +4063,7 @@
         <v/>
       </c>
       <c r="Q69" s="22" t="str">
-        <f aca="false">IF(OR(OR(A69="",B69=""),P69=""),"",IFERROR(P69/(IF(N(H69)&gt;0,H69,IF(N(G69)&gt;0,G69,IF(COUNTIFS($B$12:$B$211,B69,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B69,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B69,$A$5:$A$7,0)))))),""))</f>
+        <f aca="false">IF(OR(OR(A69="",B69=""),P69=""),"",IFERROR(P69/(IF(N(G69)&gt;0,G69,IF(N(H69)&gt;0,H69,IF(COUNTIFS($B$12:$B$211,B69,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B69,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B69,$A$5:$A$7,0)))))),""))</f>
         <v/>
       </c>
       <c r="R69" s="23" t="str">
@@ -3963,7 +4099,7 @@
         <v/>
       </c>
       <c r="Q70" s="22" t="str">
-        <f aca="false">IF(OR(OR(A70="",B70=""),P70=""),"",IFERROR(P70/(IF(N(H70)&gt;0,H70,IF(N(G70)&gt;0,G70,IF(COUNTIFS($B$12:$B$211,B70,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B70,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B70,$A$5:$A$7,0)))))),""))</f>
+        <f aca="false">IF(OR(OR(A70="",B70=""),P70=""),"",IFERROR(P70/(IF(N(G70)&gt;0,G70,IF(N(H70)&gt;0,H70,IF(COUNTIFS($B$12:$B$211,B70,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B70,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B70,$A$5:$A$7,0)))))),""))</f>
         <v/>
       </c>
       <c r="R70" s="23" t="str">
@@ -3999,7 +4135,7 @@
         <v/>
       </c>
       <c r="Q71" s="22" t="str">
-        <f aca="false">IF(OR(OR(A71="",B71=""),P71=""),"",IFERROR(P71/(IF(N(H71)&gt;0,H71,IF(N(G71)&gt;0,G71,IF(COUNTIFS($B$12:$B$211,B71,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B71,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B71,$A$5:$A$7,0)))))),""))</f>
+        <f aca="false">IF(OR(OR(A71="",B71=""),P71=""),"",IFERROR(P71/(IF(N(G71)&gt;0,G71,IF(N(H71)&gt;0,H71,IF(COUNTIFS($B$12:$B$211,B71,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B71,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B71,$A$5:$A$7,0)))))),""))</f>
         <v/>
       </c>
       <c r="R71" s="23" t="str">
@@ -4035,7 +4171,7 @@
         <v/>
       </c>
       <c r="Q72" s="22" t="str">
-        <f aca="false">IF(OR(OR(A72="",B72=""),P72=""),"",IFERROR(P72/(IF(N(H72)&gt;0,H72,IF(N(G72)&gt;0,G72,IF(COUNTIFS($B$12:$B$211,B72,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B72,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B72,$A$5:$A$7,0)))))),""))</f>
+        <f aca="false">IF(OR(OR(A72="",B72=""),P72=""),"",IFERROR(P72/(IF(N(G72)&gt;0,G72,IF(N(H72)&gt;0,H72,IF(COUNTIFS($B$12:$B$211,B72,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B72,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B72,$A$5:$A$7,0)))))),""))</f>
         <v/>
       </c>
       <c r="R72" s="23" t="str">
@@ -4071,7 +4207,7 @@
         <v/>
       </c>
       <c r="Q73" s="22" t="str">
-        <f aca="false">IF(OR(OR(A73="",B73=""),P73=""),"",IFERROR(P73/(IF(N(H73)&gt;0,H73,IF(N(G73)&gt;0,G73,IF(COUNTIFS($B$12:$B$211,B73,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B73,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B73,$A$5:$A$7,0)))))),""))</f>
+        <f aca="false">IF(OR(OR(A73="",B73=""),P73=""),"",IFERROR(P73/(IF(N(G73)&gt;0,G73,IF(N(H73)&gt;0,H73,IF(COUNTIFS($B$12:$B$211,B73,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B73,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B73,$A$5:$A$7,0)))))),""))</f>
         <v/>
       </c>
       <c r="R73" s="23" t="str">
@@ -4107,7 +4243,7 @@
         <v/>
       </c>
       <c r="Q74" s="22" t="str">
-        <f aca="false">IF(OR(OR(A74="",B74=""),P74=""),"",IFERROR(P74/(IF(N(H74)&gt;0,H74,IF(N(G74)&gt;0,G74,IF(COUNTIFS($B$12:$B$211,B74,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B74,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B74,$A$5:$A$7,0)))))),""))</f>
+        <f aca="false">IF(OR(OR(A74="",B74=""),P74=""),"",IFERROR(P74/(IF(N(G74)&gt;0,G74,IF(N(H74)&gt;0,H74,IF(COUNTIFS($B$12:$B$211,B74,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B74,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B74,$A$5:$A$7,0)))))),""))</f>
         <v/>
       </c>
       <c r="R74" s="23" t="str">
@@ -4143,7 +4279,7 @@
         <v/>
       </c>
       <c r="Q75" s="22" t="str">
-        <f aca="false">IF(OR(OR(A75="",B75=""),P75=""),"",IFERROR(P75/(IF(N(H75)&gt;0,H75,IF(N(G75)&gt;0,G75,IF(COUNTIFS($B$12:$B$211,B75,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B75,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B75,$A$5:$A$7,0)))))),""))</f>
+        <f aca="false">IF(OR(OR(A75="",B75=""),P75=""),"",IFERROR(P75/(IF(N(G75)&gt;0,G75,IF(N(H75)&gt;0,H75,IF(COUNTIFS($B$12:$B$211,B75,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B75,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B75,$A$5:$A$7,0)))))),""))</f>
         <v/>
       </c>
       <c r="R75" s="23" t="str">
@@ -4179,7 +4315,7 @@
         <v/>
       </c>
       <c r="Q76" s="22" t="str">
-        <f aca="false">IF(OR(OR(A76="",B76=""),P76=""),"",IFERROR(P76/(IF(N(H76)&gt;0,H76,IF(N(G76)&gt;0,G76,IF(COUNTIFS($B$12:$B$211,B76,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B76,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B76,$A$5:$A$7,0)))))),""))</f>
+        <f aca="false">IF(OR(OR(A76="",B76=""),P76=""),"",IFERROR(P76/(IF(N(G76)&gt;0,G76,IF(N(H76)&gt;0,H76,IF(COUNTIFS($B$12:$B$211,B76,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B76,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B76,$A$5:$A$7,0)))))),""))</f>
         <v/>
       </c>
       <c r="R76" s="23" t="str">
@@ -4215,7 +4351,7 @@
         <v/>
       </c>
       <c r="Q77" s="22" t="str">
-        <f aca="false">IF(OR(OR(A77="",B77=""),P77=""),"",IFERROR(P77/(IF(N(H77)&gt;0,H77,IF(N(G77)&gt;0,G77,IF(COUNTIFS($B$12:$B$211,B77,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B77,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B77,$A$5:$A$7,0)))))),""))</f>
+        <f aca="false">IF(OR(OR(A77="",B77=""),P77=""),"",IFERROR(P77/(IF(N(G77)&gt;0,G77,IF(N(H77)&gt;0,H77,IF(COUNTIFS($B$12:$B$211,B77,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B77,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B77,$A$5:$A$7,0)))))),""))</f>
         <v/>
       </c>
       <c r="R77" s="23" t="str">
@@ -4251,7 +4387,7 @@
         <v/>
       </c>
       <c r="Q78" s="22" t="str">
-        <f aca="false">IF(OR(OR(A78="",B78=""),P78=""),"",IFERROR(P78/(IF(N(H78)&gt;0,H78,IF(N(G78)&gt;0,G78,IF(COUNTIFS($B$12:$B$211,B78,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B78,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B78,$A$5:$A$7,0)))))),""))</f>
+        <f aca="false">IF(OR(OR(A78="",B78=""),P78=""),"",IFERROR(P78/(IF(N(G78)&gt;0,G78,IF(N(H78)&gt;0,H78,IF(COUNTIFS($B$12:$B$211,B78,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B78,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B78,$A$5:$A$7,0)))))),""))</f>
         <v/>
       </c>
       <c r="R78" s="23" t="str">
@@ -4287,7 +4423,7 @@
         <v/>
       </c>
       <c r="Q79" s="22" t="str">
-        <f aca="false">IF(OR(OR(A79="",B79=""),P79=""),"",IFERROR(P79/(IF(N(H79)&gt;0,H79,IF(N(G79)&gt;0,G79,IF(COUNTIFS($B$12:$B$211,B79,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B79,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B79,$A$5:$A$7,0)))))),""))</f>
+        <f aca="false">IF(OR(OR(A79="",B79=""),P79=""),"",IFERROR(P79/(IF(N(G79)&gt;0,G79,IF(N(H79)&gt;0,H79,IF(COUNTIFS($B$12:$B$211,B79,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B79,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B79,$A$5:$A$7,0)))))),""))</f>
         <v/>
       </c>
       <c r="R79" s="23" t="str">
@@ -4323,7 +4459,7 @@
         <v/>
       </c>
       <c r="Q80" s="22" t="str">
-        <f aca="false">IF(OR(OR(A80="",B80=""),P80=""),"",IFERROR(P80/(IF(N(H80)&gt;0,H80,IF(N(G80)&gt;0,G80,IF(COUNTIFS($B$12:$B$211,B80,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B80,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B80,$A$5:$A$7,0)))))),""))</f>
+        <f aca="false">IF(OR(OR(A80="",B80=""),P80=""),"",IFERROR(P80/(IF(N(G80)&gt;0,G80,IF(N(H80)&gt;0,H80,IF(COUNTIFS($B$12:$B$211,B80,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B80,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B80,$A$5:$A$7,0)))))),""))</f>
         <v/>
       </c>
       <c r="R80" s="23" t="str">
@@ -4359,7 +4495,7 @@
         <v/>
       </c>
       <c r="Q81" s="22" t="str">
-        <f aca="false">IF(OR(OR(A81="",B81=""),P81=""),"",IFERROR(P81/(IF(N(H81)&gt;0,H81,IF(N(G81)&gt;0,G81,IF(COUNTIFS($B$12:$B$211,B81,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B81,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B81,$A$5:$A$7,0)))))),""))</f>
+        <f aca="false">IF(OR(OR(A81="",B81=""),P81=""),"",IFERROR(P81/(IF(N(G81)&gt;0,G81,IF(N(H81)&gt;0,H81,IF(COUNTIFS($B$12:$B$211,B81,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B81,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B81,$A$5:$A$7,0)))))),""))</f>
         <v/>
       </c>
       <c r="R81" s="23" t="str">
@@ -4395,7 +4531,7 @@
         <v/>
       </c>
       <c r="Q82" s="22" t="str">
-        <f aca="false">IF(OR(OR(A82="",B82=""),P82=""),"",IFERROR(P82/(IF(N(H82)&gt;0,H82,IF(N(G82)&gt;0,G82,IF(COUNTIFS($B$12:$B$211,B82,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B82,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B82,$A$5:$A$7,0)))))),""))</f>
+        <f aca="false">IF(OR(OR(A82="",B82=""),P82=""),"",IFERROR(P82/(IF(N(G82)&gt;0,G82,IF(N(H82)&gt;0,H82,IF(COUNTIFS($B$12:$B$211,B82,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B82,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B82,$A$5:$A$7,0)))))),""))</f>
         <v/>
       </c>
       <c r="R82" s="23" t="str">
@@ -4431,7 +4567,7 @@
         <v/>
       </c>
       <c r="Q83" s="22" t="str">
-        <f aca="false">IF(OR(OR(A83="",B83=""),P83=""),"",IFERROR(P83/(IF(N(H83)&gt;0,H83,IF(N(G83)&gt;0,G83,IF(COUNTIFS($B$12:$B$211,B83,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B83,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B83,$A$5:$A$7,0)))))),""))</f>
+        <f aca="false">IF(OR(OR(A83="",B83=""),P83=""),"",IFERROR(P83/(IF(N(G83)&gt;0,G83,IF(N(H83)&gt;0,H83,IF(COUNTIFS($B$12:$B$211,B83,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B83,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B83,$A$5:$A$7,0)))))),""))</f>
         <v/>
       </c>
       <c r="R83" s="23" t="str">
@@ -4467,7 +4603,7 @@
         <v/>
       </c>
       <c r="Q84" s="22" t="str">
-        <f aca="false">IF(OR(OR(A84="",B84=""),P84=""),"",IFERROR(P84/(IF(N(H84)&gt;0,H84,IF(N(G84)&gt;0,G84,IF(COUNTIFS($B$12:$B$211,B84,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B84,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B84,$A$5:$A$7,0)))))),""))</f>
+        <f aca="false">IF(OR(OR(A84="",B84=""),P84=""),"",IFERROR(P84/(IF(N(G84)&gt;0,G84,IF(N(H84)&gt;0,H84,IF(COUNTIFS($B$12:$B$211,B84,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B84,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B84,$A$5:$A$7,0)))))),""))</f>
         <v/>
       </c>
       <c r="R84" s="23" t="str">
@@ -4503,7 +4639,7 @@
         <v/>
       </c>
       <c r="Q85" s="22" t="str">
-        <f aca="false">IF(OR(OR(A85="",B85=""),P85=""),"",IFERROR(P85/(IF(N(H85)&gt;0,H85,IF(N(G85)&gt;0,G85,IF(COUNTIFS($B$12:$B$211,B85,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B85,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B85,$A$5:$A$7,0)))))),""))</f>
+        <f aca="false">IF(OR(OR(A85="",B85=""),P85=""),"",IFERROR(P85/(IF(N(G85)&gt;0,G85,IF(N(H85)&gt;0,H85,IF(COUNTIFS($B$12:$B$211,B85,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B85,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B85,$A$5:$A$7,0)))))),""))</f>
         <v/>
       </c>
       <c r="R85" s="23" t="str">
@@ -4539,7 +4675,7 @@
         <v/>
       </c>
       <c r="Q86" s="22" t="str">
-        <f aca="false">IF(OR(OR(A86="",B86=""),P86=""),"",IFERROR(P86/(IF(N(H86)&gt;0,H86,IF(N(G86)&gt;0,G86,IF(COUNTIFS($B$12:$B$211,B86,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B86,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B86,$A$5:$A$7,0)))))),""))</f>
+        <f aca="false">IF(OR(OR(A86="",B86=""),P86=""),"",IFERROR(P86/(IF(N(G86)&gt;0,G86,IF(N(H86)&gt;0,H86,IF(COUNTIFS($B$12:$B$211,B86,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B86,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B86,$A$5:$A$7,0)))))),""))</f>
         <v/>
       </c>
       <c r="R86" s="23" t="str">
@@ -4575,7 +4711,7 @@
         <v/>
       </c>
       <c r="Q87" s="22" t="str">
-        <f aca="false">IF(OR(OR(A87="",B87=""),P87=""),"",IFERROR(P87/(IF(N(H87)&gt;0,H87,IF(N(G87)&gt;0,G87,IF(COUNTIFS($B$12:$B$211,B87,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B87,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B87,$A$5:$A$7,0)))))),""))</f>
+        <f aca="false">IF(OR(OR(A87="",B87=""),P87=""),"",IFERROR(P87/(IF(N(G87)&gt;0,G87,IF(N(H87)&gt;0,H87,IF(COUNTIFS($B$12:$B$211,B87,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B87,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B87,$A$5:$A$7,0)))))),""))</f>
         <v/>
       </c>
       <c r="R87" s="23" t="str">
@@ -4611,7 +4747,7 @@
         <v/>
       </c>
       <c r="Q88" s="22" t="str">
-        <f aca="false">IF(OR(OR(A88="",B88=""),P88=""),"",IFERROR(P88/(IF(N(H88)&gt;0,H88,IF(N(G88)&gt;0,G88,IF(COUNTIFS($B$12:$B$211,B88,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B88,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B88,$A$5:$A$7,0)))))),""))</f>
+        <f aca="false">IF(OR(OR(A88="",B88=""),P88=""),"",IFERROR(P88/(IF(N(G88)&gt;0,G88,IF(N(H88)&gt;0,H88,IF(COUNTIFS($B$12:$B$211,B88,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B88,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B88,$A$5:$A$7,0)))))),""))</f>
         <v/>
       </c>
       <c r="R88" s="23" t="str">
@@ -4647,7 +4783,7 @@
         <v/>
       </c>
       <c r="Q89" s="22" t="str">
-        <f aca="false">IF(OR(OR(A89="",B89=""),P89=""),"",IFERROR(P89/(IF(N(H89)&gt;0,H89,IF(N(G89)&gt;0,G89,IF(COUNTIFS($B$12:$B$211,B89,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B89,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B89,$A$5:$A$7,0)))))),""))</f>
+        <f aca="false">IF(OR(OR(A89="",B89=""),P89=""),"",IFERROR(P89/(IF(N(G89)&gt;0,G89,IF(N(H89)&gt;0,H89,IF(COUNTIFS($B$12:$B$211,B89,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B89,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B89,$A$5:$A$7,0)))))),""))</f>
         <v/>
       </c>
       <c r="R89" s="23" t="str">
@@ -4683,7 +4819,7 @@
         <v/>
       </c>
       <c r="Q90" s="22" t="str">
-        <f aca="false">IF(OR(OR(A90="",B90=""),P90=""),"",IFERROR(P90/(IF(N(H90)&gt;0,H90,IF(N(G90)&gt;0,G90,IF(COUNTIFS($B$12:$B$211,B90,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B90,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B90,$A$5:$A$7,0)))))),""))</f>
+        <f aca="false">IF(OR(OR(A90="",B90=""),P90=""),"",IFERROR(P90/(IF(N(G90)&gt;0,G90,IF(N(H90)&gt;0,H90,IF(COUNTIFS($B$12:$B$211,B90,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B90,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B90,$A$5:$A$7,0)))))),""))</f>
         <v/>
       </c>
       <c r="R90" s="23" t="str">
@@ -4719,7 +4855,7 @@
         <v/>
       </c>
       <c r="Q91" s="22" t="str">
-        <f aca="false">IF(OR(OR(A91="",B91=""),P91=""),"",IFERROR(P91/(IF(N(H91)&gt;0,H91,IF(N(G91)&gt;0,G91,IF(COUNTIFS($B$12:$B$211,B91,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B91,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B91,$A$5:$A$7,0)))))),""))</f>
+        <f aca="false">IF(OR(OR(A91="",B91=""),P91=""),"",IFERROR(P91/(IF(N(G91)&gt;0,G91,IF(N(H91)&gt;0,H91,IF(COUNTIFS($B$12:$B$211,B91,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B91,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B91,$A$5:$A$7,0)))))),""))</f>
         <v/>
       </c>
       <c r="R91" s="23" t="str">
@@ -4755,7 +4891,7 @@
         <v/>
       </c>
       <c r="Q92" s="22" t="str">
-        <f aca="false">IF(OR(OR(A92="",B92=""),P92=""),"",IFERROR(P92/(IF(N(H92)&gt;0,H92,IF(N(G92)&gt;0,G92,IF(COUNTIFS($B$12:$B$211,B92,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B92,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B92,$A$5:$A$7,0)))))),""))</f>
+        <f aca="false">IF(OR(OR(A92="",B92=""),P92=""),"",IFERROR(P92/(IF(N(G92)&gt;0,G92,IF(N(H92)&gt;0,H92,IF(COUNTIFS($B$12:$B$211,B92,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B92,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B92,$A$5:$A$7,0)))))),""))</f>
         <v/>
       </c>
       <c r="R92" s="23" t="str">
@@ -4791,7 +4927,7 @@
         <v/>
       </c>
       <c r="Q93" s="22" t="str">
-        <f aca="false">IF(OR(OR(A93="",B93=""),P93=""),"",IFERROR(P93/(IF(N(H93)&gt;0,H93,IF(N(G93)&gt;0,G93,IF(COUNTIFS($B$12:$B$211,B93,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B93,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B93,$A$5:$A$7,0)))))),""))</f>
+        <f aca="false">IF(OR(OR(A93="",B93=""),P93=""),"",IFERROR(P93/(IF(N(G93)&gt;0,G93,IF(N(H93)&gt;0,H93,IF(COUNTIFS($B$12:$B$211,B93,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B93,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B93,$A$5:$A$7,0)))))),""))</f>
         <v/>
       </c>
       <c r="R93" s="23" t="str">
@@ -4827,7 +4963,7 @@
         <v/>
       </c>
       <c r="Q94" s="22" t="str">
-        <f aca="false">IF(OR(OR(A94="",B94=""),P94=""),"",IFERROR(P94/(IF(N(H94)&gt;0,H94,IF(N(G94)&gt;0,G94,IF(COUNTIFS($B$12:$B$211,B94,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B94,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B94,$A$5:$A$7,0)))))),""))</f>
+        <f aca="false">IF(OR(OR(A94="",B94=""),P94=""),"",IFERROR(P94/(IF(N(G94)&gt;0,G94,IF(N(H94)&gt;0,H94,IF(COUNTIFS($B$12:$B$211,B94,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B94,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B94,$A$5:$A$7,0)))))),""))</f>
         <v/>
       </c>
       <c r="R94" s="23" t="str">
@@ -4863,7 +4999,7 @@
         <v/>
       </c>
       <c r="Q95" s="22" t="str">
-        <f aca="false">IF(OR(OR(A95="",B95=""),P95=""),"",IFERROR(P95/(IF(N(H95)&gt;0,H95,IF(N(G95)&gt;0,G95,IF(COUNTIFS($B$12:$B$211,B95,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B95,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B95,$A$5:$A$7,0)))))),""))</f>
+        <f aca="false">IF(OR(OR(A95="",B95=""),P95=""),"",IFERROR(P95/(IF(N(G95)&gt;0,G95,IF(N(H95)&gt;0,H95,IF(COUNTIFS($B$12:$B$211,B95,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B95,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B95,$A$5:$A$7,0)))))),""))</f>
         <v/>
       </c>
       <c r="R95" s="23" t="str">
@@ -4899,7 +5035,7 @@
         <v/>
       </c>
       <c r="Q96" s="22" t="str">
-        <f aca="false">IF(OR(OR(A96="",B96=""),P96=""),"",IFERROR(P96/(IF(N(H96)&gt;0,H96,IF(N(G96)&gt;0,G96,IF(COUNTIFS($B$12:$B$211,B96,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B96,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B96,$A$5:$A$7,0)))))),""))</f>
+        <f aca="false">IF(OR(OR(A96="",B96=""),P96=""),"",IFERROR(P96/(IF(N(G96)&gt;0,G96,IF(N(H96)&gt;0,H96,IF(COUNTIFS($B$12:$B$211,B96,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B96,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B96,$A$5:$A$7,0)))))),""))</f>
         <v/>
       </c>
       <c r="R96" s="23" t="str">
@@ -4935,7 +5071,7 @@
         <v/>
       </c>
       <c r="Q97" s="22" t="str">
-        <f aca="false">IF(OR(OR(A97="",B97=""),P97=""),"",IFERROR(P97/(IF(N(H97)&gt;0,H97,IF(N(G97)&gt;0,G97,IF(COUNTIFS($B$12:$B$211,B97,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B97,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B97,$A$5:$A$7,0)))))),""))</f>
+        <f aca="false">IF(OR(OR(A97="",B97=""),P97=""),"",IFERROR(P97/(IF(N(G97)&gt;0,G97,IF(N(H97)&gt;0,H97,IF(COUNTIFS($B$12:$B$211,B97,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B97,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B97,$A$5:$A$7,0)))))),""))</f>
         <v/>
       </c>
       <c r="R97" s="23" t="str">
@@ -4971,7 +5107,7 @@
         <v/>
       </c>
       <c r="Q98" s="22" t="str">
-        <f aca="false">IF(OR(OR(A98="",B98=""),P98=""),"",IFERROR(P98/(IF(N(H98)&gt;0,H98,IF(N(G98)&gt;0,G98,IF(COUNTIFS($B$12:$B$211,B98,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B98,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B98,$A$5:$A$7,0)))))),""))</f>
+        <f aca="false">IF(OR(OR(A98="",B98=""),P98=""),"",IFERROR(P98/(IF(N(G98)&gt;0,G98,IF(N(H98)&gt;0,H98,IF(COUNTIFS($B$12:$B$211,B98,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B98,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B98,$A$5:$A$7,0)))))),""))</f>
         <v/>
       </c>
       <c r="R98" s="23" t="str">
@@ -5007,7 +5143,7 @@
         <v/>
       </c>
       <c r="Q99" s="22" t="str">
-        <f aca="false">IF(OR(OR(A99="",B99=""),P99=""),"",IFERROR(P99/(IF(N(H99)&gt;0,H99,IF(N(G99)&gt;0,G99,IF(COUNTIFS($B$12:$B$211,B99,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B99,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B99,$A$5:$A$7,0)))))),""))</f>
+        <f aca="false">IF(OR(OR(A99="",B99=""),P99=""),"",IFERROR(P99/(IF(N(G99)&gt;0,G99,IF(N(H99)&gt;0,H99,IF(COUNTIFS($B$12:$B$211,B99,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B99,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B99,$A$5:$A$7,0)))))),""))</f>
         <v/>
       </c>
       <c r="R99" s="23" t="str">
@@ -5043,7 +5179,7 @@
         <v/>
       </c>
       <c r="Q100" s="22" t="str">
-        <f aca="false">IF(OR(OR(A100="",B100=""),P100=""),"",IFERROR(P100/(IF(N(H100)&gt;0,H100,IF(N(G100)&gt;0,G100,IF(COUNTIFS($B$12:$B$211,B100,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B100,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B100,$A$5:$A$7,0)))))),""))</f>
+        <f aca="false">IF(OR(OR(A100="",B100=""),P100=""),"",IFERROR(P100/(IF(N(G100)&gt;0,G100,IF(N(H100)&gt;0,H100,IF(COUNTIFS($B$12:$B$211,B100,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B100,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B100,$A$5:$A$7,0)))))),""))</f>
         <v/>
       </c>
       <c r="R100" s="23" t="str">
@@ -5079,7 +5215,7 @@
         <v/>
       </c>
       <c r="Q101" s="22" t="str">
-        <f aca="false">IF(OR(OR(A101="",B101=""),P101=""),"",IFERROR(P101/(IF(N(H101)&gt;0,H101,IF(N(G101)&gt;0,G101,IF(COUNTIFS($B$12:$B$211,B101,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B101,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B101,$A$5:$A$7,0)))))),""))</f>
+        <f aca="false">IF(OR(OR(A101="",B101=""),P101=""),"",IFERROR(P101/(IF(N(G101)&gt;0,G101,IF(N(H101)&gt;0,H101,IF(COUNTIFS($B$12:$B$211,B101,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B101,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B101,$A$5:$A$7,0)))))),""))</f>
         <v/>
       </c>
       <c r="R101" s="23" t="str">
@@ -5115,7 +5251,7 @@
         <v/>
       </c>
       <c r="Q102" s="22" t="str">
-        <f aca="false">IF(OR(OR(A102="",B102=""),P102=""),"",IFERROR(P102/(IF(N(H102)&gt;0,H102,IF(N(G102)&gt;0,G102,IF(COUNTIFS($B$12:$B$211,B102,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B102,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B102,$A$5:$A$7,0)))))),""))</f>
+        <f aca="false">IF(OR(OR(A102="",B102=""),P102=""),"",IFERROR(P102/(IF(N(G102)&gt;0,G102,IF(N(H102)&gt;0,H102,IF(COUNTIFS($B$12:$B$211,B102,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B102,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B102,$A$5:$A$7,0)))))),""))</f>
         <v/>
       </c>
       <c r="R102" s="23" t="str">
@@ -5151,7 +5287,7 @@
         <v/>
       </c>
       <c r="Q103" s="22" t="str">
-        <f aca="false">IF(OR(OR(A103="",B103=""),P103=""),"",IFERROR(P103/(IF(N(H103)&gt;0,H103,IF(N(G103)&gt;0,G103,IF(COUNTIFS($B$12:$B$211,B103,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B103,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B103,$A$5:$A$7,0)))))),""))</f>
+        <f aca="false">IF(OR(OR(A103="",B103=""),P103=""),"",IFERROR(P103/(IF(N(G103)&gt;0,G103,IF(N(H103)&gt;0,H103,IF(COUNTIFS($B$12:$B$211,B103,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B103,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B103,$A$5:$A$7,0)))))),""))</f>
         <v/>
       </c>
       <c r="R103" s="23" t="str">
@@ -5187,7 +5323,7 @@
         <v/>
       </c>
       <c r="Q104" s="22" t="str">
-        <f aca="false">IF(OR(OR(A104="",B104=""),P104=""),"",IFERROR(P104/(IF(N(H104)&gt;0,H104,IF(N(G104)&gt;0,G104,IF(COUNTIFS($B$12:$B$211,B104,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B104,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B104,$A$5:$A$7,0)))))),""))</f>
+        <f aca="false">IF(OR(OR(A104="",B104=""),P104=""),"",IFERROR(P104/(IF(N(G104)&gt;0,G104,IF(N(H104)&gt;0,H104,IF(COUNTIFS($B$12:$B$211,B104,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B104,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B104,$A$5:$A$7,0)))))),""))</f>
         <v/>
       </c>
       <c r="R104" s="23" t="str">
@@ -5223,7 +5359,7 @@
         <v/>
       </c>
       <c r="Q105" s="22" t="str">
-        <f aca="false">IF(OR(OR(A105="",B105=""),P105=""),"",IFERROR(P105/(IF(N(H105)&gt;0,H105,IF(N(G105)&gt;0,G105,IF(COUNTIFS($B$12:$B$211,B105,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B105,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B105,$A$5:$A$7,0)))))),""))</f>
+        <f aca="false">IF(OR(OR(A105="",B105=""),P105=""),"",IFERROR(P105/(IF(N(G105)&gt;0,G105,IF(N(H105)&gt;0,H105,IF(COUNTIFS($B$12:$B$211,B105,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B105,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B105,$A$5:$A$7,0)))))),""))</f>
         <v/>
       </c>
       <c r="R105" s="23" t="str">
@@ -5259,7 +5395,7 @@
         <v/>
       </c>
       <c r="Q106" s="22" t="str">
-        <f aca="false">IF(OR(OR(A106="",B106=""),P106=""),"",IFERROR(P106/(IF(N(H106)&gt;0,H106,IF(N(G106)&gt;0,G106,IF(COUNTIFS($B$12:$B$211,B106,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B106,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B106,$A$5:$A$7,0)))))),""))</f>
+        <f aca="false">IF(OR(OR(A106="",B106=""),P106=""),"",IFERROR(P106/(IF(N(G106)&gt;0,G106,IF(N(H106)&gt;0,H106,IF(COUNTIFS($B$12:$B$211,B106,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B106,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B106,$A$5:$A$7,0)))))),""))</f>
         <v/>
       </c>
       <c r="R106" s="23" t="str">
@@ -5295,7 +5431,7 @@
         <v/>
       </c>
       <c r="Q107" s="22" t="str">
-        <f aca="false">IF(OR(OR(A107="",B107=""),P107=""),"",IFERROR(P107/(IF(N(H107)&gt;0,H107,IF(N(G107)&gt;0,G107,IF(COUNTIFS($B$12:$B$211,B107,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B107,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B107,$A$5:$A$7,0)))))),""))</f>
+        <f aca="false">IF(OR(OR(A107="",B107=""),P107=""),"",IFERROR(P107/(IF(N(G107)&gt;0,G107,IF(N(H107)&gt;0,H107,IF(COUNTIFS($B$12:$B$211,B107,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B107,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B107,$A$5:$A$7,0)))))),""))</f>
         <v/>
       </c>
       <c r="R107" s="23" t="str">
@@ -5331,7 +5467,7 @@
         <v/>
       </c>
       <c r="Q108" s="22" t="str">
-        <f aca="false">IF(OR(OR(A108="",B108=""),P108=""),"",IFERROR(P108/(IF(N(H108)&gt;0,H108,IF(N(G108)&gt;0,G108,IF(COUNTIFS($B$12:$B$211,B108,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B108,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B108,$A$5:$A$7,0)))))),""))</f>
+        <f aca="false">IF(OR(OR(A108="",B108=""),P108=""),"",IFERROR(P108/(IF(N(G108)&gt;0,G108,IF(N(H108)&gt;0,H108,IF(COUNTIFS($B$12:$B$211,B108,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B108,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B108,$A$5:$A$7,0)))))),""))</f>
         <v/>
       </c>
       <c r="R108" s="23" t="str">
@@ -5367,7 +5503,7 @@
         <v/>
       </c>
       <c r="Q109" s="22" t="str">
-        <f aca="false">IF(OR(OR(A109="",B109=""),P109=""),"",IFERROR(P109/(IF(N(H109)&gt;0,H109,IF(N(G109)&gt;0,G109,IF(COUNTIFS($B$12:$B$211,B109,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B109,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B109,$A$5:$A$7,0)))))),""))</f>
+        <f aca="false">IF(OR(OR(A109="",B109=""),P109=""),"",IFERROR(P109/(IF(N(G109)&gt;0,G109,IF(N(H109)&gt;0,H109,IF(COUNTIFS($B$12:$B$211,B109,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B109,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B109,$A$5:$A$7,0)))))),""))</f>
         <v/>
       </c>
       <c r="R109" s="23" t="str">
@@ -5403,7 +5539,7 @@
         <v/>
       </c>
       <c r="Q110" s="22" t="str">
-        <f aca="false">IF(OR(OR(A110="",B110=""),P110=""),"",IFERROR(P110/(IF(N(H110)&gt;0,H110,IF(N(G110)&gt;0,G110,IF(COUNTIFS($B$12:$B$211,B110,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B110,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B110,$A$5:$A$7,0)))))),""))</f>
+        <f aca="false">IF(OR(OR(A110="",B110=""),P110=""),"",IFERROR(P110/(IF(N(G110)&gt;0,G110,IF(N(H110)&gt;0,H110,IF(COUNTIFS($B$12:$B$211,B110,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B110,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B110,$A$5:$A$7,0)))))),""))</f>
         <v/>
       </c>
       <c r="R110" s="23" t="str">
@@ -5439,7 +5575,7 @@
         <v/>
       </c>
       <c r="Q111" s="22" t="str">
-        <f aca="false">IF(OR(OR(A111="",B111=""),P111=""),"",IFERROR(P111/(IF(N(H111)&gt;0,H111,IF(N(G111)&gt;0,G111,IF(COUNTIFS($B$12:$B$211,B111,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B111,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B111,$A$5:$A$7,0)))))),""))</f>
+        <f aca="false">IF(OR(OR(A111="",B111=""),P111=""),"",IFERROR(P111/(IF(N(G111)&gt;0,G111,IF(N(H111)&gt;0,H111,IF(COUNTIFS($B$12:$B$211,B111,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B111,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B111,$A$5:$A$7,0)))))),""))</f>
         <v/>
       </c>
       <c r="R111" s="23" t="str">
@@ -5475,7 +5611,7 @@
         <v/>
       </c>
       <c r="Q112" s="22" t="str">
-        <f aca="false">IF(OR(OR(A112="",B112=""),P112=""),"",IFERROR(P112/(IF(N(H112)&gt;0,H112,IF(N(G112)&gt;0,G112,IF(COUNTIFS($B$12:$B$211,B112,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B112,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B112,$A$5:$A$7,0)))))),""))</f>
+        <f aca="false">IF(OR(OR(A112="",B112=""),P112=""),"",IFERROR(P112/(IF(N(G112)&gt;0,G112,IF(N(H112)&gt;0,H112,IF(COUNTIFS($B$12:$B$211,B112,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B112,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B112,$A$5:$A$7,0)))))),""))</f>
         <v/>
       </c>
       <c r="R112" s="23" t="str">
@@ -5511,7 +5647,7 @@
         <v/>
       </c>
       <c r="Q113" s="22" t="str">
-        <f aca="false">IF(OR(OR(A113="",B113=""),P113=""),"",IFERROR(P113/(IF(N(H113)&gt;0,H113,IF(N(G113)&gt;0,G113,IF(COUNTIFS($B$12:$B$211,B113,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B113,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B113,$A$5:$A$7,0)))))),""))</f>
+        <f aca="false">IF(OR(OR(A113="",B113=""),P113=""),"",IFERROR(P113/(IF(N(G113)&gt;0,G113,IF(N(H113)&gt;0,H113,IF(COUNTIFS($B$12:$B$211,B113,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B113,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B113,$A$5:$A$7,0)))))),""))</f>
         <v/>
       </c>
       <c r="R113" s="23" t="str">
@@ -5547,7 +5683,7 @@
         <v/>
       </c>
       <c r="Q114" s="22" t="str">
-        <f aca="false">IF(OR(OR(A114="",B114=""),P114=""),"",IFERROR(P114/(IF(N(H114)&gt;0,H114,IF(N(G114)&gt;0,G114,IF(COUNTIFS($B$12:$B$211,B114,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B114,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B114,$A$5:$A$7,0)))))),""))</f>
+        <f aca="false">IF(OR(OR(A114="",B114=""),P114=""),"",IFERROR(P114/(IF(N(G114)&gt;0,G114,IF(N(H114)&gt;0,H114,IF(COUNTIFS($B$12:$B$211,B114,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B114,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B114,$A$5:$A$7,0)))))),""))</f>
         <v/>
       </c>
       <c r="R114" s="23" t="str">
@@ -5583,7 +5719,7 @@
         <v/>
       </c>
       <c r="Q115" s="22" t="str">
-        <f aca="false">IF(OR(OR(A115="",B115=""),P115=""),"",IFERROR(P115/(IF(N(H115)&gt;0,H115,IF(N(G115)&gt;0,G115,IF(COUNTIFS($B$12:$B$211,B115,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B115,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B115,$A$5:$A$7,0)))))),""))</f>
+        <f aca="false">IF(OR(OR(A115="",B115=""),P115=""),"",IFERROR(P115/(IF(N(G115)&gt;0,G115,IF(N(H115)&gt;0,H115,IF(COUNTIFS($B$12:$B$211,B115,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B115,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B115,$A$5:$A$7,0)))))),""))</f>
         <v/>
       </c>
       <c r="R115" s="23" t="str">
@@ -5619,7 +5755,7 @@
         <v/>
       </c>
       <c r="Q116" s="22" t="str">
-        <f aca="false">IF(OR(OR(A116="",B116=""),P116=""),"",IFERROR(P116/(IF(N(H116)&gt;0,H116,IF(N(G116)&gt;0,G116,IF(COUNTIFS($B$12:$B$211,B116,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B116,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B116,$A$5:$A$7,0)))))),""))</f>
+        <f aca="false">IF(OR(OR(A116="",B116=""),P116=""),"",IFERROR(P116/(IF(N(G116)&gt;0,G116,IF(N(H116)&gt;0,H116,IF(COUNTIFS($B$12:$B$211,B116,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B116,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B116,$A$5:$A$7,0)))))),""))</f>
         <v/>
       </c>
       <c r="R116" s="23" t="str">
@@ -5655,7 +5791,7 @@
         <v/>
       </c>
       <c r="Q117" s="22" t="str">
-        <f aca="false">IF(OR(OR(A117="",B117=""),P117=""),"",IFERROR(P117/(IF(N(H117)&gt;0,H117,IF(N(G117)&gt;0,G117,IF(COUNTIFS($B$12:$B$211,B117,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B117,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B117,$A$5:$A$7,0)))))),""))</f>
+        <f aca="false">IF(OR(OR(A117="",B117=""),P117=""),"",IFERROR(P117/(IF(N(G117)&gt;0,G117,IF(N(H117)&gt;0,H117,IF(COUNTIFS($B$12:$B$211,B117,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B117,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B117,$A$5:$A$7,0)))))),""))</f>
         <v/>
       </c>
       <c r="R117" s="23" t="str">
@@ -5691,7 +5827,7 @@
         <v/>
       </c>
       <c r="Q118" s="22" t="str">
-        <f aca="false">IF(OR(OR(A118="",B118=""),P118=""),"",IFERROR(P118/(IF(N(H118)&gt;0,H118,IF(N(G118)&gt;0,G118,IF(COUNTIFS($B$12:$B$211,B118,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B118,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B118,$A$5:$A$7,0)))))),""))</f>
+        <f aca="false">IF(OR(OR(A118="",B118=""),P118=""),"",IFERROR(P118/(IF(N(G118)&gt;0,G118,IF(N(H118)&gt;0,H118,IF(COUNTIFS($B$12:$B$211,B118,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B118,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B118,$A$5:$A$7,0)))))),""))</f>
         <v/>
       </c>
       <c r="R118" s="23" t="str">
@@ -5727,7 +5863,7 @@
         <v/>
       </c>
       <c r="Q119" s="22" t="str">
-        <f aca="false">IF(OR(OR(A119="",B119=""),P119=""),"",IFERROR(P119/(IF(N(H119)&gt;0,H119,IF(N(G119)&gt;0,G119,IF(COUNTIFS($B$12:$B$211,B119,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B119,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B119,$A$5:$A$7,0)))))),""))</f>
+        <f aca="false">IF(OR(OR(A119="",B119=""),P119=""),"",IFERROR(P119/(IF(N(G119)&gt;0,G119,IF(N(H119)&gt;0,H119,IF(COUNTIFS($B$12:$B$211,B119,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B119,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B119,$A$5:$A$7,0)))))),""))</f>
         <v/>
       </c>
       <c r="R119" s="23" t="str">
@@ -5763,7 +5899,7 @@
         <v/>
       </c>
       <c r="Q120" s="22" t="str">
-        <f aca="false">IF(OR(OR(A120="",B120=""),P120=""),"",IFERROR(P120/(IF(N(H120)&gt;0,H120,IF(N(G120)&gt;0,G120,IF(COUNTIFS($B$12:$B$211,B120,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B120,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B120,$A$5:$A$7,0)))))),""))</f>
+        <f aca="false">IF(OR(OR(A120="",B120=""),P120=""),"",IFERROR(P120/(IF(N(G120)&gt;0,G120,IF(N(H120)&gt;0,H120,IF(COUNTIFS($B$12:$B$211,B120,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B120,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B120,$A$5:$A$7,0)))))),""))</f>
         <v/>
       </c>
       <c r="R120" s="23" t="str">
@@ -5799,7 +5935,7 @@
         <v/>
       </c>
       <c r="Q121" s="22" t="str">
-        <f aca="false">IF(OR(OR(A121="",B121=""),P121=""),"",IFERROR(P121/(IF(N(H121)&gt;0,H121,IF(N(G121)&gt;0,G121,IF(COUNTIFS($B$12:$B$211,B121,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B121,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B121,$A$5:$A$7,0)))))),""))</f>
+        <f aca="false">IF(OR(OR(A121="",B121=""),P121=""),"",IFERROR(P121/(IF(N(G121)&gt;0,G121,IF(N(H121)&gt;0,H121,IF(COUNTIFS($B$12:$B$211,B121,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B121,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B121,$A$5:$A$7,0)))))),""))</f>
         <v/>
       </c>
       <c r="R121" s="23" t="str">
@@ -5835,7 +5971,7 @@
         <v/>
       </c>
       <c r="Q122" s="22" t="str">
-        <f aca="false">IF(OR(OR(A122="",B122=""),P122=""),"",IFERROR(P122/(IF(N(H122)&gt;0,H122,IF(N(G122)&gt;0,G122,IF(COUNTIFS($B$12:$B$211,B122,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B122,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B122,$A$5:$A$7,0)))))),""))</f>
+        <f aca="false">IF(OR(OR(A122="",B122=""),P122=""),"",IFERROR(P122/(IF(N(G122)&gt;0,G122,IF(N(H122)&gt;0,H122,IF(COUNTIFS($B$12:$B$211,B122,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B122,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B122,$A$5:$A$7,0)))))),""))</f>
         <v/>
       </c>
       <c r="R122" s="23" t="str">
@@ -5871,7 +6007,7 @@
         <v/>
       </c>
       <c r="Q123" s="22" t="str">
-        <f aca="false">IF(OR(OR(A123="",B123=""),P123=""),"",IFERROR(P123/(IF(N(H123)&gt;0,H123,IF(N(G123)&gt;0,G123,IF(COUNTIFS($B$12:$B$211,B123,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B123,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B123,$A$5:$A$7,0)))))),""))</f>
+        <f aca="false">IF(OR(OR(A123="",B123=""),P123=""),"",IFERROR(P123/(IF(N(G123)&gt;0,G123,IF(N(H123)&gt;0,H123,IF(COUNTIFS($B$12:$B$211,B123,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B123,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B123,$A$5:$A$7,0)))))),""))</f>
         <v/>
       </c>
       <c r="R123" s="23" t="str">
@@ -5907,7 +6043,7 @@
         <v/>
       </c>
       <c r="Q124" s="22" t="str">
-        <f aca="false">IF(OR(OR(A124="",B124=""),P124=""),"",IFERROR(P124/(IF(N(H124)&gt;0,H124,IF(N(G124)&gt;0,G124,IF(COUNTIFS($B$12:$B$211,B124,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B124,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B124,$A$5:$A$7,0)))))),""))</f>
+        <f aca="false">IF(OR(OR(A124="",B124=""),P124=""),"",IFERROR(P124/(IF(N(G124)&gt;0,G124,IF(N(H124)&gt;0,H124,IF(COUNTIFS($B$12:$B$211,B124,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B124,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B124,$A$5:$A$7,0)))))),""))</f>
         <v/>
       </c>
       <c r="R124" s="23" t="str">
@@ -5943,7 +6079,7 @@
         <v/>
       </c>
       <c r="Q125" s="22" t="str">
-        <f aca="false">IF(OR(OR(A125="",B125=""),P125=""),"",IFERROR(P125/(IF(N(H125)&gt;0,H125,IF(N(G125)&gt;0,G125,IF(COUNTIFS($B$12:$B$211,B125,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B125,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B125,$A$5:$A$7,0)))))),""))</f>
+        <f aca="false">IF(OR(OR(A125="",B125=""),P125=""),"",IFERROR(P125/(IF(N(G125)&gt;0,G125,IF(N(H125)&gt;0,H125,IF(COUNTIFS($B$12:$B$211,B125,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B125,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B125,$A$5:$A$7,0)))))),""))</f>
         <v/>
       </c>
       <c r="R125" s="23" t="str">
@@ -5979,7 +6115,7 @@
         <v/>
       </c>
       <c r="Q126" s="22" t="str">
-        <f aca="false">IF(OR(OR(A126="",B126=""),P126=""),"",IFERROR(P126/(IF(N(H126)&gt;0,H126,IF(N(G126)&gt;0,G126,IF(COUNTIFS($B$12:$B$211,B126,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B126,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B126,$A$5:$A$7,0)))))),""))</f>
+        <f aca="false">IF(OR(OR(A126="",B126=""),P126=""),"",IFERROR(P126/(IF(N(G126)&gt;0,G126,IF(N(H126)&gt;0,H126,IF(COUNTIFS($B$12:$B$211,B126,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B126,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B126,$A$5:$A$7,0)))))),""))</f>
         <v/>
       </c>
       <c r="R126" s="23" t="str">
@@ -6015,7 +6151,7 @@
         <v/>
       </c>
       <c r="Q127" s="22" t="str">
-        <f aca="false">IF(OR(OR(A127="",B127=""),P127=""),"",IFERROR(P127/(IF(N(H127)&gt;0,H127,IF(N(G127)&gt;0,G127,IF(COUNTIFS($B$12:$B$211,B127,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B127,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B127,$A$5:$A$7,0)))))),""))</f>
+        <f aca="false">IF(OR(OR(A127="",B127=""),P127=""),"",IFERROR(P127/(IF(N(G127)&gt;0,G127,IF(N(H127)&gt;0,H127,IF(COUNTIFS($B$12:$B$211,B127,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B127,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B127,$A$5:$A$7,0)))))),""))</f>
         <v/>
       </c>
       <c r="R127" s="23" t="str">
@@ -6051,7 +6187,7 @@
         <v/>
       </c>
       <c r="Q128" s="22" t="str">
-        <f aca="false">IF(OR(OR(A128="",B128=""),P128=""),"",IFERROR(P128/(IF(N(H128)&gt;0,H128,IF(N(G128)&gt;0,G128,IF(COUNTIFS($B$12:$B$211,B128,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B128,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B128,$A$5:$A$7,0)))))),""))</f>
+        <f aca="false">IF(OR(OR(A128="",B128=""),P128=""),"",IFERROR(P128/(IF(N(G128)&gt;0,G128,IF(N(H128)&gt;0,H128,IF(COUNTIFS($B$12:$B$211,B128,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B128,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B128,$A$5:$A$7,0)))))),""))</f>
         <v/>
       </c>
       <c r="R128" s="23" t="str">
@@ -6087,7 +6223,7 @@
         <v/>
       </c>
       <c r="Q129" s="22" t="str">
-        <f aca="false">IF(OR(OR(A129="",B129=""),P129=""),"",IFERROR(P129/(IF(N(H129)&gt;0,H129,IF(N(G129)&gt;0,G129,IF(COUNTIFS($B$12:$B$211,B129,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B129,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B129,$A$5:$A$7,0)))))),""))</f>
+        <f aca="false">IF(OR(OR(A129="",B129=""),P129=""),"",IFERROR(P129/(IF(N(G129)&gt;0,G129,IF(N(H129)&gt;0,H129,IF(COUNTIFS($B$12:$B$211,B129,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B129,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B129,$A$5:$A$7,0)))))),""))</f>
         <v/>
       </c>
       <c r="R129" s="23" t="str">
@@ -6123,7 +6259,7 @@
         <v/>
       </c>
       <c r="Q130" s="22" t="str">
-        <f aca="false">IF(OR(OR(A130="",B130=""),P130=""),"",IFERROR(P130/(IF(N(H130)&gt;0,H130,IF(N(G130)&gt;0,G130,IF(COUNTIFS($B$12:$B$211,B130,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B130,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B130,$A$5:$A$7,0)))))),""))</f>
+        <f aca="false">IF(OR(OR(A130="",B130=""),P130=""),"",IFERROR(P130/(IF(N(G130)&gt;0,G130,IF(N(H130)&gt;0,H130,IF(COUNTIFS($B$12:$B$211,B130,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B130,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B130,$A$5:$A$7,0)))))),""))</f>
         <v/>
       </c>
       <c r="R130" s="23" t="str">
@@ -6159,7 +6295,7 @@
         <v/>
       </c>
       <c r="Q131" s="22" t="str">
-        <f aca="false">IF(OR(OR(A131="",B131=""),P131=""),"",IFERROR(P131/(IF(N(H131)&gt;0,H131,IF(N(G131)&gt;0,G131,IF(COUNTIFS($B$12:$B$211,B131,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B131,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B131,$A$5:$A$7,0)))))),""))</f>
+        <f aca="false">IF(OR(OR(A131="",B131=""),P131=""),"",IFERROR(P131/(IF(N(G131)&gt;0,G131,IF(N(H131)&gt;0,H131,IF(COUNTIFS($B$12:$B$211,B131,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B131,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B131,$A$5:$A$7,0)))))),""))</f>
         <v/>
       </c>
       <c r="R131" s="23" t="str">
@@ -6195,7 +6331,7 @@
         <v/>
       </c>
       <c r="Q132" s="22" t="str">
-        <f aca="false">IF(OR(OR(A132="",B132=""),P132=""),"",IFERROR(P132/(IF(N(H132)&gt;0,H132,IF(N(G132)&gt;0,G132,IF(COUNTIFS($B$12:$B$211,B132,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B132,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B132,$A$5:$A$7,0)))))),""))</f>
+        <f aca="false">IF(OR(OR(A132="",B132=""),P132=""),"",IFERROR(P132/(IF(N(G132)&gt;0,G132,IF(N(H132)&gt;0,H132,IF(COUNTIFS($B$12:$B$211,B132,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B132,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B132,$A$5:$A$7,0)))))),""))</f>
         <v/>
       </c>
       <c r="R132" s="23" t="str">
@@ -6231,7 +6367,7 @@
         <v/>
       </c>
       <c r="Q133" s="22" t="str">
-        <f aca="false">IF(OR(OR(A133="",B133=""),P133=""),"",IFERROR(P133/(IF(N(H133)&gt;0,H133,IF(N(G133)&gt;0,G133,IF(COUNTIFS($B$12:$B$211,B133,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B133,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B133,$A$5:$A$7,0)))))),""))</f>
+        <f aca="false">IF(OR(OR(A133="",B133=""),P133=""),"",IFERROR(P133/(IF(N(G133)&gt;0,G133,IF(N(H133)&gt;0,H133,IF(COUNTIFS($B$12:$B$211,B133,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B133,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B133,$A$5:$A$7,0)))))),""))</f>
         <v/>
       </c>
       <c r="R133" s="23" t="str">
@@ -6267,7 +6403,7 @@
         <v/>
       </c>
       <c r="Q134" s="22" t="str">
-        <f aca="false">IF(OR(OR(A134="",B134=""),P134=""),"",IFERROR(P134/(IF(N(H134)&gt;0,H134,IF(N(G134)&gt;0,G134,IF(COUNTIFS($B$12:$B$211,B134,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B134,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B134,$A$5:$A$7,0)))))),""))</f>
+        <f aca="false">IF(OR(OR(A134="",B134=""),P134=""),"",IFERROR(P134/(IF(N(G134)&gt;0,G134,IF(N(H134)&gt;0,H134,IF(COUNTIFS($B$12:$B$211,B134,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B134,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B134,$A$5:$A$7,0)))))),""))</f>
         <v/>
       </c>
       <c r="R134" s="23" t="str">
@@ -6303,7 +6439,7 @@
         <v/>
       </c>
       <c r="Q135" s="22" t="str">
-        <f aca="false">IF(OR(OR(A135="",B135=""),P135=""),"",IFERROR(P135/(IF(N(H135)&gt;0,H135,IF(N(G135)&gt;0,G135,IF(COUNTIFS($B$12:$B$211,B135,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B135,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B135,$A$5:$A$7,0)))))),""))</f>
+        <f aca="false">IF(OR(OR(A135="",B135=""),P135=""),"",IFERROR(P135/(IF(N(G135)&gt;0,G135,IF(N(H135)&gt;0,H135,IF(COUNTIFS($B$12:$B$211,B135,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B135,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B135,$A$5:$A$7,0)))))),""))</f>
         <v/>
       </c>
       <c r="R135" s="23" t="str">
@@ -6339,7 +6475,7 @@
         <v/>
       </c>
       <c r="Q136" s="22" t="str">
-        <f aca="false">IF(OR(OR(A136="",B136=""),P136=""),"",IFERROR(P136/(IF(N(H136)&gt;0,H136,IF(N(G136)&gt;0,G136,IF(COUNTIFS($B$12:$B$211,B136,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B136,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B136,$A$5:$A$7,0)))))),""))</f>
+        <f aca="false">IF(OR(OR(A136="",B136=""),P136=""),"",IFERROR(P136/(IF(N(G136)&gt;0,G136,IF(N(H136)&gt;0,H136,IF(COUNTIFS($B$12:$B$211,B136,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B136,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B136,$A$5:$A$7,0)))))),""))</f>
         <v/>
       </c>
       <c r="R136" s="23" t="str">
@@ -6375,7 +6511,7 @@
         <v/>
       </c>
       <c r="Q137" s="22" t="str">
-        <f aca="false">IF(OR(OR(A137="",B137=""),P137=""),"",IFERROR(P137/(IF(N(H137)&gt;0,H137,IF(N(G137)&gt;0,G137,IF(COUNTIFS($B$12:$B$211,B137,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B137,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B137,$A$5:$A$7,0)))))),""))</f>
+        <f aca="false">IF(OR(OR(A137="",B137=""),P137=""),"",IFERROR(P137/(IF(N(G137)&gt;0,G137,IF(N(H137)&gt;0,H137,IF(COUNTIFS($B$12:$B$211,B137,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B137,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B137,$A$5:$A$7,0)))))),""))</f>
         <v/>
       </c>
       <c r="R137" s="23" t="str">
@@ -6411,7 +6547,7 @@
         <v/>
       </c>
       <c r="Q138" s="22" t="str">
-        <f aca="false">IF(OR(OR(A138="",B138=""),P138=""),"",IFERROR(P138/(IF(N(H138)&gt;0,H138,IF(N(G138)&gt;0,G138,IF(COUNTIFS($B$12:$B$211,B138,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B138,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B138,$A$5:$A$7,0)))))),""))</f>
+        <f aca="false">IF(OR(OR(A138="",B138=""),P138=""),"",IFERROR(P138/(IF(N(G138)&gt;0,G138,IF(N(H138)&gt;0,H138,IF(COUNTIFS($B$12:$B$211,B138,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B138,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B138,$A$5:$A$7,0)))))),""))</f>
         <v/>
       </c>
       <c r="R138" s="23" t="str">
@@ -6447,7 +6583,7 @@
         <v/>
       </c>
       <c r="Q139" s="22" t="str">
-        <f aca="false">IF(OR(OR(A139="",B139=""),P139=""),"",IFERROR(P139/(IF(N(H139)&gt;0,H139,IF(N(G139)&gt;0,G139,IF(COUNTIFS($B$12:$B$211,B139,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B139,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B139,$A$5:$A$7,0)))))),""))</f>
+        <f aca="false">IF(OR(OR(A139="",B139=""),P139=""),"",IFERROR(P139/(IF(N(G139)&gt;0,G139,IF(N(H139)&gt;0,H139,IF(COUNTIFS($B$12:$B$211,B139,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B139,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B139,$A$5:$A$7,0)))))),""))</f>
         <v/>
       </c>
       <c r="R139" s="23" t="str">
@@ -6483,7 +6619,7 @@
         <v/>
       </c>
       <c r="Q140" s="22" t="str">
-        <f aca="false">IF(OR(OR(A140="",B140=""),P140=""),"",IFERROR(P140/(IF(N(H140)&gt;0,H140,IF(N(G140)&gt;0,G140,IF(COUNTIFS($B$12:$B$211,B140,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B140,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B140,$A$5:$A$7,0)))))),""))</f>
+        <f aca="false">IF(OR(OR(A140="",B140=""),P140=""),"",IFERROR(P140/(IF(N(G140)&gt;0,G140,IF(N(H140)&gt;0,H140,IF(COUNTIFS($B$12:$B$211,B140,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B140,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B140,$A$5:$A$7,0)))))),""))</f>
         <v/>
       </c>
       <c r="R140" s="23" t="str">
@@ -6519,7 +6655,7 @@
         <v/>
       </c>
       <c r="Q141" s="22" t="str">
-        <f aca="false">IF(OR(OR(A141="",B141=""),P141=""),"",IFERROR(P141/(IF(N(H141)&gt;0,H141,IF(N(G141)&gt;0,G141,IF(COUNTIFS($B$12:$B$211,B141,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B141,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B141,$A$5:$A$7,0)))))),""))</f>
+        <f aca="false">IF(OR(OR(A141="",B141=""),P141=""),"",IFERROR(P141/(IF(N(G141)&gt;0,G141,IF(N(H141)&gt;0,H141,IF(COUNTIFS($B$12:$B$211,B141,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B141,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B141,$A$5:$A$7,0)))))),""))</f>
         <v/>
       </c>
       <c r="R141" s="23" t="str">
@@ -6555,7 +6691,7 @@
         <v/>
       </c>
       <c r="Q142" s="22" t="str">
-        <f aca="false">IF(OR(OR(A142="",B142=""),P142=""),"",IFERROR(P142/(IF(N(H142)&gt;0,H142,IF(N(G142)&gt;0,G142,IF(COUNTIFS($B$12:$B$211,B142,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B142,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B142,$A$5:$A$7,0)))))),""))</f>
+        <f aca="false">IF(OR(OR(A142="",B142=""),P142=""),"",IFERROR(P142/(IF(N(G142)&gt;0,G142,IF(N(H142)&gt;0,H142,IF(COUNTIFS($B$12:$B$211,B142,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B142,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B142,$A$5:$A$7,0)))))),""))</f>
         <v/>
       </c>
       <c r="R142" s="23" t="str">
@@ -6591,7 +6727,7 @@
         <v/>
       </c>
       <c r="Q143" s="22" t="str">
-        <f aca="false">IF(OR(OR(A143="",B143=""),P143=""),"",IFERROR(P143/(IF(N(H143)&gt;0,H143,IF(N(G143)&gt;0,G143,IF(COUNTIFS($B$12:$B$211,B143,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B143,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B143,$A$5:$A$7,0)))))),""))</f>
+        <f aca="false">IF(OR(OR(A143="",B143=""),P143=""),"",IFERROR(P143/(IF(N(G143)&gt;0,G143,IF(N(H143)&gt;0,H143,IF(COUNTIFS($B$12:$B$211,B143,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B143,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B143,$A$5:$A$7,0)))))),""))</f>
         <v/>
       </c>
       <c r="R143" s="23" t="str">
@@ -6627,7 +6763,7 @@
         <v/>
       </c>
       <c r="Q144" s="22" t="str">
-        <f aca="false">IF(OR(OR(A144="",B144=""),P144=""),"",IFERROR(P144/(IF(N(H144)&gt;0,H144,IF(N(G144)&gt;0,G144,IF(COUNTIFS($B$12:$B$211,B144,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B144,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B144,$A$5:$A$7,0)))))),""))</f>
+        <f aca="false">IF(OR(OR(A144="",B144=""),P144=""),"",IFERROR(P144/(IF(N(G144)&gt;0,G144,IF(N(H144)&gt;0,H144,IF(COUNTIFS($B$12:$B$211,B144,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B144,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B144,$A$5:$A$7,0)))))),""))</f>
         <v/>
       </c>
       <c r="R144" s="23" t="str">
@@ -6663,7 +6799,7 @@
         <v/>
       </c>
       <c r="Q145" s="22" t="str">
-        <f aca="false">IF(OR(OR(A145="",B145=""),P145=""),"",IFERROR(P145/(IF(N(H145)&gt;0,H145,IF(N(G145)&gt;0,G145,IF(COUNTIFS($B$12:$B$211,B145,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B145,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B145,$A$5:$A$7,0)))))),""))</f>
+        <f aca="false">IF(OR(OR(A145="",B145=""),P145=""),"",IFERROR(P145/(IF(N(G145)&gt;0,G145,IF(N(H145)&gt;0,H145,IF(COUNTIFS($B$12:$B$211,B145,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B145,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B145,$A$5:$A$7,0)))))),""))</f>
         <v/>
       </c>
       <c r="R145" s="23" t="str">
@@ -6699,7 +6835,7 @@
         <v/>
       </c>
       <c r="Q146" s="22" t="str">
-        <f aca="false">IF(OR(OR(A146="",B146=""),P146=""),"",IFERROR(P146/(IF(N(H146)&gt;0,H146,IF(N(G146)&gt;0,G146,IF(COUNTIFS($B$12:$B$211,B146,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B146,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B146,$A$5:$A$7,0)))))),""))</f>
+        <f aca="false">IF(OR(OR(A146="",B146=""),P146=""),"",IFERROR(P146/(IF(N(G146)&gt;0,G146,IF(N(H146)&gt;0,H146,IF(COUNTIFS($B$12:$B$211,B146,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B146,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B146,$A$5:$A$7,0)))))),""))</f>
         <v/>
       </c>
       <c r="R146" s="23" t="str">
@@ -6735,7 +6871,7 @@
         <v/>
       </c>
       <c r="Q147" s="22" t="str">
-        <f aca="false">IF(OR(OR(A147="",B147=""),P147=""),"",IFERROR(P147/(IF(N(H147)&gt;0,H147,IF(N(G147)&gt;0,G147,IF(COUNTIFS($B$12:$B$211,B147,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B147,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B147,$A$5:$A$7,0)))))),""))</f>
+        <f aca="false">IF(OR(OR(A147="",B147=""),P147=""),"",IFERROR(P147/(IF(N(G147)&gt;0,G147,IF(N(H147)&gt;0,H147,IF(COUNTIFS($B$12:$B$211,B147,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B147,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B147,$A$5:$A$7,0)))))),""))</f>
         <v/>
       </c>
       <c r="R147" s="23" t="str">
@@ -6771,7 +6907,7 @@
         <v/>
       </c>
       <c r="Q148" s="22" t="str">
-        <f aca="false">IF(OR(OR(A148="",B148=""),P148=""),"",IFERROR(P148/(IF(N(H148)&gt;0,H148,IF(N(G148)&gt;0,G148,IF(COUNTIFS($B$12:$B$211,B148,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B148,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B148,$A$5:$A$7,0)))))),""))</f>
+        <f aca="false">IF(OR(OR(A148="",B148=""),P148=""),"",IFERROR(P148/(IF(N(G148)&gt;0,G148,IF(N(H148)&gt;0,H148,IF(COUNTIFS($B$12:$B$211,B148,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B148,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B148,$A$5:$A$7,0)))))),""))</f>
         <v/>
       </c>
       <c r="R148" s="23" t="str">
@@ -6807,7 +6943,7 @@
         <v/>
       </c>
       <c r="Q149" s="22" t="str">
-        <f aca="false">IF(OR(OR(A149="",B149=""),P149=""),"",IFERROR(P149/(IF(N(H149)&gt;0,H149,IF(N(G149)&gt;0,G149,IF(COUNTIFS($B$12:$B$211,B149,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B149,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B149,$A$5:$A$7,0)))))),""))</f>
+        <f aca="false">IF(OR(OR(A149="",B149=""),P149=""),"",IFERROR(P149/(IF(N(G149)&gt;0,G149,IF(N(H149)&gt;0,H149,IF(COUNTIFS($B$12:$B$211,B149,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B149,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B149,$A$5:$A$7,0)))))),""))</f>
         <v/>
       </c>
       <c r="R149" s="23" t="str">
@@ -6843,7 +6979,7 @@
         <v/>
       </c>
       <c r="Q150" s="22" t="str">
-        <f aca="false">IF(OR(OR(A150="",B150=""),P150=""),"",IFERROR(P150/(IF(N(H150)&gt;0,H150,IF(N(G150)&gt;0,G150,IF(COUNTIFS($B$12:$B$211,B150,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B150,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B150,$A$5:$A$7,0)))))),""))</f>
+        <f aca="false">IF(OR(OR(A150="",B150=""),P150=""),"",IFERROR(P150/(IF(N(G150)&gt;0,G150,IF(N(H150)&gt;0,H150,IF(COUNTIFS($B$12:$B$211,B150,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B150,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B150,$A$5:$A$7,0)))))),""))</f>
         <v/>
       </c>
       <c r="R150" s="23" t="str">
@@ -6879,7 +7015,7 @@
         <v/>
       </c>
       <c r="Q151" s="22" t="str">
-        <f aca="false">IF(OR(OR(A151="",B151=""),P151=""),"",IFERROR(P151/(IF(N(H151)&gt;0,H151,IF(N(G151)&gt;0,G151,IF(COUNTIFS($B$12:$B$211,B151,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B151,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B151,$A$5:$A$7,0)))))),""))</f>
+        <f aca="false">IF(OR(OR(A151="",B151=""),P151=""),"",IFERROR(P151/(IF(N(G151)&gt;0,G151,IF(N(H151)&gt;0,H151,IF(COUNTIFS($B$12:$B$211,B151,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B151,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B151,$A$5:$A$7,0)))))),""))</f>
         <v/>
       </c>
       <c r="R151" s="23" t="str">
@@ -6915,7 +7051,7 @@
         <v/>
       </c>
       <c r="Q152" s="22" t="str">
-        <f aca="false">IF(OR(OR(A152="",B152=""),P152=""),"",IFERROR(P152/(IF(N(H152)&gt;0,H152,IF(N(G152)&gt;0,G152,IF(COUNTIFS($B$12:$B$211,B152,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B152,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B152,$A$5:$A$7,0)))))),""))</f>
+        <f aca="false">IF(OR(OR(A152="",B152=""),P152=""),"",IFERROR(P152/(IF(N(G152)&gt;0,G152,IF(N(H152)&gt;0,H152,IF(COUNTIFS($B$12:$B$211,B152,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B152,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B152,$A$5:$A$7,0)))))),""))</f>
         <v/>
       </c>
       <c r="R152" s="23" t="str">
@@ -6951,7 +7087,7 @@
         <v/>
       </c>
       <c r="Q153" s="22" t="str">
-        <f aca="false">IF(OR(OR(A153="",B153=""),P153=""),"",IFERROR(P153/(IF(N(H153)&gt;0,H153,IF(N(G153)&gt;0,G153,IF(COUNTIFS($B$12:$B$211,B153,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B153,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B153,$A$5:$A$7,0)))))),""))</f>
+        <f aca="false">IF(OR(OR(A153="",B153=""),P153=""),"",IFERROR(P153/(IF(N(G153)&gt;0,G153,IF(N(H153)&gt;0,H153,IF(COUNTIFS($B$12:$B$211,B153,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B153,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B153,$A$5:$A$7,0)))))),""))</f>
         <v/>
       </c>
       <c r="R153" s="23" t="str">
@@ -6987,7 +7123,7 @@
         <v/>
       </c>
       <c r="Q154" s="22" t="str">
-        <f aca="false">IF(OR(OR(A154="",B154=""),P154=""),"",IFERROR(P154/(IF(N(H154)&gt;0,H154,IF(N(G154)&gt;0,G154,IF(COUNTIFS($B$12:$B$211,B154,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B154,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B154,$A$5:$A$7,0)))))),""))</f>
+        <f aca="false">IF(OR(OR(A154="",B154=""),P154=""),"",IFERROR(P154/(IF(N(G154)&gt;0,G154,IF(N(H154)&gt;0,H154,IF(COUNTIFS($B$12:$B$211,B154,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B154,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B154,$A$5:$A$7,0)))))),""))</f>
         <v/>
       </c>
       <c r="R154" s="23" t="str">
@@ -7023,7 +7159,7 @@
         <v/>
       </c>
       <c r="Q155" s="22" t="str">
-        <f aca="false">IF(OR(OR(A155="",B155=""),P155=""),"",IFERROR(P155/(IF(N(H155)&gt;0,H155,IF(N(G155)&gt;0,G155,IF(COUNTIFS($B$12:$B$211,B155,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B155,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B155,$A$5:$A$7,0)))))),""))</f>
+        <f aca="false">IF(OR(OR(A155="",B155=""),P155=""),"",IFERROR(P155/(IF(N(G155)&gt;0,G155,IF(N(H155)&gt;0,H155,IF(COUNTIFS($B$12:$B$211,B155,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B155,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B155,$A$5:$A$7,0)))))),""))</f>
         <v/>
       </c>
       <c r="R155" s="23" t="str">
@@ -7059,7 +7195,7 @@
         <v/>
       </c>
       <c r="Q156" s="22" t="str">
-        <f aca="false">IF(OR(OR(A156="",B156=""),P156=""),"",IFERROR(P156/(IF(N(H156)&gt;0,H156,IF(N(G156)&gt;0,G156,IF(COUNTIFS($B$12:$B$211,B156,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B156,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B156,$A$5:$A$7,0)))))),""))</f>
+        <f aca="false">IF(OR(OR(A156="",B156=""),P156=""),"",IFERROR(P156/(IF(N(G156)&gt;0,G156,IF(N(H156)&gt;0,H156,IF(COUNTIFS($B$12:$B$211,B156,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B156,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B156,$A$5:$A$7,0)))))),""))</f>
         <v/>
       </c>
       <c r="R156" s="23" t="str">
@@ -7095,7 +7231,7 @@
         <v/>
       </c>
       <c r="Q157" s="22" t="str">
-        <f aca="false">IF(OR(OR(A157="",B157=""),P157=""),"",IFERROR(P157/(IF(N(H157)&gt;0,H157,IF(N(G157)&gt;0,G157,IF(COUNTIFS($B$12:$B$211,B157,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B157,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B157,$A$5:$A$7,0)))))),""))</f>
+        <f aca="false">IF(OR(OR(A157="",B157=""),P157=""),"",IFERROR(P157/(IF(N(G157)&gt;0,G157,IF(N(H157)&gt;0,H157,IF(COUNTIFS($B$12:$B$211,B157,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B157,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B157,$A$5:$A$7,0)))))),""))</f>
         <v/>
       </c>
       <c r="R157" s="23" t="str">
@@ -7131,7 +7267,7 @@
         <v/>
       </c>
       <c r="Q158" s="22" t="str">
-        <f aca="false">IF(OR(OR(A158="",B158=""),P158=""),"",IFERROR(P158/(IF(N(H158)&gt;0,H158,IF(N(G158)&gt;0,G158,IF(COUNTIFS($B$12:$B$211,B158,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B158,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B158,$A$5:$A$7,0)))))),""))</f>
+        <f aca="false">IF(OR(OR(A158="",B158=""),P158=""),"",IFERROR(P158/(IF(N(G158)&gt;0,G158,IF(N(H158)&gt;0,H158,IF(COUNTIFS($B$12:$B$211,B158,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B158,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B158,$A$5:$A$7,0)))))),""))</f>
         <v/>
       </c>
       <c r="R158" s="23" t="str">
@@ -7167,7 +7303,7 @@
         <v/>
       </c>
       <c r="Q159" s="22" t="str">
-        <f aca="false">IF(OR(OR(A159="",B159=""),P159=""),"",IFERROR(P159/(IF(N(H159)&gt;0,H159,IF(N(G159)&gt;0,G159,IF(COUNTIFS($B$12:$B$211,B159,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B159,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B159,$A$5:$A$7,0)))))),""))</f>
+        <f aca="false">IF(OR(OR(A159="",B159=""),P159=""),"",IFERROR(P159/(IF(N(G159)&gt;0,G159,IF(N(H159)&gt;0,H159,IF(COUNTIFS($B$12:$B$211,B159,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B159,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B159,$A$5:$A$7,0)))))),""))</f>
         <v/>
       </c>
       <c r="R159" s="23" t="str">
@@ -7203,7 +7339,7 @@
         <v/>
       </c>
       <c r="Q160" s="22" t="str">
-        <f aca="false">IF(OR(OR(A160="",B160=""),P160=""),"",IFERROR(P160/(IF(N(H160)&gt;0,H160,IF(N(G160)&gt;0,G160,IF(COUNTIFS($B$12:$B$211,B160,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B160,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B160,$A$5:$A$7,0)))))),""))</f>
+        <f aca="false">IF(OR(OR(A160="",B160=""),P160=""),"",IFERROR(P160/(IF(N(G160)&gt;0,G160,IF(N(H160)&gt;0,H160,IF(COUNTIFS($B$12:$B$211,B160,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B160,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B160,$A$5:$A$7,0)))))),""))</f>
         <v/>
       </c>
       <c r="R160" s="23" t="str">
@@ -7239,7 +7375,7 @@
         <v/>
       </c>
       <c r="Q161" s="22" t="str">
-        <f aca="false">IF(OR(OR(A161="",B161=""),P161=""),"",IFERROR(P161/(IF(N(H161)&gt;0,H161,IF(N(G161)&gt;0,G161,IF(COUNTIFS($B$12:$B$211,B161,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B161,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B161,$A$5:$A$7,0)))))),""))</f>
+        <f aca="false">IF(OR(OR(A161="",B161=""),P161=""),"",IFERROR(P161/(IF(N(G161)&gt;0,G161,IF(N(H161)&gt;0,H161,IF(COUNTIFS($B$12:$B$211,B161,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B161,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B161,$A$5:$A$7,0)))))),""))</f>
         <v/>
       </c>
       <c r="R161" s="23" t="str">
@@ -7275,7 +7411,7 @@
         <v/>
       </c>
       <c r="Q162" s="22" t="str">
-        <f aca="false">IF(OR(OR(A162="",B162=""),P162=""),"",IFERROR(P162/(IF(N(H162)&gt;0,H162,IF(N(G162)&gt;0,G162,IF(COUNTIFS($B$12:$B$211,B162,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B162,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B162,$A$5:$A$7,0)))))),""))</f>
+        <f aca="false">IF(OR(OR(A162="",B162=""),P162=""),"",IFERROR(P162/(IF(N(G162)&gt;0,G162,IF(N(H162)&gt;0,H162,IF(COUNTIFS($B$12:$B$211,B162,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B162,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B162,$A$5:$A$7,0)))))),""))</f>
         <v/>
       </c>
       <c r="R162" s="23" t="str">
@@ -7311,7 +7447,7 @@
         <v/>
       </c>
       <c r="Q163" s="22" t="str">
-        <f aca="false">IF(OR(OR(A163="",B163=""),P163=""),"",IFERROR(P163/(IF(N(H163)&gt;0,H163,IF(N(G163)&gt;0,G163,IF(COUNTIFS($B$12:$B$211,B163,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B163,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B163,$A$5:$A$7,0)))))),""))</f>
+        <f aca="false">IF(OR(OR(A163="",B163=""),P163=""),"",IFERROR(P163/(IF(N(G163)&gt;0,G163,IF(N(H163)&gt;0,H163,IF(COUNTIFS($B$12:$B$211,B163,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B163,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B163,$A$5:$A$7,0)))))),""))</f>
         <v/>
       </c>
       <c r="R163" s="23" t="str">
@@ -7347,7 +7483,7 @@
         <v/>
       </c>
       <c r="Q164" s="22" t="str">
-        <f aca="false">IF(OR(OR(A164="",B164=""),P164=""),"",IFERROR(P164/(IF(N(H164)&gt;0,H164,IF(N(G164)&gt;0,G164,IF(COUNTIFS($B$12:$B$211,B164,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B164,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B164,$A$5:$A$7,0)))))),""))</f>
+        <f aca="false">IF(OR(OR(A164="",B164=""),P164=""),"",IFERROR(P164/(IF(N(G164)&gt;0,G164,IF(N(H164)&gt;0,H164,IF(COUNTIFS($B$12:$B$211,B164,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B164,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B164,$A$5:$A$7,0)))))),""))</f>
         <v/>
       </c>
       <c r="R164" s="23" t="str">
@@ -7383,7 +7519,7 @@
         <v/>
       </c>
       <c r="Q165" s="22" t="str">
-        <f aca="false">IF(OR(OR(A165="",B165=""),P165=""),"",IFERROR(P165/(IF(N(H165)&gt;0,H165,IF(N(G165)&gt;0,G165,IF(COUNTIFS($B$12:$B$211,B165,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B165,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B165,$A$5:$A$7,0)))))),""))</f>
+        <f aca="false">IF(OR(OR(A165="",B165=""),P165=""),"",IFERROR(P165/(IF(N(G165)&gt;0,G165,IF(N(H165)&gt;0,H165,IF(COUNTIFS($B$12:$B$211,B165,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B165,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B165,$A$5:$A$7,0)))))),""))</f>
         <v/>
       </c>
       <c r="R165" s="23" t="str">
@@ -7419,7 +7555,7 @@
         <v/>
       </c>
       <c r="Q166" s="22" t="str">
-        <f aca="false">IF(OR(OR(A166="",B166=""),P166=""),"",IFERROR(P166/(IF(N(H166)&gt;0,H166,IF(N(G166)&gt;0,G166,IF(COUNTIFS($B$12:$B$211,B166,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B166,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B166,$A$5:$A$7,0)))))),""))</f>
+        <f aca="false">IF(OR(OR(A166="",B166=""),P166=""),"",IFERROR(P166/(IF(N(G166)&gt;0,G166,IF(N(H166)&gt;0,H166,IF(COUNTIFS($B$12:$B$211,B166,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B166,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B166,$A$5:$A$7,0)))))),""))</f>
         <v/>
       </c>
       <c r="R166" s="23" t="str">
@@ -7455,7 +7591,7 @@
         <v/>
       </c>
       <c r="Q167" s="22" t="str">
-        <f aca="false">IF(OR(OR(A167="",B167=""),P167=""),"",IFERROR(P167/(IF(N(H167)&gt;0,H167,IF(N(G167)&gt;0,G167,IF(COUNTIFS($B$12:$B$211,B167,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B167,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B167,$A$5:$A$7,0)))))),""))</f>
+        <f aca="false">IF(OR(OR(A167="",B167=""),P167=""),"",IFERROR(P167/(IF(N(G167)&gt;0,G167,IF(N(H167)&gt;0,H167,IF(COUNTIFS($B$12:$B$211,B167,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B167,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B167,$A$5:$A$7,0)))))),""))</f>
         <v/>
       </c>
       <c r="R167" s="23" t="str">
@@ -7491,7 +7627,7 @@
         <v/>
       </c>
       <c r="Q168" s="22" t="str">
-        <f aca="false">IF(OR(OR(A168="",B168=""),P168=""),"",IFERROR(P168/(IF(N(H168)&gt;0,H168,IF(N(G168)&gt;0,G168,IF(COUNTIFS($B$12:$B$211,B168,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B168,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B168,$A$5:$A$7,0)))))),""))</f>
+        <f aca="false">IF(OR(OR(A168="",B168=""),P168=""),"",IFERROR(P168/(IF(N(G168)&gt;0,G168,IF(N(H168)&gt;0,H168,IF(COUNTIFS($B$12:$B$211,B168,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B168,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B168,$A$5:$A$7,0)))))),""))</f>
         <v/>
       </c>
       <c r="R168" s="23" t="str">
@@ -7527,7 +7663,7 @@
         <v/>
       </c>
       <c r="Q169" s="22" t="str">
-        <f aca="false">IF(OR(OR(A169="",B169=""),P169=""),"",IFERROR(P169/(IF(N(H169)&gt;0,H169,IF(N(G169)&gt;0,G169,IF(COUNTIFS($B$12:$B$211,B169,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B169,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B169,$A$5:$A$7,0)))))),""))</f>
+        <f aca="false">IF(OR(OR(A169="",B169=""),P169=""),"",IFERROR(P169/(IF(N(G169)&gt;0,G169,IF(N(H169)&gt;0,H169,IF(COUNTIFS($B$12:$B$211,B169,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B169,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B169,$A$5:$A$7,0)))))),""))</f>
         <v/>
       </c>
       <c r="R169" s="23" t="str">
@@ -7563,7 +7699,7 @@
         <v/>
       </c>
       <c r="Q170" s="22" t="str">
-        <f aca="false">IF(OR(OR(A170="",B170=""),P170=""),"",IFERROR(P170/(IF(N(H170)&gt;0,H170,IF(N(G170)&gt;0,G170,IF(COUNTIFS($B$12:$B$211,B170,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B170,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B170,$A$5:$A$7,0)))))),""))</f>
+        <f aca="false">IF(OR(OR(A170="",B170=""),P170=""),"",IFERROR(P170/(IF(N(G170)&gt;0,G170,IF(N(H170)&gt;0,H170,IF(COUNTIFS($B$12:$B$211,B170,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B170,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B170,$A$5:$A$7,0)))))),""))</f>
         <v/>
       </c>
       <c r="R170" s="23" t="str">
@@ -7599,7 +7735,7 @@
         <v/>
       </c>
       <c r="Q171" s="22" t="str">
-        <f aca="false">IF(OR(OR(A171="",B171=""),P171=""),"",IFERROR(P171/(IF(N(H171)&gt;0,H171,IF(N(G171)&gt;0,G171,IF(COUNTIFS($B$12:$B$211,B171,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B171,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B171,$A$5:$A$7,0)))))),""))</f>
+        <f aca="false">IF(OR(OR(A171="",B171=""),P171=""),"",IFERROR(P171/(IF(N(G171)&gt;0,G171,IF(N(H171)&gt;0,H171,IF(COUNTIFS($B$12:$B$211,B171,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B171,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B171,$A$5:$A$7,0)))))),""))</f>
         <v/>
       </c>
       <c r="R171" s="23" t="str">
@@ -7635,7 +7771,7 @@
         <v/>
       </c>
       <c r="Q172" s="22" t="str">
-        <f aca="false">IF(OR(OR(A172="",B172=""),P172=""),"",IFERROR(P172/(IF(N(H172)&gt;0,H172,IF(N(G172)&gt;0,G172,IF(COUNTIFS($B$12:$B$211,B172,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B172,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B172,$A$5:$A$7,0)))))),""))</f>
+        <f aca="false">IF(OR(OR(A172="",B172=""),P172=""),"",IFERROR(P172/(IF(N(G172)&gt;0,G172,IF(N(H172)&gt;0,H172,IF(COUNTIFS($B$12:$B$211,B172,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B172,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B172,$A$5:$A$7,0)))))),""))</f>
         <v/>
       </c>
       <c r="R172" s="23" t="str">
@@ -7671,7 +7807,7 @@
         <v/>
       </c>
       <c r="Q173" s="22" t="str">
-        <f aca="false">IF(OR(OR(A173="",B173=""),P173=""),"",IFERROR(P173/(IF(N(H173)&gt;0,H173,IF(N(G173)&gt;0,G173,IF(COUNTIFS($B$12:$B$211,B173,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B173,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B173,$A$5:$A$7,0)))))),""))</f>
+        <f aca="false">IF(OR(OR(A173="",B173=""),P173=""),"",IFERROR(P173/(IF(N(G173)&gt;0,G173,IF(N(H173)&gt;0,H173,IF(COUNTIFS($B$12:$B$211,B173,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B173,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B173,$A$5:$A$7,0)))))),""))</f>
         <v/>
       </c>
       <c r="R173" s="23" t="str">
@@ -7707,7 +7843,7 @@
         <v/>
       </c>
       <c r="Q174" s="22" t="str">
-        <f aca="false">IF(OR(OR(A174="",B174=""),P174=""),"",IFERROR(P174/(IF(N(H174)&gt;0,H174,IF(N(G174)&gt;0,G174,IF(COUNTIFS($B$12:$B$211,B174,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B174,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B174,$A$5:$A$7,0)))))),""))</f>
+        <f aca="false">IF(OR(OR(A174="",B174=""),P174=""),"",IFERROR(P174/(IF(N(G174)&gt;0,G174,IF(N(H174)&gt;0,H174,IF(COUNTIFS($B$12:$B$211,B174,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B174,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B174,$A$5:$A$7,0)))))),""))</f>
         <v/>
       </c>
       <c r="R174" s="23" t="str">
@@ -7743,7 +7879,7 @@
         <v/>
       </c>
       <c r="Q175" s="22" t="str">
-        <f aca="false">IF(OR(OR(A175="",B175=""),P175=""),"",IFERROR(P175/(IF(N(H175)&gt;0,H175,IF(N(G175)&gt;0,G175,IF(COUNTIFS($B$12:$B$211,B175,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B175,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B175,$A$5:$A$7,0)))))),""))</f>
+        <f aca="false">IF(OR(OR(A175="",B175=""),P175=""),"",IFERROR(P175/(IF(N(G175)&gt;0,G175,IF(N(H175)&gt;0,H175,IF(COUNTIFS($B$12:$B$211,B175,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B175,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B175,$A$5:$A$7,0)))))),""))</f>
         <v/>
       </c>
       <c r="R175" s="23" t="str">
@@ -7779,7 +7915,7 @@
         <v/>
       </c>
       <c r="Q176" s="22" t="str">
-        <f aca="false">IF(OR(OR(A176="",B176=""),P176=""),"",IFERROR(P176/(IF(N(H176)&gt;0,H176,IF(N(G176)&gt;0,G176,IF(COUNTIFS($B$12:$B$211,B176,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B176,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B176,$A$5:$A$7,0)))))),""))</f>
+        <f aca="false">IF(OR(OR(A176="",B176=""),P176=""),"",IFERROR(P176/(IF(N(G176)&gt;0,G176,IF(N(H176)&gt;0,H176,IF(COUNTIFS($B$12:$B$211,B176,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B176,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B176,$A$5:$A$7,0)))))),""))</f>
         <v/>
       </c>
       <c r="R176" s="23" t="str">
@@ -7815,7 +7951,7 @@
         <v/>
       </c>
       <c r="Q177" s="22" t="str">
-        <f aca="false">IF(OR(OR(A177="",B177=""),P177=""),"",IFERROR(P177/(IF(N(H177)&gt;0,H177,IF(N(G177)&gt;0,G177,IF(COUNTIFS($B$12:$B$211,B177,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B177,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B177,$A$5:$A$7,0)))))),""))</f>
+        <f aca="false">IF(OR(OR(A177="",B177=""),P177=""),"",IFERROR(P177/(IF(N(G177)&gt;0,G177,IF(N(H177)&gt;0,H177,IF(COUNTIFS($B$12:$B$211,B177,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B177,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B177,$A$5:$A$7,0)))))),""))</f>
         <v/>
       </c>
       <c r="R177" s="23" t="str">
@@ -7851,7 +7987,7 @@
         <v/>
       </c>
       <c r="Q178" s="22" t="str">
-        <f aca="false">IF(OR(OR(A178="",B178=""),P178=""),"",IFERROR(P178/(IF(N(H178)&gt;0,H178,IF(N(G178)&gt;0,G178,IF(COUNTIFS($B$12:$B$211,B178,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B178,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B178,$A$5:$A$7,0)))))),""))</f>
+        <f aca="false">IF(OR(OR(A178="",B178=""),P178=""),"",IFERROR(P178/(IF(N(G178)&gt;0,G178,IF(N(H178)&gt;0,H178,IF(COUNTIFS($B$12:$B$211,B178,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B178,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B178,$A$5:$A$7,0)))))),""))</f>
         <v/>
       </c>
       <c r="R178" s="23" t="str">
@@ -7887,7 +8023,7 @@
         <v/>
       </c>
       <c r="Q179" s="22" t="str">
-        <f aca="false">IF(OR(OR(A179="",B179=""),P179=""),"",IFERROR(P179/(IF(N(H179)&gt;0,H179,IF(N(G179)&gt;0,G179,IF(COUNTIFS($B$12:$B$211,B179,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B179,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B179,$A$5:$A$7,0)))))),""))</f>
+        <f aca="false">IF(OR(OR(A179="",B179=""),P179=""),"",IFERROR(P179/(IF(N(G179)&gt;0,G179,IF(N(H179)&gt;0,H179,IF(COUNTIFS($B$12:$B$211,B179,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B179,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B179,$A$5:$A$7,0)))))),""))</f>
         <v/>
       </c>
       <c r="R179" s="23" t="str">
@@ -7923,7 +8059,7 @@
         <v/>
       </c>
       <c r="Q180" s="22" t="str">
-        <f aca="false">IF(OR(OR(A180="",B180=""),P180=""),"",IFERROR(P180/(IF(N(H180)&gt;0,H180,IF(N(G180)&gt;0,G180,IF(COUNTIFS($B$12:$B$211,B180,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B180,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B180,$A$5:$A$7,0)))))),""))</f>
+        <f aca="false">IF(OR(OR(A180="",B180=""),P180=""),"",IFERROR(P180/(IF(N(G180)&gt;0,G180,IF(N(H180)&gt;0,H180,IF(COUNTIFS($B$12:$B$211,B180,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B180,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B180,$A$5:$A$7,0)))))),""))</f>
         <v/>
       </c>
       <c r="R180" s="23" t="str">
@@ -7959,7 +8095,7 @@
         <v/>
       </c>
       <c r="Q181" s="22" t="str">
-        <f aca="false">IF(OR(OR(A181="",B181=""),P181=""),"",IFERROR(P181/(IF(N(H181)&gt;0,H181,IF(N(G181)&gt;0,G181,IF(COUNTIFS($B$12:$B$211,B181,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B181,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B181,$A$5:$A$7,0)))))),""))</f>
+        <f aca="false">IF(OR(OR(A181="",B181=""),P181=""),"",IFERROR(P181/(IF(N(G181)&gt;0,G181,IF(N(H181)&gt;0,H181,IF(COUNTIFS($B$12:$B$211,B181,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B181,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B181,$A$5:$A$7,0)))))),""))</f>
         <v/>
       </c>
       <c r="R181" s="23" t="str">
@@ -7995,7 +8131,7 @@
         <v/>
       </c>
       <c r="Q182" s="22" t="str">
-        <f aca="false">IF(OR(OR(A182="",B182=""),P182=""),"",IFERROR(P182/(IF(N(H182)&gt;0,H182,IF(N(G182)&gt;0,G182,IF(COUNTIFS($B$12:$B$211,B182,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B182,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B182,$A$5:$A$7,0)))))),""))</f>
+        <f aca="false">IF(OR(OR(A182="",B182=""),P182=""),"",IFERROR(P182/(IF(N(G182)&gt;0,G182,IF(N(H182)&gt;0,H182,IF(COUNTIFS($B$12:$B$211,B182,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B182,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B182,$A$5:$A$7,0)))))),""))</f>
         <v/>
       </c>
       <c r="R182" s="23" t="str">
@@ -8031,7 +8167,7 @@
         <v/>
       </c>
       <c r="Q183" s="22" t="str">
-        <f aca="false">IF(OR(OR(A183="",B183=""),P183=""),"",IFERROR(P183/(IF(N(H183)&gt;0,H183,IF(N(G183)&gt;0,G183,IF(COUNTIFS($B$12:$B$211,B183,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B183,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B183,$A$5:$A$7,0)))))),""))</f>
+        <f aca="false">IF(OR(OR(A183="",B183=""),P183=""),"",IFERROR(P183/(IF(N(G183)&gt;0,G183,IF(N(H183)&gt;0,H183,IF(COUNTIFS($B$12:$B$211,B183,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B183,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B183,$A$5:$A$7,0)))))),""))</f>
         <v/>
       </c>
       <c r="R183" s="23" t="str">
@@ -8067,7 +8203,7 @@
         <v/>
       </c>
       <c r="Q184" s="22" t="str">
-        <f aca="false">IF(OR(OR(A184="",B184=""),P184=""),"",IFERROR(P184/(IF(N(H184)&gt;0,H184,IF(N(G184)&gt;0,G184,IF(COUNTIFS($B$12:$B$211,B184,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B184,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B184,$A$5:$A$7,0)))))),""))</f>
+        <f aca="false">IF(OR(OR(A184="",B184=""),P184=""),"",IFERROR(P184/(IF(N(G184)&gt;0,G184,IF(N(H184)&gt;0,H184,IF(COUNTIFS($B$12:$B$211,B184,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B184,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B184,$A$5:$A$7,0)))))),""))</f>
         <v/>
       </c>
       <c r="R184" s="23" t="str">
@@ -8103,7 +8239,7 @@
         <v/>
       </c>
       <c r="Q185" s="22" t="str">
-        <f aca="false">IF(OR(OR(A185="",B185=""),P185=""),"",IFERROR(P185/(IF(N(H185)&gt;0,H185,IF(N(G185)&gt;0,G185,IF(COUNTIFS($B$12:$B$211,B185,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B185,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B185,$A$5:$A$7,0)))))),""))</f>
+        <f aca="false">IF(OR(OR(A185="",B185=""),P185=""),"",IFERROR(P185/(IF(N(G185)&gt;0,G185,IF(N(H185)&gt;0,H185,IF(COUNTIFS($B$12:$B$211,B185,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B185,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B185,$A$5:$A$7,0)))))),""))</f>
         <v/>
       </c>
       <c r="R185" s="23" t="str">
@@ -8139,7 +8275,7 @@
         <v/>
       </c>
       <c r="Q186" s="22" t="str">
-        <f aca="false">IF(OR(OR(A186="",B186=""),P186=""),"",IFERROR(P186/(IF(N(H186)&gt;0,H186,IF(N(G186)&gt;0,G186,IF(COUNTIFS($B$12:$B$211,B186,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B186,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B186,$A$5:$A$7,0)))))),""))</f>
+        <f aca="false">IF(OR(OR(A186="",B186=""),P186=""),"",IFERROR(P186/(IF(N(G186)&gt;0,G186,IF(N(H186)&gt;0,H186,IF(COUNTIFS($B$12:$B$211,B186,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B186,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B186,$A$5:$A$7,0)))))),""))</f>
         <v/>
       </c>
       <c r="R186" s="23" t="str">
@@ -8175,7 +8311,7 @@
         <v/>
       </c>
       <c r="Q187" s="22" t="str">
-        <f aca="false">IF(OR(OR(A187="",B187=""),P187=""),"",IFERROR(P187/(IF(N(H187)&gt;0,H187,IF(N(G187)&gt;0,G187,IF(COUNTIFS($B$12:$B$211,B187,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B187,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B187,$A$5:$A$7,0)))))),""))</f>
+        <f aca="false">IF(OR(OR(A187="",B187=""),P187=""),"",IFERROR(P187/(IF(N(G187)&gt;0,G187,IF(N(H187)&gt;0,H187,IF(COUNTIFS($B$12:$B$211,B187,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B187,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B187,$A$5:$A$7,0)))))),""))</f>
         <v/>
       </c>
       <c r="R187" s="23" t="str">
@@ -8211,7 +8347,7 @@
         <v/>
       </c>
       <c r="Q188" s="22" t="str">
-        <f aca="false">IF(OR(OR(A188="",B188=""),P188=""),"",IFERROR(P188/(IF(N(H188)&gt;0,H188,IF(N(G188)&gt;0,G188,IF(COUNTIFS($B$12:$B$211,B188,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B188,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B188,$A$5:$A$7,0)))))),""))</f>
+        <f aca="false">IF(OR(OR(A188="",B188=""),P188=""),"",IFERROR(P188/(IF(N(G188)&gt;0,G188,IF(N(H188)&gt;0,H188,IF(COUNTIFS($B$12:$B$211,B188,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B188,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B188,$A$5:$A$7,0)))))),""))</f>
         <v/>
       </c>
       <c r="R188" s="23" t="str">
@@ -8247,7 +8383,7 @@
         <v/>
       </c>
       <c r="Q189" s="22" t="str">
-        <f aca="false">IF(OR(OR(A189="",B189=""),P189=""),"",IFERROR(P189/(IF(N(H189)&gt;0,H189,IF(N(G189)&gt;0,G189,IF(COUNTIFS($B$12:$B$211,B189,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B189,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B189,$A$5:$A$7,0)))))),""))</f>
+        <f aca="false">IF(OR(OR(A189="",B189=""),P189=""),"",IFERROR(P189/(IF(N(G189)&gt;0,G189,IF(N(H189)&gt;0,H189,IF(COUNTIFS($B$12:$B$211,B189,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B189,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B189,$A$5:$A$7,0)))))),""))</f>
         <v/>
       </c>
       <c r="R189" s="23" t="str">
@@ -8283,7 +8419,7 @@
         <v/>
       </c>
       <c r="Q190" s="22" t="str">
-        <f aca="false">IF(OR(OR(A190="",B190=""),P190=""),"",IFERROR(P190/(IF(N(H190)&gt;0,H190,IF(N(G190)&gt;0,G190,IF(COUNTIFS($B$12:$B$211,B190,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B190,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B190,$A$5:$A$7,0)))))),""))</f>
+        <f aca="false">IF(OR(OR(A190="",B190=""),P190=""),"",IFERROR(P190/(IF(N(G190)&gt;0,G190,IF(N(H190)&gt;0,H190,IF(COUNTIFS($B$12:$B$211,B190,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B190,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B190,$A$5:$A$7,0)))))),""))</f>
         <v/>
       </c>
       <c r="R190" s="23" t="str">
@@ -8319,7 +8455,7 @@
         <v/>
       </c>
       <c r="Q191" s="22" t="str">
-        <f aca="false">IF(OR(OR(A191="",B191=""),P191=""),"",IFERROR(P191/(IF(N(H191)&gt;0,H191,IF(N(G191)&gt;0,G191,IF(COUNTIFS($B$12:$B$211,B191,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B191,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B191,$A$5:$A$7,0)))))),""))</f>
+        <f aca="false">IF(OR(OR(A191="",B191=""),P191=""),"",IFERROR(P191/(IF(N(G191)&gt;0,G191,IF(N(H191)&gt;0,H191,IF(COUNTIFS($B$12:$B$211,B191,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B191,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B191,$A$5:$A$7,0)))))),""))</f>
         <v/>
       </c>
       <c r="R191" s="23" t="str">
@@ -8355,7 +8491,7 @@
         <v/>
       </c>
       <c r="Q192" s="22" t="str">
-        <f aca="false">IF(OR(OR(A192="",B192=""),P192=""),"",IFERROR(P192/(IF(N(H192)&gt;0,H192,IF(N(G192)&gt;0,G192,IF(COUNTIFS($B$12:$B$211,B192,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B192,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B192,$A$5:$A$7,0)))))),""))</f>
+        <f aca="false">IF(OR(OR(A192="",B192=""),P192=""),"",IFERROR(P192/(IF(N(G192)&gt;0,G192,IF(N(H192)&gt;0,H192,IF(COUNTIFS($B$12:$B$211,B192,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B192,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B192,$A$5:$A$7,0)))))),""))</f>
         <v/>
       </c>
       <c r="R192" s="23" t="str">
@@ -8391,7 +8527,7 @@
         <v/>
       </c>
       <c r="Q193" s="22" t="str">
-        <f aca="false">IF(OR(OR(A193="",B193=""),P193=""),"",IFERROR(P193/(IF(N(H193)&gt;0,H193,IF(N(G193)&gt;0,G193,IF(COUNTIFS($B$12:$B$211,B193,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B193,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B193,$A$5:$A$7,0)))))),""))</f>
+        <f aca="false">IF(OR(OR(A193="",B193=""),P193=""),"",IFERROR(P193/(IF(N(G193)&gt;0,G193,IF(N(H193)&gt;0,H193,IF(COUNTIFS($B$12:$B$211,B193,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B193,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B193,$A$5:$A$7,0)))))),""))</f>
         <v/>
       </c>
       <c r="R193" s="23" t="str">
@@ -8427,7 +8563,7 @@
         <v/>
       </c>
       <c r="Q194" s="22" t="str">
-        <f aca="false">IF(OR(OR(A194="",B194=""),P194=""),"",IFERROR(P194/(IF(N(H194)&gt;0,H194,IF(N(G194)&gt;0,G194,IF(COUNTIFS($B$12:$B$211,B194,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B194,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B194,$A$5:$A$7,0)))))),""))</f>
+        <f aca="false">IF(OR(OR(A194="",B194=""),P194=""),"",IFERROR(P194/(IF(N(G194)&gt;0,G194,IF(N(H194)&gt;0,H194,IF(COUNTIFS($B$12:$B$211,B194,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B194,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B194,$A$5:$A$7,0)))))),""))</f>
         <v/>
       </c>
       <c r="R194" s="23" t="str">
@@ -8463,7 +8599,7 @@
         <v/>
       </c>
       <c r="Q195" s="22" t="str">
-        <f aca="false">IF(OR(OR(A195="",B195=""),P195=""),"",IFERROR(P195/(IF(N(H195)&gt;0,H195,IF(N(G195)&gt;0,G195,IF(COUNTIFS($B$12:$B$211,B195,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B195,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B195,$A$5:$A$7,0)))))),""))</f>
+        <f aca="false">IF(OR(OR(A195="",B195=""),P195=""),"",IFERROR(P195/(IF(N(G195)&gt;0,G195,IF(N(H195)&gt;0,H195,IF(COUNTIFS($B$12:$B$211,B195,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B195,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B195,$A$5:$A$7,0)))))),""))</f>
         <v/>
       </c>
       <c r="R195" s="23" t="str">
@@ -8499,7 +8635,7 @@
         <v/>
       </c>
       <c r="Q196" s="22" t="str">
-        <f aca="false">IF(OR(OR(A196="",B196=""),P196=""),"",IFERROR(P196/(IF(N(H196)&gt;0,H196,IF(N(G196)&gt;0,G196,IF(COUNTIFS($B$12:$B$211,B196,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B196,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B196,$A$5:$A$7,0)))))),""))</f>
+        <f aca="false">IF(OR(OR(A196="",B196=""),P196=""),"",IFERROR(P196/(IF(N(G196)&gt;0,G196,IF(N(H196)&gt;0,H196,IF(COUNTIFS($B$12:$B$211,B196,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B196,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B196,$A$5:$A$7,0)))))),""))</f>
         <v/>
       </c>
       <c r="R196" s="23" t="str">
@@ -8535,7 +8671,7 @@
         <v/>
       </c>
       <c r="Q197" s="22" t="str">
-        <f aca="false">IF(OR(OR(A197="",B197=""),P197=""),"",IFERROR(P197/(IF(N(H197)&gt;0,H197,IF(N(G197)&gt;0,G197,IF(COUNTIFS($B$12:$B$211,B197,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B197,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B197,$A$5:$A$7,0)))))),""))</f>
+        <f aca="false">IF(OR(OR(A197="",B197=""),P197=""),"",IFERROR(P197/(IF(N(G197)&gt;0,G197,IF(N(H197)&gt;0,H197,IF(COUNTIFS($B$12:$B$211,B197,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B197,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B197,$A$5:$A$7,0)))))),""))</f>
         <v/>
       </c>
       <c r="R197" s="23" t="str">
@@ -8571,7 +8707,7 @@
         <v/>
       </c>
       <c r="Q198" s="22" t="str">
-        <f aca="false">IF(OR(OR(A198="",B198=""),P198=""),"",IFERROR(P198/(IF(N(H198)&gt;0,H198,IF(N(G198)&gt;0,G198,IF(COUNTIFS($B$12:$B$211,B198,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B198,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B198,$A$5:$A$7,0)))))),""))</f>
+        <f aca="false">IF(OR(OR(A198="",B198=""),P198=""),"",IFERROR(P198/(IF(N(G198)&gt;0,G198,IF(N(H198)&gt;0,H198,IF(COUNTIFS($B$12:$B$211,B198,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B198,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B198,$A$5:$A$7,0)))))),""))</f>
         <v/>
       </c>
       <c r="R198" s="23" t="str">
@@ -8607,7 +8743,7 @@
         <v/>
       </c>
       <c r="Q199" s="22" t="str">
-        <f aca="false">IF(OR(OR(A199="",B199=""),P199=""),"",IFERROR(P199/(IF(N(H199)&gt;0,H199,IF(N(G199)&gt;0,G199,IF(COUNTIFS($B$12:$B$211,B199,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B199,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B199,$A$5:$A$7,0)))))),""))</f>
+        <f aca="false">IF(OR(OR(A199="",B199=""),P199=""),"",IFERROR(P199/(IF(N(G199)&gt;0,G199,IF(N(H199)&gt;0,H199,IF(COUNTIFS($B$12:$B$211,B199,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B199,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B199,$A$5:$A$7,0)))))),""))</f>
         <v/>
       </c>
       <c r="R199" s="23" t="str">
@@ -8643,7 +8779,7 @@
         <v/>
       </c>
       <c r="Q200" s="22" t="str">
-        <f aca="false">IF(OR(OR(A200="",B200=""),P200=""),"",IFERROR(P200/(IF(N(H200)&gt;0,H200,IF(N(G200)&gt;0,G200,IF(COUNTIFS($B$12:$B$211,B200,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B200,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B200,$A$5:$A$7,0)))))),""))</f>
+        <f aca="false">IF(OR(OR(A200="",B200=""),P200=""),"",IFERROR(P200/(IF(N(G200)&gt;0,G200,IF(N(H200)&gt;0,H200,IF(COUNTIFS($B$12:$B$211,B200,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B200,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B200,$A$5:$A$7,0)))))),""))</f>
         <v/>
       </c>
       <c r="R200" s="23" t="str">
@@ -8679,7 +8815,7 @@
         <v/>
       </c>
       <c r="Q201" s="22" t="str">
-        <f aca="false">IF(OR(OR(A201="",B201=""),P201=""),"",IFERROR(P201/(IF(N(H201)&gt;0,H201,IF(N(G201)&gt;0,G201,IF(COUNTIFS($B$12:$B$211,B201,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B201,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B201,$A$5:$A$7,0)))))),""))</f>
+        <f aca="false">IF(OR(OR(A201="",B201=""),P201=""),"",IFERROR(P201/(IF(N(G201)&gt;0,G201,IF(N(H201)&gt;0,H201,IF(COUNTIFS($B$12:$B$211,B201,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B201,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B201,$A$5:$A$7,0)))))),""))</f>
         <v/>
       </c>
       <c r="R201" s="23" t="str">
@@ -8715,7 +8851,7 @@
         <v/>
       </c>
       <c r="Q202" s="22" t="str">
-        <f aca="false">IF(OR(OR(A202="",B202=""),P202=""),"",IFERROR(P202/(IF(N(H202)&gt;0,H202,IF(N(G202)&gt;0,G202,IF(COUNTIFS($B$12:$B$211,B202,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B202,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B202,$A$5:$A$7,0)))))),""))</f>
+        <f aca="false">IF(OR(OR(A202="",B202=""),P202=""),"",IFERROR(P202/(IF(N(G202)&gt;0,G202,IF(N(H202)&gt;0,H202,IF(COUNTIFS($B$12:$B$211,B202,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B202,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B202,$A$5:$A$7,0)))))),""))</f>
         <v/>
       </c>
       <c r="R202" s="23" t="str">
@@ -8751,7 +8887,7 @@
         <v/>
       </c>
       <c r="Q203" s="22" t="str">
-        <f aca="false">IF(OR(OR(A203="",B203=""),P203=""),"",IFERROR(P203/(IF(N(H203)&gt;0,H203,IF(N(G203)&gt;0,G203,IF(COUNTIFS($B$12:$B$211,B203,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B203,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B203,$A$5:$A$7,0)))))),""))</f>
+        <f aca="false">IF(OR(OR(A203="",B203=""),P203=""),"",IFERROR(P203/(IF(N(G203)&gt;0,G203,IF(N(H203)&gt;0,H203,IF(COUNTIFS($B$12:$B$211,B203,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B203,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B203,$A$5:$A$7,0)))))),""))</f>
         <v/>
       </c>
       <c r="R203" s="23" t="str">
@@ -8787,7 +8923,7 @@
         <v/>
       </c>
       <c r="Q204" s="22" t="str">
-        <f aca="false">IF(OR(OR(A204="",B204=""),P204=""),"",IFERROR(P204/(IF(N(H204)&gt;0,H204,IF(N(G204)&gt;0,G204,IF(COUNTIFS($B$12:$B$211,B204,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B204,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B204,$A$5:$A$7,0)))))),""))</f>
+        <f aca="false">IF(OR(OR(A204="",B204=""),P204=""),"",IFERROR(P204/(IF(N(G204)&gt;0,G204,IF(N(H204)&gt;0,H204,IF(COUNTIFS($B$12:$B$211,B204,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B204,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B204,$A$5:$A$7,0)))))),""))</f>
         <v/>
       </c>
       <c r="R204" s="23" t="str">
@@ -8823,7 +8959,7 @@
         <v/>
       </c>
       <c r="Q205" s="22" t="str">
-        <f aca="false">IF(OR(OR(A205="",B205=""),P205=""),"",IFERROR(P205/(IF(N(H205)&gt;0,H205,IF(N(G205)&gt;0,G205,IF(COUNTIFS($B$12:$B$211,B205,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B205,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B205,$A$5:$A$7,0)))))),""))</f>
+        <f aca="false">IF(OR(OR(A205="",B205=""),P205=""),"",IFERROR(P205/(IF(N(G205)&gt;0,G205,IF(N(H205)&gt;0,H205,IF(COUNTIFS($B$12:$B$211,B205,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B205,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B205,$A$5:$A$7,0)))))),""))</f>
         <v/>
       </c>
       <c r="R205" s="23" t="str">
@@ -8859,7 +8995,7 @@
         <v/>
       </c>
       <c r="Q206" s="22" t="str">
-        <f aca="false">IF(OR(OR(A206="",B206=""),P206=""),"",IFERROR(P206/(IF(N(H206)&gt;0,H206,IF(N(G206)&gt;0,G206,IF(COUNTIFS($B$12:$B$211,B206,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B206,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B206,$A$5:$A$7,0)))))),""))</f>
+        <f aca="false">IF(OR(OR(A206="",B206=""),P206=""),"",IFERROR(P206/(IF(N(G206)&gt;0,G206,IF(N(H206)&gt;0,H206,IF(COUNTIFS($B$12:$B$211,B206,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B206,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B206,$A$5:$A$7,0)))))),""))</f>
         <v/>
       </c>
       <c r="R206" s="23" t="str">
@@ -8895,7 +9031,7 @@
         <v/>
       </c>
       <c r="Q207" s="22" t="str">
-        <f aca="false">IF(OR(OR(A207="",B207=""),P207=""),"",IFERROR(P207/(IF(N(H207)&gt;0,H207,IF(N(G207)&gt;0,G207,IF(COUNTIFS($B$12:$B$211,B207,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B207,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B207,$A$5:$A$7,0)))))),""))</f>
+        <f aca="false">IF(OR(OR(A207="",B207=""),P207=""),"",IFERROR(P207/(IF(N(G207)&gt;0,G207,IF(N(H207)&gt;0,H207,IF(COUNTIFS($B$12:$B$211,B207,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B207,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B207,$A$5:$A$7,0)))))),""))</f>
         <v/>
       </c>
       <c r="R207" s="23" t="str">
@@ -8931,7 +9067,7 @@
         <v/>
       </c>
       <c r="Q208" s="22" t="str">
-        <f aca="false">IF(OR(OR(A208="",B208=""),P208=""),"",IFERROR(P208/(IF(N(H208)&gt;0,H208,IF(N(G208)&gt;0,G208,IF(COUNTIFS($B$12:$B$211,B208,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B208,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B208,$A$5:$A$7,0)))))),""))</f>
+        <f aca="false">IF(OR(OR(A208="",B208=""),P208=""),"",IFERROR(P208/(IF(N(G208)&gt;0,G208,IF(N(H208)&gt;0,H208,IF(COUNTIFS($B$12:$B$211,B208,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B208,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B208,$A$5:$A$7,0)))))),""))</f>
         <v/>
       </c>
       <c r="R208" s="23" t="str">
@@ -8967,7 +9103,7 @@
         <v/>
       </c>
       <c r="Q209" s="22" t="str">
-        <f aca="false">IF(OR(OR(A209="",B209=""),P209=""),"",IFERROR(P209/(IF(N(H209)&gt;0,H209,IF(N(G209)&gt;0,G209,IF(COUNTIFS($B$12:$B$211,B209,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B209,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B209,$A$5:$A$7,0)))))),""))</f>
+        <f aca="false">IF(OR(OR(A209="",B209=""),P209=""),"",IFERROR(P209/(IF(N(G209)&gt;0,G209,IF(N(H209)&gt;0,H209,IF(COUNTIFS($B$12:$B$211,B209,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B209,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B209,$A$5:$A$7,0)))))),""))</f>
         <v/>
       </c>
       <c r="R209" s="23" t="str">
@@ -9003,7 +9139,7 @@
         <v/>
       </c>
       <c r="Q210" s="22" t="str">
-        <f aca="false">IF(OR(OR(A210="",B210=""),P210=""),"",IFERROR(P210/(IF(N(H210)&gt;0,H210,IF(N(G210)&gt;0,G210,IF(COUNTIFS($B$12:$B$211,B210,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B210,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B210,$A$5:$A$7,0)))))),""))</f>
+        <f aca="false">IF(OR(OR(A210="",B210=""),P210=""),"",IFERROR(P210/(IF(N(G210)&gt;0,G210,IF(N(H210)&gt;0,H210,IF(COUNTIFS($B$12:$B$211,B210,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B210,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B210,$A$5:$A$7,0)))))),""))</f>
         <v/>
       </c>
       <c r="R210" s="23" t="str">
@@ -9039,7 +9175,7 @@
         <v/>
       </c>
       <c r="Q211" s="22" t="str">
-        <f aca="false">IF(OR(OR(A211="",B211=""),P211=""),"",IFERROR(P211/(IF(N(H211)&gt;0,H211,IF(N(G211)&gt;0,G211,IF(COUNTIFS($B$12:$B$211,B211,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B211,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B211,$A$5:$A$7,0)))))),""))</f>
+        <f aca="false">IF(OR(OR(A211="",B211=""),P211=""),"",IFERROR(P211/(IF(N(G211)&gt;0,G211,IF(N(H211)&gt;0,H211,IF(COUNTIFS($B$12:$B$211,B211,$G$12:$G$211,"&gt;0")+COUNTIFS($B$12:$B$211,B211,$H$12:$H$211,"&gt;0")&gt;0,"",INDEX($B$5:$B$7,MATCH(B211,$A$5:$A$7,0)))))),""))</f>
         <v/>
       </c>
       <c r="R211" s="23" t="str">

</xml_diff>